<commit_message>
Feat: add Hometown project in side projects on 261002
</commit_message>
<xml_diff>
--- a/side-project/Scrimba全栈学习路径进度追踪表.xlsx
+++ b/side-project/Scrimba全栈学习路径进度追踪表.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10920"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10927"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ersheng/Desktop/scrimba/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ersheng/Desktop/web_project/public-note/side-project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD975D8A-F106-D044-AA7A-66FFDD489780}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D098BA1-B226-4B4B-BF33-EABE606DC73F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10240" yWindow="2920" windowWidth="40960" windowHeight="23360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="10240" yWindow="2920" windowWidth="40960" windowHeight="23360" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="学习进度追踪" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,6 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">学习进度追踪!$A$1:$I$215</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -39,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="961" uniqueCount="450">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="966" uniqueCount="455">
   <si>
     <t>Introduction</t>
   </si>
@@ -1922,9 +1921,6 @@
     <t>Super!! Sub-reddits</t>
   </si>
   <si>
-    <t xml:space="preserve">ongoing… </t>
-  </si>
-  <si>
     <t>外</t>
   </si>
   <si>
@@ -1938,6 +1934,24 @@
   </si>
   <si>
     <t>号外，手写代码</t>
+  </si>
+  <si>
+    <t>MDN Core Modules</t>
+  </si>
+  <si>
+    <t>Getting started Modules</t>
+  </si>
+  <si>
+    <t>Module List</t>
+  </si>
+  <si>
+    <t>HTML Modules</t>
+  </si>
+  <si>
+    <t>CSS for styling</t>
+  </si>
+  <si>
+    <t>进行中，家乡推介</t>
   </si>
 </sst>
 </file>
@@ -1948,7 +1962,7 @@
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="14">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2026,6 +2040,25 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Yahei"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Yahei"/>
     </font>
   </fonts>
   <fills count="11">
@@ -2134,11 +2167,12 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="9" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -2197,15 +2231,22 @@
     <xf numFmtId="0" fontId="1" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="2"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
+    <cellStyle name="Hyperlink" xfId="2" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
@@ -2614,10 +2655,10 @@
     </row>
     <row r="2" spans="1:12" ht="20" customHeight="1">
       <c r="A2" s="1"/>
-      <c r="B2" s="24" t="s">
+      <c r="B2" s="25" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="24"/>
+      <c r="C2" s="25"/>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
       <c r="F2" s="1"/>
@@ -2879,10 +2920,10 @@
     </row>
     <row r="12" spans="1:12" ht="20" customHeight="1">
       <c r="A12" s="1"/>
-      <c r="B12" s="24" t="s">
+      <c r="B12" s="25" t="s">
         <v>410</v>
       </c>
-      <c r="C12" s="24"/>
+      <c r="C12" s="25"/>
       <c r="D12" s="1"/>
       <c r="E12" s="1"/>
       <c r="F12" s="1"/>
@@ -3172,7 +3213,7 @@
         <f t="shared" ref="J22:J25" si="2">IF(G22="Pending","",K22/195)</f>
         <v>9.7435897435897437E-2</v>
       </c>
-      <c r="K22" s="26">
+      <c r="K22" s="24">
         <f>COUNTIF($G$3:G22,"Done")</f>
         <v>19</v>
       </c>
@@ -3208,7 +3249,7 @@
         <f t="shared" si="2"/>
         <v>0.10256410256410256</v>
       </c>
-      <c r="K23" s="26">
+      <c r="K23" s="24">
         <f>COUNTIF($G$3:G23,"Done")</f>
         <v>20</v>
       </c>
@@ -3244,7 +3285,7 @@
         <f t="shared" si="2"/>
         <v>0.1076923076923077</v>
       </c>
-      <c r="K24" s="26">
+      <c r="K24" s="24">
         <f>COUNTIF($G$3:G24,"Done")</f>
         <v>21</v>
       </c>
@@ -3280,7 +3321,7 @@
         <f t="shared" si="2"/>
         <v>0.11282051282051282</v>
       </c>
-      <c r="K25" s="26">
+      <c r="K25" s="24">
         <f>COUNTIF($G$3:G25,"Done")</f>
         <v>22</v>
       </c>
@@ -3316,7 +3357,7 @@
         <f>IF(G26="Pending","",K26/195)</f>
         <v>0.11794871794871795</v>
       </c>
-      <c r="K26" s="26">
+      <c r="K26" s="24">
         <f>COUNTIF($G$3:G26,"Done")</f>
         <v>23</v>
       </c>
@@ -3352,7 +3393,7 @@
         <f t="shared" ref="J27:J91" si="3">IF(G27="Pending","",K27/195)</f>
         <v>0.12307692307692308</v>
       </c>
-      <c r="K27" s="26">
+      <c r="K27" s="24">
         <f>COUNTIF($G$3:G27,"Done")</f>
         <v>24</v>
       </c>
@@ -3390,7 +3431,7 @@
         <f t="shared" si="3"/>
         <v>0.12820512820512819</v>
       </c>
-      <c r="K28" s="26">
+      <c r="K28" s="24">
         <f>COUNTIF($G$3:G28,"Done")</f>
         <v>25</v>
       </c>
@@ -3426,7 +3467,7 @@
         <f t="shared" si="3"/>
         <v>0.13333333333333333</v>
       </c>
-      <c r="K29" s="26">
+      <c r="K29" s="24">
         <f>COUNTIF($G$3:G29,"Done")</f>
         <v>26</v>
       </c>
@@ -3464,7 +3505,7 @@
         <f t="shared" si="3"/>
         <v>0.13846153846153847</v>
       </c>
-      <c r="K30" s="26">
+      <c r="K30" s="24">
         <f>COUNTIF($G$3:G30,"Done")</f>
         <v>27</v>
       </c>
@@ -3500,7 +3541,7 @@
         <f t="shared" si="3"/>
         <v>0.14358974358974358</v>
       </c>
-      <c r="K31" s="26">
+      <c r="K31" s="24">
         <f>COUNTIF($G$3:G31,"Done")</f>
         <v>28</v>
       </c>
@@ -3536,7 +3577,7 @@
         <f t="shared" si="3"/>
         <v>0.14871794871794872</v>
       </c>
-      <c r="K32" s="26">
+      <c r="K32" s="24">
         <f>COUNTIF($G$3:G32,"Done")</f>
         <v>29</v>
       </c>
@@ -3572,7 +3613,7 @@
         <f t="shared" si="3"/>
         <v>0.15384615384615385</v>
       </c>
-      <c r="K33" s="26">
+      <c r="K33" s="24">
         <f>COUNTIF($G$3:G33,"Done")</f>
         <v>30</v>
       </c>
@@ -3608,7 +3649,7 @@
         <f t="shared" si="3"/>
         <v>0.15897435897435896</v>
       </c>
-      <c r="K34" s="26">
+      <c r="K34" s="24">
         <f>COUNTIF($G$3:G34,"Done")</f>
         <v>31</v>
       </c>
@@ -3644,7 +3685,7 @@
         <f t="shared" si="3"/>
         <v>0.1641025641025641</v>
       </c>
-      <c r="K35" s="26">
+      <c r="K35" s="24">
         <f>COUNTIF($G$3:G35,"Done")</f>
         <v>32</v>
       </c>
@@ -3680,7 +3721,7 @@
         <f t="shared" si="3"/>
         <v>0.16923076923076924</v>
       </c>
-      <c r="K36" s="26">
+      <c r="K36" s="24">
         <f>COUNTIF($G$3:G36,"Done")</f>
         <v>33</v>
       </c>
@@ -3716,7 +3757,7 @@
         <f t="shared" si="3"/>
         <v>0.17435897435897435</v>
       </c>
-      <c r="K37" s="26">
+      <c r="K37" s="24">
         <f>COUNTIF($G$3:G37,"Done")</f>
         <v>34</v>
       </c>
@@ -3752,7 +3793,7 @@
         <f t="shared" si="3"/>
         <v>0.17948717948717949</v>
       </c>
-      <c r="K38" s="26">
+      <c r="K38" s="24">
         <f>COUNTIF($G$3:G38,"Done")</f>
         <v>35</v>
       </c>
@@ -3788,7 +3829,7 @@
         <f t="shared" si="3"/>
         <v>0.18461538461538463</v>
       </c>
-      <c r="K39" s="26">
+      <c r="K39" s="24">
         <f>COUNTIF($G$3:G39,"Done")</f>
         <v>36</v>
       </c>
@@ -3824,7 +3865,7 @@
         <f t="shared" si="3"/>
         <v>0.18974358974358974</v>
       </c>
-      <c r="K40" s="26">
+      <c r="K40" s="24">
         <f>COUNTIF($G$3:G40,"Done")</f>
         <v>37</v>
       </c>
@@ -3860,7 +3901,7 @@
         <f t="shared" si="3"/>
         <v>0.19487179487179487</v>
       </c>
-      <c r="K41" s="26">
+      <c r="K41" s="24">
         <f>COUNTIF($G$3:G41,"Done")</f>
         <v>38</v>
       </c>
@@ -3896,7 +3937,7 @@
         <f t="shared" si="3"/>
         <v>0.2</v>
       </c>
-      <c r="K42" s="26">
+      <c r="K42" s="24">
         <f>COUNTIF($G$3:G42,"Done")</f>
         <v>39</v>
       </c>
@@ -3932,7 +3973,7 @@
         <f t="shared" si="3"/>
         <v>0.20512820512820512</v>
       </c>
-      <c r="K43" s="26">
+      <c r="K43" s="24">
         <f>COUNTIF($G$3:G43,"Done")</f>
         <v>40</v>
       </c>
@@ -3968,7 +4009,7 @@
         <f t="shared" si="3"/>
         <v>0.21025641025641026</v>
       </c>
-      <c r="K44" s="26">
+      <c r="K44" s="24">
         <f>COUNTIF($G$3:G44,"Done")</f>
         <v>41</v>
       </c>
@@ -4004,7 +4045,7 @@
         <f t="shared" si="3"/>
         <v>0.2153846153846154</v>
       </c>
-      <c r="K45" s="26">
+      <c r="K45" s="24">
         <f>COUNTIF($G$3:G45,"Done")</f>
         <v>42</v>
       </c>
@@ -4040,7 +4081,7 @@
         <f t="shared" si="3"/>
         <v>0.22051282051282051</v>
       </c>
-      <c r="K46" s="26">
+      <c r="K46" s="24">
         <f>COUNTIF($G$3:G46,"Done")</f>
         <v>43</v>
       </c>
@@ -4076,7 +4117,7 @@
         <f t="shared" si="3"/>
         <v>0.22564102564102564</v>
       </c>
-      <c r="K47" s="26">
+      <c r="K47" s="24">
         <f>COUNTIF($G$3:G47,"Done")</f>
         <v>44</v>
       </c>
@@ -4112,7 +4153,7 @@
         <f t="shared" si="3"/>
         <v>0.23076923076923078</v>
       </c>
-      <c r="K48" s="26">
+      <c r="K48" s="24">
         <f>COUNTIF($G$3:G48,"Done")</f>
         <v>45</v>
       </c>
@@ -4148,7 +4189,7 @@
         <f t="shared" si="3"/>
         <v>0.23589743589743589</v>
       </c>
-      <c r="K49" s="26">
+      <c r="K49" s="24">
         <f>COUNTIF($G$3:G49,"Done")</f>
         <v>46</v>
       </c>
@@ -4184,7 +4225,7 @@
         <f t="shared" si="3"/>
         <v>0.24102564102564103</v>
       </c>
-      <c r="K50" s="26">
+      <c r="K50" s="24">
         <f>COUNTIF($G$3:G50,"Done")</f>
         <v>47</v>
       </c>
@@ -4220,7 +4261,7 @@
         <f t="shared" si="3"/>
         <v>0.24615384615384617</v>
       </c>
-      <c r="K51" s="26">
+      <c r="K51" s="24">
         <f>COUNTIF($G$3:G51,"Done")</f>
         <v>48</v>
       </c>
@@ -4256,7 +4297,7 @@
         <f t="shared" si="3"/>
         <v>0.25128205128205128</v>
       </c>
-      <c r="K52" s="26">
+      <c r="K52" s="24">
         <f>COUNTIF($G$3:G52,"Done")</f>
         <v>49</v>
       </c>
@@ -4292,7 +4333,7 @@
         <f t="shared" si="3"/>
         <v>0.25641025641025639</v>
       </c>
-      <c r="K53" s="26">
+      <c r="K53" s="24">
         <f>COUNTIF($G$3:G53,"Done")</f>
         <v>50</v>
       </c>
@@ -4328,7 +4369,7 @@
         <f t="shared" si="3"/>
         <v>0.26153846153846155</v>
       </c>
-      <c r="K54" s="26">
+      <c r="K54" s="24">
         <f>COUNTIF($G$3:G54,"Done")</f>
         <v>51</v>
       </c>
@@ -4364,7 +4405,7 @@
         <f t="shared" si="3"/>
         <v>0.26666666666666666</v>
       </c>
-      <c r="K55" s="26">
+      <c r="K55" s="24">
         <f>COUNTIF($G$3:G55,"Done")</f>
         <v>52</v>
       </c>
@@ -4400,7 +4441,7 @@
         <f t="shared" si="3"/>
         <v>0.27179487179487177</v>
       </c>
-      <c r="K56" s="26">
+      <c r="K56" s="24">
         <f>COUNTIF($G$3:G56,"Done")</f>
         <v>53</v>
       </c>
@@ -4436,7 +4477,7 @@
         <f t="shared" si="3"/>
         <v>0.27692307692307694</v>
       </c>
-      <c r="K57" s="26">
+      <c r="K57" s="24">
         <f>COUNTIF($G$3:G57,"Done")</f>
         <v>54</v>
       </c>
@@ -4472,7 +4513,7 @@
         <f t="shared" si="3"/>
         <v>0.28205128205128205</v>
       </c>
-      <c r="K58" s="26">
+      <c r="K58" s="24">
         <f>COUNTIF($G$3:G58,"Done")</f>
         <v>55</v>
       </c>
@@ -4508,7 +4549,7 @@
         <f t="shared" si="3"/>
         <v>0.28717948717948716</v>
       </c>
-      <c r="K59" s="26">
+      <c r="K59" s="24">
         <f>COUNTIF($G$3:G59,"Done")</f>
         <v>56</v>
       </c>
@@ -4544,7 +4585,7 @@
         <f t="shared" si="3"/>
         <v>0.29230769230769232</v>
       </c>
-      <c r="K60" s="26">
+      <c r="K60" s="24">
         <f>COUNTIF($G$3:G60,"Done")</f>
         <v>57</v>
       </c>
@@ -4580,7 +4621,7 @@
         <f t="shared" si="3"/>
         <v>0.29743589743589743</v>
       </c>
-      <c r="K61" s="26">
+      <c r="K61" s="24">
         <f>COUNTIF($G$3:G61,"Done")</f>
         <v>58</v>
       </c>
@@ -4616,7 +4657,7 @@
         <f t="shared" si="3"/>
         <v>0.30256410256410254</v>
       </c>
-      <c r="K62" s="26">
+      <c r="K62" s="24">
         <f>COUNTIF($G$3:G62,"Done")</f>
         <v>59</v>
       </c>
@@ -4652,7 +4693,7 @@
         <f t="shared" si="3"/>
         <v>0.30769230769230771</v>
       </c>
-      <c r="K63" s="26">
+      <c r="K63" s="24">
         <f>COUNTIF($G$3:G63,"Done")</f>
         <v>60</v>
       </c>
@@ -4688,7 +4729,7 @@
         <f t="shared" si="3"/>
         <v>0.31282051282051282</v>
       </c>
-      <c r="K64" s="26">
+      <c r="K64" s="24">
         <f>COUNTIF($G$3:G64,"Done")</f>
         <v>61</v>
       </c>
@@ -4724,7 +4765,7 @@
         <f t="shared" si="3"/>
         <v>0.31794871794871793</v>
       </c>
-      <c r="K65" s="26">
+      <c r="K65" s="24">
         <f>COUNTIF($G$3:G65,"Done")</f>
         <v>62</v>
       </c>
@@ -4760,7 +4801,7 @@
         <f t="shared" si="3"/>
         <v>0.32307692307692309</v>
       </c>
-      <c r="K66" s="26">
+      <c r="K66" s="24">
         <f>COUNTIF($G$3:G66,"Done")</f>
         <v>63</v>
       </c>
@@ -4796,7 +4837,7 @@
         <f t="shared" si="3"/>
         <v>0.3282051282051282</v>
       </c>
-      <c r="K67" s="26">
+      <c r="K67" s="24">
         <f>COUNTIF($G$3:G67,"Done")</f>
         <v>64</v>
       </c>
@@ -4832,7 +4873,7 @@
         <f t="shared" si="3"/>
         <v>0.33333333333333331</v>
       </c>
-      <c r="K68" s="26">
+      <c r="K68" s="24">
         <f>COUNTIF($G$3:G68,"Done")</f>
         <v>65</v>
       </c>
@@ -4868,7 +4909,7 @@
         <f t="shared" si="3"/>
         <v>0.33846153846153848</v>
       </c>
-      <c r="K69" s="26">
+      <c r="K69" s="24">
         <f>COUNTIF($G$3:G69,"Done")</f>
         <v>66</v>
       </c>
@@ -4904,7 +4945,7 @@
         <f t="shared" si="3"/>
         <v>0.34358974358974359</v>
       </c>
-      <c r="K70" s="26">
+      <c r="K70" s="24">
         <f>COUNTIF($G$3:G70,"Done")</f>
         <v>67</v>
       </c>
@@ -4940,7 +4981,7 @@
         <f t="shared" si="3"/>
         <v>0.3487179487179487</v>
       </c>
-      <c r="K71" s="26">
+      <c r="K71" s="24">
         <f>COUNTIF($G$3:G71,"Done")</f>
         <v>68</v>
       </c>
@@ -4976,7 +5017,7 @@
         <f t="shared" si="3"/>
         <v>0.35384615384615387</v>
       </c>
-      <c r="K72" s="26">
+      <c r="K72" s="24">
         <f>COUNTIF($G$3:G72,"Done")</f>
         <v>69</v>
       </c>
@@ -5012,7 +5053,7 @@
         <f t="shared" si="3"/>
         <v>0.35897435897435898</v>
       </c>
-      <c r="K73" s="26">
+      <c r="K73" s="24">
         <f>COUNTIF($G$3:G73,"Done")</f>
         <v>70</v>
       </c>
@@ -5048,7 +5089,7 @@
         <f t="shared" si="3"/>
         <v>0.36410256410256409</v>
       </c>
-      <c r="K74" s="26">
+      <c r="K74" s="24">
         <f>COUNTIF($G$3:G74,"Done")</f>
         <v>71</v>
       </c>
@@ -5084,7 +5125,7 @@
         <f t="shared" si="3"/>
         <v>0.36923076923076925</v>
       </c>
-      <c r="K75" s="26">
+      <c r="K75" s="24">
         <f>COUNTIF($G$3:G75,"Done")</f>
         <v>72</v>
       </c>
@@ -5120,33 +5161,33 @@
         <f t="shared" si="3"/>
         <v>0.37435897435897436</v>
       </c>
-      <c r="K76" s="26">
+      <c r="K76" s="24">
         <f>COUNTIF($G$3:G76,"Done")</f>
         <v>73</v>
       </c>
     </row>
     <row r="77" spans="1:11" ht="20" customHeight="1">
       <c r="A77" s="2" t="s">
+        <v>444</v>
+      </c>
+      <c r="B77" s="3" t="s">
         <v>445</v>
       </c>
-      <c r="B77" s="3" t="s">
+      <c r="C77" s="3" t="s">
         <v>446</v>
-      </c>
-      <c r="C77" s="3" t="s">
-        <v>447</v>
       </c>
       <c r="D77" s="3"/>
       <c r="E77" s="2"/>
       <c r="F77" s="4"/>
       <c r="G77" s="5"/>
       <c r="H77" s="6" t="s">
+        <v>447</v>
+      </c>
+      <c r="I77" s="3" t="s">
         <v>448</v>
       </c>
-      <c r="I77" s="3" t="s">
-        <v>449</v>
-      </c>
       <c r="J77" s="21"/>
-      <c r="K77" s="26"/>
+      <c r="K77" s="24"/>
     </row>
     <row r="78" spans="1:11" ht="20" customHeight="1">
       <c r="A78" s="7">
@@ -5171,15 +5212,17 @@
         <f t="shared" ref="G78:G79" si="4">IF(H78&lt;&gt;"","Done","Pending")</f>
         <v>Done</v>
       </c>
-      <c r="H78" s="6" t="s">
-        <v>444</v>
-      </c>
-      <c r="I78" s="8"/>
+      <c r="H78" s="6">
+        <v>46296</v>
+      </c>
+      <c r="I78" s="8" t="s">
+        <v>454</v>
+      </c>
       <c r="J78" s="21">
         <f t="shared" si="3"/>
         <v>0.37948717948717947</v>
       </c>
-      <c r="K78" s="26">
+      <c r="K78" s="24">
         <f>COUNTIF($G$3:G78,"Done")</f>
         <v>74</v>
       </c>
@@ -5205,34 +5248,36 @@
       </c>
       <c r="G79" s="5" t="str">
         <f t="shared" si="4"/>
-        <v>Pending</v>
-      </c>
-      <c r="H79" s="6"/>
+        <v>Done</v>
+      </c>
+      <c r="H79" s="6">
+        <v>46297</v>
+      </c>
       <c r="I79" s="3"/>
-      <c r="J79" s="21" t="str">
+      <c r="J79" s="21">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="K79" s="26">
+        <v>0.38461538461538464</v>
+      </c>
+      <c r="K79" s="24">
         <f>COUNTIF($G$3:G79,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="80" spans="1:11" ht="20" customHeight="1">
       <c r="A80" s="1"/>
-      <c r="B80" s="24" t="s">
+      <c r="B80" s="25" t="s">
         <v>153</v>
       </c>
-      <c r="C80" s="24"/>
+      <c r="C80" s="25"/>
       <c r="D80" s="1"/>
       <c r="E80" s="1"/>
       <c r="F80" s="1"/>
       <c r="G80" s="1"/>
       <c r="H80" s="1"/>
       <c r="I80" s="1"/>
-      <c r="K80" s="26">
+      <c r="K80" s="24">
         <f>COUNTIF($G$3:G80,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="81" spans="1:11" ht="20" customHeight="1">
@@ -5262,9 +5307,9 @@
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="K81" s="26">
+      <c r="K81" s="24">
         <f>COUNTIF($G$3:G81,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="82" spans="1:11" ht="20" customHeight="1">
@@ -5294,9 +5339,9 @@
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="K82" s="26">
+      <c r="K82" s="24">
         <f>COUNTIF($G$3:G82,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="83" spans="1:11" ht="20" customHeight="1">
@@ -5326,9 +5371,9 @@
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="K83" s="26">
+      <c r="K83" s="24">
         <f>COUNTIF($G$3:G83,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="84" spans="1:11" ht="20" customHeight="1">
@@ -5358,9 +5403,9 @@
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="K84" s="26">
+      <c r="K84" s="24">
         <f>COUNTIF($G$3:G84,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="85" spans="1:11" ht="20" customHeight="1">
@@ -5390,9 +5435,9 @@
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="K85" s="26">
+      <c r="K85" s="24">
         <f>COUNTIF($G$3:G85,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="86" spans="1:11" ht="20" customHeight="1">
@@ -5422,9 +5467,9 @@
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="K86" s="26">
+      <c r="K86" s="24">
         <f>COUNTIF($G$3:G86,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="87" spans="1:11" ht="20" customHeight="1">
@@ -5454,9 +5499,9 @@
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="K87" s="26">
+      <c r="K87" s="24">
         <f>COUNTIF($G$3:G87,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="88" spans="1:11" ht="20" customHeight="1">
@@ -5486,26 +5531,26 @@
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="K88" s="26">
+      <c r="K88" s="24">
         <f>COUNTIF($G$3:G88,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="89" spans="1:11" ht="20" customHeight="1">
       <c r="A89" s="1"/>
-      <c r="B89" s="24" t="s">
+      <c r="B89" s="25" t="s">
         <v>170</v>
       </c>
-      <c r="C89" s="24"/>
+      <c r="C89" s="25"/>
       <c r="D89" s="1"/>
       <c r="E89" s="1"/>
       <c r="F89" s="1"/>
       <c r="G89" s="1"/>
       <c r="H89" s="1"/>
       <c r="I89" s="1"/>
-      <c r="K89" s="26">
+      <c r="K89" s="24">
         <f>COUNTIF($G$3:G89,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="90" spans="1:11" ht="20" customHeight="1">
@@ -5535,9 +5580,9 @@
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="K90" s="26">
+      <c r="K90" s="24">
         <f>COUNTIF($G$3:G90,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="91" spans="1:11" ht="20" customHeight="1">
@@ -5567,9 +5612,9 @@
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="K91" s="26">
+      <c r="K91" s="24">
         <f>COUNTIF($G$3:G91,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="92" spans="1:11" ht="20" customHeight="1">
@@ -5599,9 +5644,9 @@
         <f t="shared" ref="J92:J155" si="7">IF(G92="Pending","",K92/195)</f>
         <v/>
       </c>
-      <c r="K92" s="26">
+      <c r="K92" s="24">
         <f>COUNTIF($G$3:G92,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="93" spans="1:11" ht="20" customHeight="1">
@@ -5631,26 +5676,26 @@
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="K93" s="26">
+      <c r="K93" s="24">
         <f>COUNTIF($G$3:G93,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="94" spans="1:11" ht="20" customHeight="1">
       <c r="A94" s="1"/>
-      <c r="B94" s="24" t="s">
+      <c r="B94" s="25" t="s">
         <v>179</v>
       </c>
-      <c r="C94" s="24"/>
+      <c r="C94" s="25"/>
       <c r="D94" s="1"/>
       <c r="E94" s="1"/>
       <c r="F94" s="1"/>
       <c r="G94" s="1"/>
       <c r="H94" s="1"/>
       <c r="I94" s="1"/>
-      <c r="K94" s="26">
+      <c r="K94" s="24">
         <f>COUNTIF($G$3:G94,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="95" spans="1:11" ht="20" customHeight="1">
@@ -5680,9 +5725,9 @@
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="K95" s="26">
+      <c r="K95" s="24">
         <f>COUNTIF($G$3:G95,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="96" spans="1:11" ht="20" customHeight="1">
@@ -5712,9 +5757,9 @@
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="K96" s="26">
+      <c r="K96" s="24">
         <f>COUNTIF($G$3:G96,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="97" spans="1:11" ht="20" customHeight="1">
@@ -5744,9 +5789,9 @@
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="K97" s="26">
+      <c r="K97" s="24">
         <f>COUNTIF($G$3:G97,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="98" spans="1:11" ht="20" customHeight="1">
@@ -5776,9 +5821,9 @@
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="K98" s="26">
+      <c r="K98" s="24">
         <f>COUNTIF($G$3:G98,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="99" spans="1:11" ht="20" customHeight="1">
@@ -5808,9 +5853,9 @@
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="K99" s="26">
+      <c r="K99" s="24">
         <f>COUNTIF($G$3:G99,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="100" spans="1:11" ht="20" customHeight="1">
@@ -5840,9 +5885,9 @@
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="K100" s="26">
+      <c r="K100" s="24">
         <f>COUNTIF($G$3:G100,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="101" spans="1:11" ht="20" customHeight="1">
@@ -5872,9 +5917,9 @@
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="K101" s="26">
+      <c r="K101" s="24">
         <f>COUNTIF($G$3:G101,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="102" spans="1:11" ht="20" customHeight="1">
@@ -5904,9 +5949,9 @@
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="K102" s="26">
+      <c r="K102" s="24">
         <f>COUNTIF($G$3:G102,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="103" spans="1:11" ht="20" customHeight="1">
@@ -5936,9 +5981,9 @@
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="K103" s="26">
+      <c r="K103" s="24">
         <f>COUNTIF($G$3:G103,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="104" spans="1:11" ht="20" customHeight="1">
@@ -5968,9 +6013,9 @@
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="K104" s="26">
+      <c r="K104" s="24">
         <f>COUNTIF($G$3:G104,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="105" spans="1:11" ht="20" customHeight="1">
@@ -6000,9 +6045,9 @@
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="K105" s="26">
+      <c r="K105" s="24">
         <f>COUNTIF($G$3:G105,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="106" spans="1:11" ht="20" customHeight="1">
@@ -6032,9 +6077,9 @@
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="K106" s="26">
+      <c r="K106" s="24">
         <f>COUNTIF($G$3:G106,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="107" spans="1:11" ht="20" customHeight="1">
@@ -6064,9 +6109,9 @@
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="K107" s="26">
+      <c r="K107" s="24">
         <f>COUNTIF($G$3:G107,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="108" spans="1:11" ht="20" customHeight="1">
@@ -6096,9 +6141,9 @@
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="K108" s="26">
+      <c r="K108" s="24">
         <f>COUNTIF($G$3:G108,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="109" spans="1:11" ht="20" customHeight="1">
@@ -6128,9 +6173,9 @@
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="K109" s="26">
+      <c r="K109" s="24">
         <f>COUNTIF($G$3:G109,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="110" spans="1:11" ht="20" customHeight="1">
@@ -6160,9 +6205,9 @@
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="K110" s="26">
+      <c r="K110" s="24">
         <f>COUNTIF($G$3:G110,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="111" spans="1:11" ht="20" customHeight="1">
@@ -6192,9 +6237,9 @@
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="K111" s="26">
+      <c r="K111" s="24">
         <f>COUNTIF($G$3:G111,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="112" spans="1:11" ht="20" customHeight="1">
@@ -6224,9 +6269,9 @@
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="K112" s="26">
+      <c r="K112" s="24">
         <f>COUNTIF($G$3:G112,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="113" spans="1:11" ht="20" customHeight="1">
@@ -6256,9 +6301,9 @@
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="K113" s="26">
+      <c r="K113" s="24">
         <f>COUNTIF($G$3:G113,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="114" spans="1:11" ht="20" customHeight="1">
@@ -6288,9 +6333,9 @@
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="K114" s="26">
+      <c r="K114" s="24">
         <f>COUNTIF($G$3:G114,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="115" spans="1:11" ht="20" customHeight="1">
@@ -6320,9 +6365,9 @@
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="K115" s="26">
+      <c r="K115" s="24">
         <f>COUNTIF($G$3:G115,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="116" spans="1:11" ht="20" customHeight="1">
@@ -6352,9 +6397,9 @@
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="K116" s="26">
+      <c r="K116" s="24">
         <f>COUNTIF($G$3:G116,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="117" spans="1:11" ht="20" customHeight="1">
@@ -6384,9 +6429,9 @@
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="K117" s="26">
+      <c r="K117" s="24">
         <f>COUNTIF($G$3:G117,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="118" spans="1:11" ht="20" customHeight="1">
@@ -6416,9 +6461,9 @@
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="K118" s="26">
+      <c r="K118" s="24">
         <f>COUNTIF($G$3:G118,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="119" spans="1:11" ht="20" customHeight="1">
@@ -6448,26 +6493,26 @@
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="K119" s="26">
+      <c r="K119" s="24">
         <f>COUNTIF($G$3:G119,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="120" spans="1:11" ht="20" customHeight="1">
       <c r="A120" s="1"/>
-      <c r="B120" s="24" t="s">
+      <c r="B120" s="25" t="s">
         <v>223</v>
       </c>
-      <c r="C120" s="24"/>
+      <c r="C120" s="25"/>
       <c r="D120" s="1"/>
       <c r="E120" s="1"/>
       <c r="F120" s="1"/>
       <c r="G120" s="1"/>
       <c r="H120" s="1"/>
       <c r="I120" s="1"/>
-      <c r="K120" s="26">
+      <c r="K120" s="24">
         <f>COUNTIF($G$3:G120,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="121" spans="1:11" ht="20" customHeight="1">
@@ -6497,9 +6542,9 @@
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="K121" s="26">
+      <c r="K121" s="24">
         <f>COUNTIF($G$3:G121,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="122" spans="1:11" ht="20" customHeight="1">
@@ -6529,9 +6574,9 @@
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="K122" s="26">
+      <c r="K122" s="24">
         <f>COUNTIF($G$3:G122,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="123" spans="1:11" ht="20" customHeight="1">
@@ -6561,9 +6606,9 @@
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="K123" s="26">
+      <c r="K123" s="24">
         <f>COUNTIF($G$3:G123,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="124" spans="1:11" ht="20" customHeight="1">
@@ -6593,9 +6638,9 @@
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="K124" s="26">
+      <c r="K124" s="24">
         <f>COUNTIF($G$3:G124,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="125" spans="1:11" ht="20" customHeight="1">
@@ -6625,26 +6670,26 @@
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="K125" s="26">
+      <c r="K125" s="24">
         <f>COUNTIF($G$3:G125,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="126" spans="1:11" ht="20" customHeight="1">
       <c r="A126" s="1"/>
-      <c r="B126" s="24" t="s">
+      <c r="B126" s="25" t="s">
         <v>234</v>
       </c>
-      <c r="C126" s="24"/>
+      <c r="C126" s="25"/>
       <c r="D126" s="1"/>
       <c r="E126" s="1"/>
       <c r="F126" s="1"/>
       <c r="G126" s="1"/>
       <c r="H126" s="1"/>
       <c r="I126" s="1"/>
-      <c r="K126" s="26">
+      <c r="K126" s="24">
         <f>COUNTIF($G$3:G126,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="127" spans="1:11" ht="20" customHeight="1">
@@ -6674,9 +6719,9 @@
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="K127" s="26">
+      <c r="K127" s="24">
         <f>COUNTIF($G$3:G127,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="128" spans="1:11" ht="20" customHeight="1">
@@ -6706,9 +6751,9 @@
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="K128" s="26">
+      <c r="K128" s="24">
         <f>COUNTIF($G$3:G128,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="129" spans="1:11" ht="20" customHeight="1">
@@ -6738,9 +6783,9 @@
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="K129" s="26">
+      <c r="K129" s="24">
         <f>COUNTIF($G$3:G129,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="130" spans="1:11" ht="20" customHeight="1">
@@ -6770,9 +6815,9 @@
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="K130" s="26">
+      <c r="K130" s="24">
         <f>COUNTIF($G$3:G130,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="131" spans="1:11" ht="20" customHeight="1">
@@ -6802,9 +6847,9 @@
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="K131" s="26">
+      <c r="K131" s="24">
         <f>COUNTIF($G$3:G131,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="132" spans="1:11" ht="20" customHeight="1">
@@ -6834,26 +6879,26 @@
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="K132" s="26">
+      <c r="K132" s="24">
         <f>COUNTIF($G$3:G132,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="133" spans="1:11" ht="20" customHeight="1">
       <c r="A133" s="1"/>
-      <c r="B133" s="24" t="s">
+      <c r="B133" s="25" t="s">
         <v>245</v>
       </c>
-      <c r="C133" s="24"/>
+      <c r="C133" s="25"/>
       <c r="D133" s="1"/>
       <c r="E133" s="1"/>
       <c r="F133" s="1"/>
       <c r="G133" s="1"/>
       <c r="H133" s="1"/>
       <c r="I133" s="1"/>
-      <c r="K133" s="26">
+      <c r="K133" s="24">
         <f>COUNTIF($G$3:G133,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="134" spans="1:11" ht="20" customHeight="1">
@@ -6883,9 +6928,9 @@
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="K134" s="26">
+      <c r="K134" s="24">
         <f>COUNTIF($G$3:G134,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="135" spans="1:11" ht="20" customHeight="1">
@@ -6915,9 +6960,9 @@
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="K135" s="26">
+      <c r="K135" s="24">
         <f>COUNTIF($G$3:G135,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="136" spans="1:11" ht="20" customHeight="1">
@@ -6947,9 +6992,9 @@
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="K136" s="26">
+      <c r="K136" s="24">
         <f>COUNTIF($G$3:G136,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="137" spans="1:11" ht="20" customHeight="1">
@@ -6979,9 +7024,9 @@
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="K137" s="26">
+      <c r="K137" s="24">
         <f>COUNTIF($G$3:G137,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="138" spans="1:11" ht="20" customHeight="1">
@@ -7011,26 +7056,26 @@
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="K138" s="26">
+      <c r="K138" s="24">
         <f>COUNTIF($G$3:G138,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="139" spans="1:11" ht="20" customHeight="1">
       <c r="A139" s="1"/>
-      <c r="B139" s="24" t="s">
+      <c r="B139" s="25" t="s">
         <v>256</v>
       </c>
-      <c r="C139" s="24"/>
+      <c r="C139" s="25"/>
       <c r="D139" s="1"/>
       <c r="E139" s="1"/>
       <c r="F139" s="1"/>
       <c r="G139" s="1"/>
       <c r="H139" s="1"/>
       <c r="I139" s="1"/>
-      <c r="K139" s="26">
+      <c r="K139" s="24">
         <f>COUNTIF($G$3:G139,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="140" spans="1:11" ht="20" customHeight="1">
@@ -7060,9 +7105,9 @@
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="K140" s="26">
+      <c r="K140" s="24">
         <f>COUNTIF($G$3:G140,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="141" spans="1:11" ht="20" customHeight="1">
@@ -7092,9 +7137,9 @@
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="K141" s="26">
+      <c r="K141" s="24">
         <f>COUNTIF($G$3:G141,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="142" spans="1:11" ht="20" customHeight="1">
@@ -7124,9 +7169,9 @@
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="K142" s="26">
+      <c r="K142" s="24">
         <f>COUNTIF($G$3:G142,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="143" spans="1:11" ht="20" customHeight="1">
@@ -7156,9 +7201,9 @@
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="K143" s="26">
+      <c r="K143" s="24">
         <f>COUNTIF($G$3:G143,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="144" spans="1:11" ht="20" customHeight="1">
@@ -7188,9 +7233,9 @@
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="K144" s="26">
+      <c r="K144" s="24">
         <f>COUNTIF($G$3:G144,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="145" spans="1:11" ht="20" customHeight="1">
@@ -7220,9 +7265,9 @@
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="K145" s="26">
+      <c r="K145" s="24">
         <f>COUNTIF($G$3:G145,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="146" spans="1:11" ht="20" customHeight="1">
@@ -7252,26 +7297,26 @@
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="K146" s="26">
+      <c r="K146" s="24">
         <f>COUNTIF($G$3:G146,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="147" spans="1:11" ht="20" customHeight="1">
       <c r="A147" s="1"/>
-      <c r="B147" s="24" t="s">
+      <c r="B147" s="25" t="s">
         <v>268</v>
       </c>
-      <c r="C147" s="24"/>
+      <c r="C147" s="25"/>
       <c r="D147" s="1"/>
       <c r="E147" s="1"/>
       <c r="F147" s="1"/>
       <c r="G147" s="1"/>
       <c r="H147" s="1"/>
       <c r="I147" s="1"/>
-      <c r="K147" s="26">
+      <c r="K147" s="24">
         <f>COUNTIF($G$3:G147,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="148" spans="1:11" ht="20" customHeight="1">
@@ -7301,9 +7346,9 @@
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="K148" s="26">
+      <c r="K148" s="24">
         <f>COUNTIF($G$3:G148,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="149" spans="1:11" ht="20" customHeight="1">
@@ -7333,9 +7378,9 @@
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="K149" s="26">
+      <c r="K149" s="24">
         <f>COUNTIF($G$3:G149,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="150" spans="1:11" ht="20" customHeight="1">
@@ -7365,9 +7410,9 @@
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="K150" s="26">
+      <c r="K150" s="24">
         <f>COUNTIF($G$3:G150,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="151" spans="1:11" ht="20" customHeight="1">
@@ -7397,9 +7442,9 @@
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="K151" s="26">
+      <c r="K151" s="24">
         <f>COUNTIF($G$3:G151,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="152" spans="1:11" ht="20" customHeight="1">
@@ -7429,9 +7474,9 @@
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="K152" s="26">
+      <c r="K152" s="24">
         <f>COUNTIF($G$3:G152,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="153" spans="1:11" ht="20" customHeight="1">
@@ -7461,26 +7506,26 @@
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="K153" s="26">
+      <c r="K153" s="24">
         <f>COUNTIF($G$3:G153,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="154" spans="1:11" ht="20" customHeight="1">
       <c r="A154" s="1"/>
-      <c r="B154" s="24" t="s">
+      <c r="B154" s="25" t="s">
         <v>279</v>
       </c>
-      <c r="C154" s="24"/>
+      <c r="C154" s="25"/>
       <c r="D154" s="1"/>
       <c r="E154" s="1"/>
       <c r="F154" s="1"/>
       <c r="G154" s="1"/>
       <c r="H154" s="1"/>
       <c r="I154" s="1"/>
-      <c r="K154" s="26">
+      <c r="K154" s="24">
         <f>COUNTIF($G$3:G154,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="155" spans="1:11" ht="20" customHeight="1">
@@ -7510,9 +7555,9 @@
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="K155" s="26">
+      <c r="K155" s="24">
         <f>COUNTIF($G$3:G155,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="156" spans="1:11" ht="20" customHeight="1">
@@ -7542,9 +7587,9 @@
         <f t="shared" ref="J156:J215" si="15">IF(G156="Pending","",K156/195)</f>
         <v/>
       </c>
-      <c r="K156" s="26">
+      <c r="K156" s="24">
         <f>COUNTIF($G$3:G156,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="157" spans="1:11" ht="20" customHeight="1">
@@ -7574,9 +7619,9 @@
         <f t="shared" si="15"/>
         <v/>
       </c>
-      <c r="K157" s="26">
+      <c r="K157" s="24">
         <f>COUNTIF($G$3:G157,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="158" spans="1:11" ht="20" customHeight="1">
@@ -7606,26 +7651,26 @@
         <f t="shared" si="15"/>
         <v/>
       </c>
-      <c r="K158" s="26">
+      <c r="K158" s="24">
         <f>COUNTIF($G$3:G158,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="159" spans="1:11" ht="20" customHeight="1">
       <c r="A159" s="1"/>
-      <c r="B159" s="24" t="s">
+      <c r="B159" s="25" t="s">
         <v>288</v>
       </c>
-      <c r="C159" s="24"/>
+      <c r="C159" s="25"/>
       <c r="D159" s="1"/>
       <c r="E159" s="1"/>
       <c r="F159" s="1"/>
       <c r="G159" s="1"/>
       <c r="H159" s="1"/>
       <c r="I159" s="1"/>
-      <c r="K159" s="26">
+      <c r="K159" s="24">
         <f>COUNTIF($G$3:G159,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="160" spans="1:11" ht="20" customHeight="1">
@@ -7655,9 +7700,9 @@
         <f t="shared" si="15"/>
         <v/>
       </c>
-      <c r="K160" s="26">
+      <c r="K160" s="24">
         <f>COUNTIF($G$3:G160,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="161" spans="1:11" ht="20" customHeight="1">
@@ -7687,9 +7732,9 @@
         <f t="shared" si="15"/>
         <v/>
       </c>
-      <c r="K161" s="26">
+      <c r="K161" s="24">
         <f>COUNTIF($G$3:G161,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="162" spans="1:11" ht="20" customHeight="1">
@@ -7719,26 +7764,26 @@
         <f t="shared" si="15"/>
         <v/>
       </c>
-      <c r="K162" s="26">
+      <c r="K162" s="24">
         <f>COUNTIF($G$3:G162,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="163" spans="1:11" ht="20" customHeight="1">
       <c r="A163" s="1"/>
-      <c r="B163" s="24" t="s">
+      <c r="B163" s="25" t="s">
         <v>295</v>
       </c>
-      <c r="C163" s="24"/>
+      <c r="C163" s="25"/>
       <c r="D163" s="1"/>
       <c r="E163" s="1"/>
       <c r="F163" s="1"/>
       <c r="G163" s="1"/>
       <c r="H163" s="1"/>
       <c r="I163" s="1"/>
-      <c r="K163" s="26">
+      <c r="K163" s="24">
         <f>COUNTIF($G$3:G163,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="164" spans="1:11" ht="20" customHeight="1">
@@ -7768,9 +7813,9 @@
         <f t="shared" si="15"/>
         <v/>
       </c>
-      <c r="K164" s="26">
+      <c r="K164" s="24">
         <f>COUNTIF($G$3:G164,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="165" spans="1:11" ht="20" customHeight="1">
@@ -7800,9 +7845,9 @@
         <f t="shared" si="15"/>
         <v/>
       </c>
-      <c r="K165" s="26">
+      <c r="K165" s="24">
         <f>COUNTIF($G$3:G165,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="166" spans="1:11" ht="20" customHeight="1">
@@ -7832,9 +7877,9 @@
         <f t="shared" si="15"/>
         <v/>
       </c>
-      <c r="K166" s="26">
+      <c r="K166" s="24">
         <f>COUNTIF($G$3:G166,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="167" spans="1:11" ht="20" customHeight="1">
@@ -7864,26 +7909,26 @@
         <f t="shared" si="15"/>
         <v/>
       </c>
-      <c r="K167" s="26">
+      <c r="K167" s="24">
         <f>COUNTIF($G$3:G167,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="168" spans="1:11" ht="20" customHeight="1">
       <c r="A168" s="1"/>
-      <c r="B168" s="24" t="s">
+      <c r="B168" s="25" t="s">
         <v>302</v>
       </c>
-      <c r="C168" s="24"/>
+      <c r="C168" s="25"/>
       <c r="D168" s="1"/>
       <c r="E168" s="1"/>
       <c r="F168" s="1"/>
       <c r="G168" s="1"/>
       <c r="H168" s="1"/>
       <c r="I168" s="1"/>
-      <c r="K168" s="26">
+      <c r="K168" s="24">
         <f>COUNTIF($G$3:G168,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="169" spans="1:11" ht="20" customHeight="1">
@@ -7913,9 +7958,9 @@
         <f t="shared" si="15"/>
         <v/>
       </c>
-      <c r="K169" s="26">
+      <c r="K169" s="24">
         <f>COUNTIF($G$3:G169,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="170" spans="1:11" ht="20" customHeight="1">
@@ -7945,9 +7990,9 @@
         <f t="shared" si="15"/>
         <v/>
       </c>
-      <c r="K170" s="26">
+      <c r="K170" s="24">
         <f>COUNTIF($G$3:G170,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="171" spans="1:11" ht="20" customHeight="1">
@@ -7977,9 +8022,9 @@
         <f t="shared" si="15"/>
         <v/>
       </c>
-      <c r="K171" s="26">
+      <c r="K171" s="24">
         <f>COUNTIF($G$3:G171,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="172" spans="1:11" ht="20" customHeight="1">
@@ -8009,26 +8054,26 @@
         <f t="shared" si="15"/>
         <v/>
       </c>
-      <c r="K172" s="26">
+      <c r="K172" s="24">
         <f>COUNTIF($G$3:G172,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="173" spans="1:11" ht="20" customHeight="1">
       <c r="A173" s="1"/>
-      <c r="B173" s="24" t="s">
+      <c r="B173" s="25" t="s">
         <v>309</v>
       </c>
-      <c r="C173" s="24"/>
+      <c r="C173" s="25"/>
       <c r="D173" s="1"/>
       <c r="E173" s="1"/>
       <c r="F173" s="1"/>
       <c r="G173" s="1"/>
       <c r="H173" s="1"/>
       <c r="I173" s="1"/>
-      <c r="K173" s="26">
+      <c r="K173" s="24">
         <f>COUNTIF($G$3:G173,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="174" spans="1:11" ht="20" customHeight="1">
@@ -8058,9 +8103,9 @@
         <f t="shared" si="15"/>
         <v/>
       </c>
-      <c r="K174" s="26">
+      <c r="K174" s="24">
         <f>COUNTIF($G$3:G174,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="175" spans="1:11" ht="20" customHeight="1">
@@ -8090,9 +8135,9 @@
         <f t="shared" si="15"/>
         <v/>
       </c>
-      <c r="K175" s="26">
+      <c r="K175" s="24">
         <f>COUNTIF($G$3:G175,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="176" spans="1:11" ht="20" customHeight="1">
@@ -8122,9 +8167,9 @@
         <f t="shared" si="15"/>
         <v/>
       </c>
-      <c r="K176" s="26">
+      <c r="K176" s="24">
         <f>COUNTIF($G$3:G176,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="177" spans="1:11" ht="20" customHeight="1">
@@ -8154,9 +8199,9 @@
         <f t="shared" si="15"/>
         <v/>
       </c>
-      <c r="K177" s="26">
+      <c r="K177" s="24">
         <f>COUNTIF($G$3:G177,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="178" spans="1:11" ht="20" customHeight="1">
@@ -8186,9 +8231,9 @@
         <f t="shared" si="15"/>
         <v/>
       </c>
-      <c r="K178" s="26">
+      <c r="K178" s="24">
         <f>COUNTIF($G$3:G178,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="179" spans="1:11" ht="20" customHeight="1">
@@ -8218,9 +8263,9 @@
         <f t="shared" si="15"/>
         <v/>
       </c>
-      <c r="K179" s="26">
+      <c r="K179" s="24">
         <f>COUNTIF($G$3:G179,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="180" spans="1:11" ht="20" customHeight="1">
@@ -8250,9 +8295,9 @@
         <f t="shared" si="15"/>
         <v/>
       </c>
-      <c r="K180" s="26">
+      <c r="K180" s="24">
         <f>COUNTIF($G$3:G180,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="181" spans="1:11" ht="20" customHeight="1">
@@ -8282,9 +8327,9 @@
         <f t="shared" si="15"/>
         <v/>
       </c>
-      <c r="K181" s="26">
+      <c r="K181" s="24">
         <f>COUNTIF($G$3:G181,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="182" spans="1:11" ht="20" customHeight="1">
@@ -8314,9 +8359,9 @@
         <f t="shared" si="15"/>
         <v/>
       </c>
-      <c r="K182" s="26">
+      <c r="K182" s="24">
         <f>COUNTIF($G$3:G182,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="183" spans="1:11" ht="20" customHeight="1">
@@ -8346,26 +8391,26 @@
         <f t="shared" si="15"/>
         <v/>
       </c>
-      <c r="K183" s="26">
+      <c r="K183" s="24">
         <f>COUNTIF($G$3:G183,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="184" spans="1:11" ht="20" customHeight="1">
       <c r="A184" s="1"/>
-      <c r="B184" s="24" t="s">
+      <c r="B184" s="25" t="s">
         <v>329</v>
       </c>
-      <c r="C184" s="24"/>
+      <c r="C184" s="25"/>
       <c r="D184" s="1"/>
       <c r="E184" s="1"/>
       <c r="F184" s="1"/>
       <c r="G184" s="1"/>
       <c r="H184" s="1"/>
       <c r="I184" s="1"/>
-      <c r="K184" s="26">
+      <c r="K184" s="24">
         <f>COUNTIF($G$3:G184,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="185" spans="1:11" ht="20" customHeight="1">
@@ -8395,9 +8440,9 @@
         <f t="shared" si="15"/>
         <v/>
       </c>
-      <c r="K185" s="26">
+      <c r="K185" s="24">
         <f>COUNTIF($G$3:G185,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="186" spans="1:11" ht="20" customHeight="1">
@@ -8427,9 +8472,9 @@
         <f t="shared" si="15"/>
         <v/>
       </c>
-      <c r="K186" s="26">
+      <c r="K186" s="24">
         <f>COUNTIF($G$3:G186,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="187" spans="1:11" ht="20" customHeight="1">
@@ -8459,9 +8504,9 @@
         <f t="shared" si="15"/>
         <v/>
       </c>
-      <c r="K187" s="26">
+      <c r="K187" s="24">
         <f>COUNTIF($G$3:G187,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="188" spans="1:11" ht="20" customHeight="1">
@@ -8491,9 +8536,9 @@
         <f t="shared" si="15"/>
         <v/>
       </c>
-      <c r="K188" s="26">
+      <c r="K188" s="24">
         <f>COUNTIF($G$3:G188,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="189" spans="1:11" ht="20" customHeight="1">
@@ -8523,9 +8568,9 @@
         <f t="shared" si="15"/>
         <v/>
       </c>
-      <c r="K189" s="26">
+      <c r="K189" s="24">
         <f>COUNTIF($G$3:G189,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="190" spans="1:11" ht="20" customHeight="1">
@@ -8555,9 +8600,9 @@
         <f t="shared" si="15"/>
         <v/>
       </c>
-      <c r="K190" s="26">
+      <c r="K190" s="24">
         <f>COUNTIF($G$3:G190,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="191" spans="1:11" ht="20" customHeight="1">
@@ -8587,9 +8632,9 @@
         <f t="shared" si="15"/>
         <v/>
       </c>
-      <c r="K191" s="26">
+      <c r="K191" s="24">
         <f>COUNTIF($G$3:G191,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="192" spans="1:11" ht="20" customHeight="1">
@@ -8619,9 +8664,9 @@
         <f t="shared" si="15"/>
         <v/>
       </c>
-      <c r="K192" s="26">
+      <c r="K192" s="24">
         <f>COUNTIF($G$3:G192,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="193" spans="1:11" ht="20" customHeight="1">
@@ -8651,9 +8696,9 @@
         <f t="shared" si="15"/>
         <v/>
       </c>
-      <c r="K193" s="26">
+      <c r="K193" s="24">
         <f>COUNTIF($G$3:G193,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="194" spans="1:11" ht="20" customHeight="1">
@@ -8683,9 +8728,9 @@
         <f t="shared" si="15"/>
         <v/>
       </c>
-      <c r="K194" s="26">
+      <c r="K194" s="24">
         <f>COUNTIF($G$3:G194,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="195" spans="1:11" ht="20" customHeight="1">
@@ -8715,9 +8760,9 @@
         <f t="shared" si="15"/>
         <v/>
       </c>
-      <c r="K195" s="26">
+      <c r="K195" s="24">
         <f>COUNTIF($G$3:G195,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="196" spans="1:11" ht="20" customHeight="1">
@@ -8747,26 +8792,26 @@
         <f t="shared" si="15"/>
         <v/>
       </c>
-      <c r="K196" s="26">
+      <c r="K196" s="24">
         <f>COUNTIF($G$3:G196,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="197" spans="1:11" ht="20" customHeight="1">
       <c r="A197" s="1"/>
-      <c r="B197" s="24" t="s">
+      <c r="B197" s="25" t="s">
         <v>348</v>
       </c>
-      <c r="C197" s="24"/>
+      <c r="C197" s="25"/>
       <c r="D197" s="1"/>
       <c r="E197" s="1"/>
       <c r="F197" s="1"/>
       <c r="G197" s="1"/>
       <c r="H197" s="1"/>
       <c r="I197" s="1"/>
-      <c r="K197" s="26">
+      <c r="K197" s="24">
         <f>COUNTIF($G$3:G197,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="198" spans="1:11" ht="20" customHeight="1">
@@ -8796,9 +8841,9 @@
         <f t="shared" si="15"/>
         <v/>
       </c>
-      <c r="K198" s="26">
+      <c r="K198" s="24">
         <f>COUNTIF($G$3:G198,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="199" spans="1:11" ht="20" customHeight="1">
@@ -8828,9 +8873,9 @@
         <f t="shared" si="15"/>
         <v/>
       </c>
-      <c r="K199" s="26">
+      <c r="K199" s="24">
         <f>COUNTIF($G$3:G199,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="200" spans="1:11" ht="20" customHeight="1">
@@ -8860,9 +8905,9 @@
         <f t="shared" si="15"/>
         <v/>
       </c>
-      <c r="K200" s="26">
+      <c r="K200" s="24">
         <f>COUNTIF($G$3:G200,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="201" spans="1:11" ht="20" customHeight="1">
@@ -8892,9 +8937,9 @@
         <f t="shared" si="15"/>
         <v/>
       </c>
-      <c r="K201" s="26">
+      <c r="K201" s="24">
         <f>COUNTIF($G$3:G201,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="202" spans="1:11" ht="20" customHeight="1">
@@ -8924,9 +8969,9 @@
         <f t="shared" si="15"/>
         <v/>
       </c>
-      <c r="K202" s="26">
+      <c r="K202" s="24">
         <f>COUNTIF($G$3:G202,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="203" spans="1:11" ht="20" customHeight="1">
@@ -8956,9 +9001,9 @@
         <f t="shared" si="15"/>
         <v/>
       </c>
-      <c r="K203" s="26">
+      <c r="K203" s="24">
         <f>COUNTIF($G$3:G203,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="204" spans="1:11" ht="20" customHeight="1">
@@ -8988,26 +9033,26 @@
         <f t="shared" si="15"/>
         <v/>
       </c>
-      <c r="K204" s="26">
+      <c r="K204" s="24">
         <f>COUNTIF($G$3:G204,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="205" spans="1:11" ht="20" customHeight="1">
       <c r="A205" s="1"/>
-      <c r="B205" s="24" t="s">
+      <c r="B205" s="25" t="s">
         <v>361</v>
       </c>
-      <c r="C205" s="24"/>
+      <c r="C205" s="25"/>
       <c r="D205" s="1"/>
       <c r="E205" s="1"/>
       <c r="F205" s="1"/>
       <c r="G205" s="1"/>
       <c r="H205" s="1"/>
       <c r="I205" s="1"/>
-      <c r="K205" s="26">
+      <c r="K205" s="24">
         <f>COUNTIF($G$3:G205,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="206" spans="1:11" ht="20" customHeight="1">
@@ -9037,9 +9082,9 @@
         <f t="shared" si="15"/>
         <v/>
       </c>
-      <c r="K206" s="26">
+      <c r="K206" s="24">
         <f>COUNTIF($G$3:G206,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="207" spans="1:11" ht="20" customHeight="1">
@@ -9069,9 +9114,9 @@
         <f t="shared" si="15"/>
         <v/>
       </c>
-      <c r="K207" s="26">
+      <c r="K207" s="24">
         <f>COUNTIF($G$3:G207,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="208" spans="1:11" ht="20" customHeight="1">
@@ -9101,9 +9146,9 @@
         <f t="shared" si="15"/>
         <v/>
       </c>
-      <c r="K208" s="26">
+      <c r="K208" s="24">
         <f>COUNTIF($G$3:G208,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="209" spans="1:11" ht="20" customHeight="1">
@@ -9133,9 +9178,9 @@
         <f t="shared" si="15"/>
         <v/>
       </c>
-      <c r="K209" s="26">
+      <c r="K209" s="24">
         <f>COUNTIF($G$3:G209,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="210" spans="1:11" ht="20" customHeight="1">
@@ -9165,26 +9210,26 @@
         <f t="shared" si="15"/>
         <v/>
       </c>
-      <c r="K210" s="26">
+      <c r="K210" s="24">
         <f>COUNTIF($G$3:G210,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="211" spans="1:11" ht="20" customHeight="1">
       <c r="A211" s="1"/>
-      <c r="B211" s="24" t="s">
+      <c r="B211" s="25" t="s">
         <v>372</v>
       </c>
-      <c r="C211" s="24"/>
+      <c r="C211" s="25"/>
       <c r="D211" s="1"/>
       <c r="E211" s="1"/>
       <c r="F211" s="1"/>
       <c r="G211" s="1"/>
       <c r="H211" s="1"/>
       <c r="I211" s="1"/>
-      <c r="K211" s="26">
+      <c r="K211" s="24">
         <f>COUNTIF($G$3:G211,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="212" spans="1:11" ht="20" customHeight="1">
@@ -9214,9 +9259,9 @@
         <f t="shared" si="15"/>
         <v/>
       </c>
-      <c r="K212" s="26">
+      <c r="K212" s="24">
         <f>COUNTIF($G$3:G212,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="213" spans="1:11" ht="20" customHeight="1">
@@ -9246,9 +9291,9 @@
         <f t="shared" si="15"/>
         <v/>
       </c>
-      <c r="K213" s="26">
+      <c r="K213" s="24">
         <f>COUNTIF($G$3:G213,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="214" spans="1:11" ht="20" customHeight="1">
@@ -9278,9 +9323,9 @@
         <f t="shared" si="15"/>
         <v/>
       </c>
-      <c r="K214" s="26">
+      <c r="K214" s="24">
         <f>COUNTIF($G$3:G214,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="215" spans="1:11" ht="20" customHeight="1">
@@ -9310,14 +9355,20 @@
         <f t="shared" si="15"/>
         <v/>
       </c>
-      <c r="K215" s="26">
+      <c r="K215" s="24">
         <f>COUNTIF($G$3:G215,"Done")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:I215" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <mergeCells count="19">
+    <mergeCell ref="B168:C168"/>
+    <mergeCell ref="B211:C211"/>
+    <mergeCell ref="B197:C197"/>
+    <mergeCell ref="B173:C173"/>
+    <mergeCell ref="B184:C184"/>
+    <mergeCell ref="B205:C205"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="B133:C133"/>
     <mergeCell ref="B89:C89"/>
@@ -9331,12 +9382,6 @@
     <mergeCell ref="B126:C126"/>
     <mergeCell ref="B94:C94"/>
     <mergeCell ref="B12:C12"/>
-    <mergeCell ref="B168:C168"/>
-    <mergeCell ref="B211:C211"/>
-    <mergeCell ref="B197:C197"/>
-    <mergeCell ref="B173:C173"/>
-    <mergeCell ref="B184:C184"/>
-    <mergeCell ref="B205:C205"/>
   </mergeCells>
   <conditionalFormatting sqref="G1:G1048576">
     <cfRule type="cellIs" dxfId="5" priority="1" operator="equal">
@@ -9360,7 +9405,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:L24"/>
+  <dimension ref="A1:O24"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="37" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -9368,26 +9413,31 @@
     <col min="6" max="6" width="20.83203125" customWidth="1"/>
     <col min="7" max="7" width="27.5" customWidth="1"/>
     <col min="8" max="8" width="87.5" style="15" customWidth="1"/>
-    <col min="11" max="11" width="12.33203125" customWidth="1"/>
+    <col min="11" max="11" width="41.6640625" customWidth="1"/>
     <col min="12" max="12" width="23.1640625" customWidth="1"/>
+    <col min="14" max="14" width="19.6640625" style="30" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="28" customHeight="1">
-      <c r="A1" s="25" t="s">
+    <row r="1" spans="1:15" ht="28" customHeight="1">
+      <c r="A1" s="26" t="s">
         <v>378</v>
       </c>
-      <c r="B1" s="25"/>
-      <c r="F1" s="25" t="s">
+      <c r="B1" s="26"/>
+      <c r="F1" s="26" t="s">
         <v>438</v>
       </c>
-      <c r="G1" s="25"/>
-      <c r="H1" s="25"/>
-      <c r="K1" s="25" t="s">
+      <c r="G1" s="26"/>
+      <c r="H1" s="26"/>
+      <c r="K1" s="26" t="s">
         <v>440</v>
       </c>
-      <c r="L1" s="25"/>
-    </row>
-    <row r="2" spans="1:12" ht="19" customHeight="1">
+      <c r="L1" s="26"/>
+      <c r="N1" s="26" t="s">
+        <v>449</v>
+      </c>
+      <c r="O1" s="26"/>
+    </row>
+    <row r="2" spans="1:15" ht="19" customHeight="1">
       <c r="A2" s="12" t="s">
         <v>379</v>
       </c>
@@ -9401,11 +9451,15 @@
       <c r="H2" s="16" t="s">
         <v>425</v>
       </c>
-      <c r="K2" t="s">
+      <c r="K2" s="27" t="s">
         <v>439</v>
       </c>
-    </row>
-    <row r="3" spans="1:12" ht="37" customHeight="1">
+      <c r="L2" s="27"/>
+      <c r="N2" s="29" t="s">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" ht="37" customHeight="1">
       <c r="A3" s="11" t="s">
         <v>380</v>
       </c>
@@ -9421,8 +9475,11 @@
       <c r="H3" s="19" t="s">
         <v>434</v>
       </c>
-    </row>
-    <row r="4" spans="1:12" ht="37" customHeight="1">
+      <c r="N3" s="28" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" ht="37" customHeight="1">
       <c r="A4" s="11" t="s">
         <v>382</v>
       </c>
@@ -9438,8 +9495,11 @@
       <c r="H4" s="19" t="s">
         <v>435</v>
       </c>
-    </row>
-    <row r="5" spans="1:12" ht="50" customHeight="1">
+      <c r="N4" s="28" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" ht="50" customHeight="1">
       <c r="A5" s="11"/>
       <c r="B5" s="11"/>
       <c r="F5" s="14" t="s">
@@ -9451,8 +9511,11 @@
       <c r="H5" s="19" t="s">
         <v>436</v>
       </c>
-    </row>
-    <row r="6" spans="1:12" ht="37" customHeight="1">
+      <c r="N5" s="29" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" ht="37" customHeight="1">
       <c r="A6" s="12" t="s">
         <v>384</v>
       </c>
@@ -9467,7 +9530,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="7" spans="1:12" ht="21" customHeight="1">
+    <row r="7" spans="1:15" ht="21" customHeight="1">
       <c r="A7" s="11" t="s">
         <v>385</v>
       </c>
@@ -9475,7 +9538,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="8" spans="1:12" ht="21" customHeight="1">
+    <row r="8" spans="1:15" ht="21" customHeight="1">
       <c r="A8" s="11" t="s">
         <v>387</v>
       </c>
@@ -9483,7 +9546,7 @@
         <v>388</v>
       </c>
     </row>
-    <row r="9" spans="1:12" ht="21" customHeight="1">
+    <row r="9" spans="1:15" ht="21" customHeight="1">
       <c r="A9" s="11" t="s">
         <v>389</v>
       </c>
@@ -9491,7 +9554,7 @@
         <v>390</v>
       </c>
     </row>
-    <row r="10" spans="1:12" ht="21" customHeight="1">
+    <row r="10" spans="1:15" ht="21" customHeight="1">
       <c r="A10" s="11" t="s">
         <v>391</v>
       </c>
@@ -9499,7 +9562,7 @@
         <v>392</v>
       </c>
     </row>
-    <row r="11" spans="1:12" ht="21" customHeight="1">
+    <row r="11" spans="1:15" ht="21" customHeight="1">
       <c r="A11" s="11" t="s">
         <v>393</v>
       </c>
@@ -9507,17 +9570,17 @@
         <v>394</v>
       </c>
     </row>
-    <row r="12" spans="1:12" ht="21" customHeight="1">
+    <row r="12" spans="1:15" ht="21" customHeight="1">
       <c r="A12" s="11"/>
       <c r="B12" s="11"/>
     </row>
-    <row r="13" spans="1:12" ht="21" customHeight="1">
+    <row r="13" spans="1:15" ht="21" customHeight="1">
       <c r="A13" s="12" t="s">
         <v>395</v>
       </c>
       <c r="B13" s="11"/>
     </row>
-    <row r="14" spans="1:12" ht="21" customHeight="1">
+    <row r="14" spans="1:15" ht="21" customHeight="1">
       <c r="A14" s="11" t="s">
         <v>4</v>
       </c>
@@ -9525,7 +9588,7 @@
         <v>396</v>
       </c>
     </row>
-    <row r="15" spans="1:12" ht="21" customHeight="1">
+    <row r="15" spans="1:15" ht="21" customHeight="1">
       <c r="A15" s="11" t="s">
         <v>8</v>
       </c>
@@ -9533,7 +9596,7 @@
         <v>397</v>
       </c>
     </row>
-    <row r="16" spans="1:12" ht="21" customHeight="1">
+    <row r="16" spans="1:15" ht="21" customHeight="1">
       <c r="A16" s="11" t="s">
         <v>14</v>
       </c>
@@ -9593,11 +9656,19 @@
     </row>
     <row r="24" spans="1:2" ht="21" customHeight="1"/>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="5">
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="K1:L1"/>
     <mergeCell ref="F1:H1"/>
+    <mergeCell ref="K2:L2"/>
+    <mergeCell ref="N1:O1"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="N2" r:id="rId1" xr:uid="{9A37A3C7-CBFE-4146-B59A-FA044143BB36}"/>
+    <hyperlink ref="N5" r:id="rId2" xr:uid="{0B0ADDF0-D173-5B4F-9902-098AA5491551}"/>
+    <hyperlink ref="N3" r:id="rId3" xr:uid="{5BC376E2-5ADC-F043-973F-256DA036B079}"/>
+    <hyperlink ref="N4" r:id="rId4" xr:uid="{C7040BD1-70D5-BC41-A914-3E6B27B4228A}"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -9638,10 +9709,10 @@
     </row>
     <row r="2" spans="2:10" ht="17">
       <c r="B2" s="1"/>
-      <c r="C2" s="24" t="s">
+      <c r="C2" s="25" t="s">
         <v>0</v>
       </c>
-      <c r="D2" s="24"/>
+      <c r="D2" s="25"/>
       <c r="E2" s="1"/>
       <c r="F2" s="1"/>
       <c r="G2" s="1"/>

</xml_diff>

<commit_message>
Feat: add JavaScript-based passengerCounter and a simple Calculatorpage
</commit_message>
<xml_diff>
--- a/side-project/Scrimba全栈学习路径进度追踪表.xlsx
+++ b/side-project/Scrimba全栈学习路径进度追踪表.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ersheng/Desktop/web_project/public-note/side-project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D098BA1-B226-4B4B-BF33-EABE606DC73F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD2C0FBA-F054-F146-938D-1301FB878B0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="10240" yWindow="2920" windowWidth="40960" windowHeight="23360" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,8 +37,34 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>tc={1F17599A-7801-DD42-9181-9FD3B35CA247}</author>
+  </authors>
+  <commentList>
+    <comment ref="O3" authorId="0" shapeId="0" xr:uid="{1F17599A-7801-DD42-9181-9FD3B35CA247}">
+      <text>
+        <t xml:space="preserve">[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    ERSHENG:
+2026-10-02，下载了firefox浏览器，以满足网页测试中的相关要求（多rendiner engine测试
+Reply:
+    如何弄一个本地测试服务器？当前在VSC中已经安装了一个插件，但不够灵活，后续可能要尝试新的选项；
+Reply:
+    尝试tinyPNG 以用于压缩图片等 操作，替代方案是苹果设备中的 preview /预览。 稍微复杂一些的选项包括 photopea  这类线上工具。 
+Reply:
+    网页部署： 1. Github Pages,在用的；Netlify，已经与github联通
+ 2. codepen, JSFiddle 做简单的demo;  3. </t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="966" uniqueCount="455">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="973" uniqueCount="461">
   <si>
     <t>Introduction</t>
   </si>
@@ -1953,6 +1979,24 @@
   <si>
     <t>进行中，家乡推介</t>
   </si>
+  <si>
+    <t xml:space="preserve">Environment setup </t>
+  </si>
+  <si>
+    <t>sub-topic</t>
+  </si>
+  <si>
+    <t>Core Modules</t>
+  </si>
+  <si>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>Browsing the web</t>
+  </si>
+  <si>
+    <t>Scrimba Docs</t>
+  </si>
 </sst>
 </file>
 
@@ -1962,7 +2006,7 @@
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="14">
+  <fonts count="21">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2050,18 +2094,63 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Yahei"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Yahei"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="16"/>
+      <color theme="1"/>
+      <name val="Yahei"/>
+    </font>
+    <font>
+      <sz val="16"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
+    <font>
       <u/>
-      <sz val="11"/>
+      <sz val="14"/>
       <color theme="10"/>
       <name val="Yahei"/>
     </font>
     <font>
-      <sz val="11"/>
+      <u/>
+      <sz val="14"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
       <color theme="1"/>
-      <name val="Yahei"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="12">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2122,6 +2211,12 @@
         <bgColor rgb="FF2F5496"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="4">
     <border>
@@ -2172,7 +2267,7 @@
     <xf numFmtId="9" fontId="9" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -2241,16 +2336,76 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="2"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="2" applyFont="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="2" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hyperlink" xfId="2" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
-  <dxfs count="6">
+  <dxfs count="9">
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i/>
+      </font>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF006100"/>
@@ -2316,6 +2471,12 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <person displayName="si Frank" id="{46818ABC-E3D4-9746-B9F4-E2842DECFE29}" userId="fbb996fee7239c93" providerId="Windows Live"/>
+</personList>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2601,6 +2762,27 @@
 </a:theme>
 </file>
 
+<file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
+<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="O3" dT="2026-10-02T14:53:42.82" personId="{46818ABC-E3D4-9746-B9F4-E2842DECFE29}" id="{1F17599A-7801-DD42-9181-9FD3B35CA247}">
+    <text xml:space="preserve">ERSHENG:
+2026-10-02，下载了firefox浏览器，以满足网页测试中的相关要求（多rendiner engine测试
+</text>
+  </threadedComment>
+  <threadedComment ref="O3" dT="2026-10-02T14:56:51.97" personId="{46818ABC-E3D4-9746-B9F4-E2842DECFE29}" id="{C5456653-DD64-7C42-A09E-F747CA2ED549}" parentId="{1F17599A-7801-DD42-9181-9FD3B35CA247}">
+    <text xml:space="preserve">如何弄一个本地测试服务器？当前在VSC中已经安装了一个插件，但不够灵活，后续可能要尝试新的选项；
+</text>
+  </threadedComment>
+  <threadedComment ref="O3" dT="2026-10-02T14:58:37.47" personId="{46818ABC-E3D4-9746-B9F4-E2842DECFE29}" id="{017E7752-6CC3-964F-999F-6B6762A30A91}" parentId="{1F17599A-7801-DD42-9181-9FD3B35CA247}">
+    <text xml:space="preserve">尝试tinyPNG 以用于压缩图片等 操作，替代方案是苹果设备中的 preview /预览。 稍微复杂一些的选项包括 photopea  这类线上工具。 </text>
+  </threadedComment>
+  <threadedComment ref="O3" dT="2026-10-02T15:13:42.36" personId="{46818ABC-E3D4-9746-B9F4-E2842DECFE29}" id="{E345D5BF-FD2B-9044-9983-C822F954991B}" parentId="{1F17599A-7801-DD42-9181-9FD3B35CA247}">
+    <text xml:space="preserve">网页部署： 1. Github Pages,在用的；Netlify，已经与github联通
+ 2. codepen, JSFiddle 做简单的demo;  3. </text>
+  </threadedComment>
+</ThreadedComments>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:L215"/>
@@ -9384,15 +9566,15 @@
     <mergeCell ref="B12:C12"/>
   </mergeCells>
   <conditionalFormatting sqref="G1:G1048576">
-    <cfRule type="cellIs" dxfId="5" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="8" priority="1" operator="equal">
       <formula>"Pending"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="7" priority="2" operator="equal">
       <formula>"Done"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G2:G215">
-    <cfRule type="cellIs" dxfId="3" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="6" priority="3" operator="equal">
       <formula>"已完成"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -9404,8 +9586,8 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:O24"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:Q32"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="37" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -9415,10 +9597,13 @@
     <col min="8" max="8" width="87.5" style="15" customWidth="1"/>
     <col min="11" max="11" width="41.6640625" customWidth="1"/>
     <col min="12" max="12" width="23.1640625" customWidth="1"/>
-    <col min="14" max="14" width="19.6640625" style="30" customWidth="1"/>
+    <col min="14" max="14" width="27.5" style="35" customWidth="1"/>
+    <col min="15" max="15" width="21.83203125" style="27" customWidth="1"/>
+    <col min="16" max="16" width="13.5" style="27" customWidth="1"/>
+    <col min="17" max="17" width="11.83203125" style="37" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="28" customHeight="1">
+    <row r="1" spans="1:17" ht="28" customHeight="1">
       <c r="A1" s="26" t="s">
         <v>378</v>
       </c>
@@ -9436,8 +9621,9 @@
         <v>449</v>
       </c>
       <c r="O1" s="26"/>
-    </row>
-    <row r="2" spans="1:15" ht="19" customHeight="1">
+      <c r="Q1" s="27"/>
+    </row>
+    <row r="2" spans="1:17" ht="19" customHeight="1">
       <c r="A2" s="12" t="s">
         <v>379</v>
       </c>
@@ -9451,15 +9637,24 @@
       <c r="H2" s="16" t="s">
         <v>425</v>
       </c>
-      <c r="K2" s="27" t="s">
+      <c r="K2" s="28" t="s">
         <v>439</v>
       </c>
-      <c r="L2" s="27"/>
+      <c r="L2" s="28"/>
       <c r="N2" s="29" t="s">
-        <v>450</v>
-      </c>
-    </row>
-    <row r="3" spans="1:15" ht="37" customHeight="1">
+        <v>457</v>
+      </c>
+      <c r="O2" s="30" t="s">
+        <v>456</v>
+      </c>
+      <c r="P2" s="30" t="s">
+        <v>417</v>
+      </c>
+      <c r="Q2" s="30" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17" ht="37" customHeight="1">
       <c r="A3" s="11" t="s">
         <v>380</v>
       </c>
@@ -9475,11 +9670,21 @@
       <c r="H3" s="19" t="s">
         <v>434</v>
       </c>
-      <c r="N3" s="28" t="s">
-        <v>452</v>
-      </c>
-    </row>
-    <row r="4" spans="1:15" ht="37" customHeight="1">
+      <c r="N3" s="31" t="s">
+        <v>450</v>
+      </c>
+      <c r="O3" s="32" t="s">
+        <v>455</v>
+      </c>
+      <c r="P3" s="38" t="str">
+        <f>IF(Q3&lt;&gt;"","Done","Pending")</f>
+        <v>Done</v>
+      </c>
+      <c r="Q3" s="36">
+        <v>46297</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17" ht="37" customHeight="1">
       <c r="A4" s="11" t="s">
         <v>382</v>
       </c>
@@ -9495,11 +9700,16 @@
       <c r="H4" s="19" t="s">
         <v>435</v>
       </c>
-      <c r="N4" s="28" t="s">
-        <v>453</v>
-      </c>
-    </row>
-    <row r="5" spans="1:15" ht="50" customHeight="1">
+      <c r="N4" s="33"/>
+      <c r="O4" s="32" t="s">
+        <v>459</v>
+      </c>
+      <c r="P4" s="38" t="str">
+        <f t="shared" ref="P4:P32" si="0">IF(Q4&lt;&gt;"","Done","Pending")</f>
+        <v>Pending</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17" ht="50" customHeight="1">
       <c r="A5" s="11"/>
       <c r="B5" s="11"/>
       <c r="F5" s="14" t="s">
@@ -9511,11 +9721,14 @@
       <c r="H5" s="19" t="s">
         <v>436</v>
       </c>
-      <c r="N5" s="29" t="s">
-        <v>451</v>
-      </c>
-    </row>
-    <row r="6" spans="1:15" ht="37" customHeight="1">
+      <c r="N5" s="33"/>
+      <c r="O5" s="32"/>
+      <c r="P5" s="38" t="str">
+        <f t="shared" si="0"/>
+        <v>Pending</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17" ht="37" customHeight="1">
       <c r="A6" s="12" t="s">
         <v>384</v>
       </c>
@@ -9529,132 +9742,274 @@
       <c r="H6" s="19" t="s">
         <v>437</v>
       </c>
-    </row>
-    <row r="7" spans="1:15" ht="21" customHeight="1">
+      <c r="N6" s="33"/>
+      <c r="O6" s="32"/>
+      <c r="P6" s="38" t="str">
+        <f t="shared" si="0"/>
+        <v>Pending</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17" ht="21" customHeight="1">
       <c r="A7" s="11" t="s">
         <v>385</v>
       </c>
       <c r="B7" s="11" t="s">
         <v>386</v>
       </c>
-    </row>
-    <row r="8" spans="1:15" ht="21" customHeight="1">
+      <c r="N7" s="34" t="s">
+        <v>452</v>
+      </c>
+      <c r="O7" s="32"/>
+      <c r="P7" s="38" t="str">
+        <f t="shared" si="0"/>
+        <v>Pending</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17" ht="21" customHeight="1">
       <c r="A8" s="11" t="s">
         <v>387</v>
       </c>
       <c r="B8" s="11" t="s">
         <v>388</v>
       </c>
-    </row>
-    <row r="9" spans="1:15" ht="21" customHeight="1">
+      <c r="N8" s="34" t="s">
+        <v>453</v>
+      </c>
+      <c r="O8" s="32"/>
+      <c r="P8" s="38" t="str">
+        <f t="shared" si="0"/>
+        <v>Pending</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17" ht="21" customHeight="1">
       <c r="A9" s="11" t="s">
         <v>389</v>
       </c>
       <c r="B9" s="11" t="s">
         <v>390</v>
       </c>
-    </row>
-    <row r="10" spans="1:15" ht="21" customHeight="1">
+      <c r="N9" s="31" t="s">
+        <v>451</v>
+      </c>
+      <c r="O9" s="32"/>
+      <c r="P9" s="38" t="str">
+        <f t="shared" si="0"/>
+        <v>Pending</v>
+      </c>
+    </row>
+    <row r="10" spans="1:17" ht="21" customHeight="1">
       <c r="A10" s="11" t="s">
         <v>391</v>
       </c>
       <c r="B10" s="11" t="s">
         <v>392</v>
       </c>
-    </row>
-    <row r="11" spans="1:15" ht="21" customHeight="1">
+      <c r="P10" s="38" t="str">
+        <f t="shared" si="0"/>
+        <v>Pending</v>
+      </c>
+    </row>
+    <row r="11" spans="1:17" ht="21" customHeight="1">
       <c r="A11" s="11" t="s">
         <v>393</v>
       </c>
       <c r="B11" s="11" t="s">
         <v>394</v>
       </c>
-    </row>
-    <row r="12" spans="1:15" ht="21" customHeight="1">
+      <c r="P11" s="38" t="str">
+        <f t="shared" si="0"/>
+        <v>Pending</v>
+      </c>
+    </row>
+    <row r="12" spans="1:17" ht="21" customHeight="1">
       <c r="A12" s="11"/>
       <c r="B12" s="11"/>
-    </row>
-    <row r="13" spans="1:15" ht="21" customHeight="1">
+      <c r="N12" s="39" t="s">
+        <v>460</v>
+      </c>
+      <c r="P12" s="38" t="str">
+        <f t="shared" si="0"/>
+        <v>Pending</v>
+      </c>
+    </row>
+    <row r="13" spans="1:17" ht="21" customHeight="1">
       <c r="A13" s="12" t="s">
         <v>395</v>
       </c>
       <c r="B13" s="11"/>
-    </row>
-    <row r="14" spans="1:15" ht="21" customHeight="1">
+      <c r="P13" s="38" t="str">
+        <f t="shared" si="0"/>
+        <v>Pending</v>
+      </c>
+    </row>
+    <row r="14" spans="1:17" ht="21" customHeight="1">
       <c r="A14" s="11" t="s">
         <v>4</v>
       </c>
       <c r="B14" s="11" t="s">
         <v>396</v>
       </c>
-    </row>
-    <row r="15" spans="1:15" ht="21" customHeight="1">
+      <c r="P14" s="38" t="str">
+        <f t="shared" si="0"/>
+        <v>Pending</v>
+      </c>
+    </row>
+    <row r="15" spans="1:17" ht="21" customHeight="1">
       <c r="A15" s="11" t="s">
         <v>8</v>
       </c>
       <c r="B15" s="11" t="s">
         <v>397</v>
       </c>
-    </row>
-    <row r="16" spans="1:15" ht="21" customHeight="1">
+      <c r="P15" s="38" t="str">
+        <f t="shared" si="0"/>
+        <v>Pending</v>
+      </c>
+    </row>
+    <row r="16" spans="1:17" ht="21" customHeight="1">
       <c r="A16" s="11" t="s">
         <v>14</v>
       </c>
       <c r="B16" s="11" t="s">
         <v>398</v>
       </c>
-    </row>
-    <row r="17" spans="1:2" ht="21" customHeight="1">
+      <c r="P16" s="38" t="str">
+        <f t="shared" si="0"/>
+        <v>Pending</v>
+      </c>
+    </row>
+    <row r="17" spans="1:16" ht="21" customHeight="1">
       <c r="A17" s="11"/>
       <c r="B17" s="11"/>
-    </row>
-    <row r="18" spans="1:2" ht="21" customHeight="1">
+      <c r="P17" s="38" t="str">
+        <f t="shared" si="0"/>
+        <v>Pending</v>
+      </c>
+    </row>
+    <row r="18" spans="1:16" ht="21" customHeight="1">
       <c r="A18" s="12" t="s">
         <v>399</v>
       </c>
       <c r="B18" s="11"/>
-    </row>
-    <row r="19" spans="1:2" ht="21" customHeight="1">
+      <c r="P18" s="38" t="str">
+        <f t="shared" si="0"/>
+        <v>Pending</v>
+      </c>
+    </row>
+    <row r="19" spans="1:16" ht="21" customHeight="1">
       <c r="A19" s="11" t="s">
         <v>400</v>
       </c>
       <c r="B19" s="11" t="s">
         <v>401</v>
       </c>
-    </row>
-    <row r="20" spans="1:2" ht="21" customHeight="1">
+      <c r="P19" s="38" t="str">
+        <f t="shared" si="0"/>
+        <v>Pending</v>
+      </c>
+    </row>
+    <row r="20" spans="1:16" ht="21" customHeight="1">
       <c r="A20" s="11" t="s">
         <v>402</v>
       </c>
       <c r="B20" s="11" t="s">
         <v>403</v>
       </c>
-    </row>
-    <row r="21" spans="1:2" ht="21" customHeight="1">
+      <c r="P20" s="38" t="str">
+        <f t="shared" si="0"/>
+        <v>Pending</v>
+      </c>
+    </row>
+    <row r="21" spans="1:16" ht="21" customHeight="1">
       <c r="A21" s="11" t="s">
         <v>404</v>
       </c>
       <c r="B21" s="11" t="s">
         <v>405</v>
       </c>
-    </row>
-    <row r="22" spans="1:2" ht="21" customHeight="1">
+      <c r="P21" s="38" t="str">
+        <f t="shared" si="0"/>
+        <v>Pending</v>
+      </c>
+    </row>
+    <row r="22" spans="1:16" ht="21" customHeight="1">
       <c r="A22" s="11" t="s">
         <v>406</v>
       </c>
       <c r="B22" s="11" t="s">
         <v>407</v>
       </c>
-    </row>
-    <row r="23" spans="1:2" ht="21" customHeight="1">
+      <c r="P22" s="38" t="str">
+        <f t="shared" si="0"/>
+        <v>Pending</v>
+      </c>
+    </row>
+    <row r="23" spans="1:16" ht="21" customHeight="1">
       <c r="A23" s="11" t="s">
         <v>408</v>
       </c>
       <c r="B23" s="11" t="s">
         <v>409</v>
       </c>
-    </row>
-    <row r="24" spans="1:2" ht="21" customHeight="1"/>
+      <c r="P23" s="38" t="str">
+        <f t="shared" si="0"/>
+        <v>Pending</v>
+      </c>
+    </row>
+    <row r="24" spans="1:16" ht="21" customHeight="1">
+      <c r="P24" s="38" t="str">
+        <f t="shared" si="0"/>
+        <v>Pending</v>
+      </c>
+    </row>
+    <row r="25" spans="1:16" ht="37" customHeight="1">
+      <c r="P25" s="38" t="str">
+        <f t="shared" si="0"/>
+        <v>Pending</v>
+      </c>
+    </row>
+    <row r="26" spans="1:16" ht="37" customHeight="1">
+      <c r="P26" s="38" t="str">
+        <f t="shared" si="0"/>
+        <v>Pending</v>
+      </c>
+    </row>
+    <row r="27" spans="1:16" ht="37" customHeight="1">
+      <c r="P27" s="38" t="str">
+        <f t="shared" si="0"/>
+        <v>Pending</v>
+      </c>
+    </row>
+    <row r="28" spans="1:16" ht="37" customHeight="1">
+      <c r="P28" s="38" t="str">
+        <f t="shared" si="0"/>
+        <v>Pending</v>
+      </c>
+    </row>
+    <row r="29" spans="1:16" ht="37" customHeight="1">
+      <c r="P29" s="38" t="str">
+        <f t="shared" si="0"/>
+        <v>Pending</v>
+      </c>
+    </row>
+    <row r="30" spans="1:16" ht="37" customHeight="1">
+      <c r="P30" s="38" t="str">
+        <f t="shared" si="0"/>
+        <v>Pending</v>
+      </c>
+    </row>
+    <row r="31" spans="1:16" ht="37" customHeight="1">
+      <c r="P31" s="38" t="str">
+        <f t="shared" si="0"/>
+        <v>Pending</v>
+      </c>
+    </row>
+    <row r="32" spans="1:16" ht="37" customHeight="1">
+      <c r="P32" s="38" t="str">
+        <f t="shared" si="0"/>
+        <v>Pending</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="A1:B1"/>
@@ -9663,13 +10018,28 @@
     <mergeCell ref="K2:L2"/>
     <mergeCell ref="N1:O1"/>
   </mergeCells>
+  <conditionalFormatting sqref="P3:P32">
+    <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
+      <formula>"Pending"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
+      <formula>"Done"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="P3:P32">
+    <cfRule type="cellIs" dxfId="0" priority="3" operator="equal">
+      <formula>"已完成"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <hyperlinks>
-    <hyperlink ref="N2" r:id="rId1" xr:uid="{9A37A3C7-CBFE-4146-B59A-FA044143BB36}"/>
-    <hyperlink ref="N5" r:id="rId2" xr:uid="{0B0ADDF0-D173-5B4F-9902-098AA5491551}"/>
-    <hyperlink ref="N3" r:id="rId3" xr:uid="{5BC376E2-5ADC-F043-973F-256DA036B079}"/>
-    <hyperlink ref="N4" r:id="rId4" xr:uid="{C7040BD1-70D5-BC41-A914-3E6B27B4228A}"/>
+    <hyperlink ref="N3" r:id="rId1" xr:uid="{9A37A3C7-CBFE-4146-B59A-FA044143BB36}"/>
+    <hyperlink ref="N9" r:id="rId2" xr:uid="{0B0ADDF0-D173-5B4F-9902-098AA5491551}"/>
+    <hyperlink ref="N7" r:id="rId3" xr:uid="{5BC376E2-5ADC-F043-973F-256DA036B079}"/>
+    <hyperlink ref="N8" r:id="rId4" xr:uid="{C7040BD1-70D5-BC41-A914-3E6B27B4228A}"/>
+    <hyperlink ref="N12" r:id="rId5" xr:uid="{9E6E4015-A9C4-4241-A135-519F25BDA421}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing r:id="rId6"/>
 </worksheet>
 </file>
 
@@ -9781,15 +10151,15 @@
     <mergeCell ref="C2:D2"/>
   </mergeCells>
   <conditionalFormatting sqref="H1:H4">
-    <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="5" priority="1" operator="equal">
       <formula>"Pending"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="4" priority="2" operator="equal">
       <formula>"Done"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H2:H4">
-    <cfRule type="cellIs" dxfId="0" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="3" priority="3" operator="equal">
       <formula>"已完成"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
feat: add game score-tracker on 261006
</commit_message>
<xml_diff>
--- a/side-project/Scrimba全栈学习路径进度追踪表.xlsx
+++ b/side-project/Scrimba全栈学习路径进度追踪表.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ersheng/Desktop/web_project/public-note/side-project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD2C0FBA-F054-F146-938D-1301FB878B0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F32077F-9EB0-7F47-B1C0-B2DF8B1A4B80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10240" yWindow="2920" windowWidth="40960" windowHeight="23360" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="10240" yWindow="3820" windowWidth="40960" windowHeight="23360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="学习进度追踪" sheetId="1" r:id="rId1"/>
@@ -5481,17 +5481,19 @@
       </c>
       <c r="G81" s="5" t="str">
         <f t="shared" ref="G81:G88" si="5">IF(H81&lt;&gt;"","Done","Pending")</f>
-        <v>Pending</v>
-      </c>
-      <c r="H81" s="6"/>
+        <v>Done</v>
+      </c>
+      <c r="H81" s="6">
+        <v>46299</v>
+      </c>
       <c r="I81" s="3"/>
-      <c r="J81" t="str">
+      <c r="J81" s="21">
         <f t="shared" si="3"/>
-        <v/>
+        <v>0.38974358974358975</v>
       </c>
       <c r="K81" s="24">
         <f>COUNTIF($G$3:G81,"Done")</f>
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="82" spans="1:11" ht="20" customHeight="1">
@@ -5513,17 +5515,19 @@
       </c>
       <c r="G82" s="5" t="str">
         <f t="shared" si="5"/>
-        <v>Pending</v>
-      </c>
-      <c r="H82" s="6"/>
+        <v>Done</v>
+      </c>
+      <c r="H82" s="6">
+        <v>46300</v>
+      </c>
       <c r="I82" s="3"/>
-      <c r="J82" t="str">
+      <c r="J82" s="21">
         <f t="shared" si="3"/>
-        <v/>
+        <v>0.39487179487179486</v>
       </c>
       <c r="K82" s="24">
         <f>COUNTIF($G$3:G82,"Done")</f>
-        <v>75</v>
+        <v>77</v>
       </c>
     </row>
     <row r="83" spans="1:11" ht="20" customHeight="1">
@@ -5545,17 +5549,19 @@
       </c>
       <c r="G83" s="5" t="str">
         <f t="shared" si="5"/>
-        <v>Pending</v>
-      </c>
-      <c r="H83" s="6"/>
+        <v>Done</v>
+      </c>
+      <c r="H83" s="6">
+        <v>46301</v>
+      </c>
       <c r="I83" s="8"/>
-      <c r="J83" t="str">
+      <c r="J83" s="21">
         <f t="shared" si="3"/>
-        <v/>
+        <v>0.4</v>
       </c>
       <c r="K83" s="24">
         <f>COUNTIF($G$3:G83,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="84" spans="1:11" ht="20" customHeight="1">
@@ -5581,13 +5587,13 @@
       </c>
       <c r="H84" s="6"/>
       <c r="I84" s="3"/>
-      <c r="J84" t="str">
+      <c r="J84" s="21" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="K84" s="24">
         <f>COUNTIF($G$3:G84,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="85" spans="1:11" ht="20" customHeight="1">
@@ -5613,13 +5619,13 @@
       </c>
       <c r="H85" s="6"/>
       <c r="I85" s="8"/>
-      <c r="J85" t="str">
+      <c r="J85" s="21" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="K85" s="24">
         <f>COUNTIF($G$3:G85,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="86" spans="1:11" ht="20" customHeight="1">
@@ -5645,13 +5651,13 @@
       </c>
       <c r="H86" s="6"/>
       <c r="I86" s="3"/>
-      <c r="J86" t="str">
+      <c r="J86" s="21" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="K86" s="24">
         <f>COUNTIF($G$3:G86,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="87" spans="1:11" ht="20" customHeight="1">
@@ -5677,13 +5683,13 @@
       </c>
       <c r="H87" s="6"/>
       <c r="I87" s="8"/>
-      <c r="J87" t="str">
+      <c r="J87" s="21" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="K87" s="24">
         <f>COUNTIF($G$3:G87,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="88" spans="1:11" ht="20" customHeight="1">
@@ -5709,13 +5715,13 @@
       </c>
       <c r="H88" s="6"/>
       <c r="I88" s="3"/>
-      <c r="J88" t="str">
+      <c r="J88" s="21" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="K88" s="24">
         <f>COUNTIF($G$3:G88,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="89" spans="1:11" ht="20" customHeight="1">
@@ -5732,7 +5738,7 @@
       <c r="I89" s="1"/>
       <c r="K89" s="24">
         <f>COUNTIF($G$3:G89,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="90" spans="1:11" ht="20" customHeight="1">
@@ -5758,13 +5764,13 @@
       </c>
       <c r="H90" s="6"/>
       <c r="I90" s="8"/>
-      <c r="J90" t="str">
+      <c r="J90" s="21" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="K90" s="24">
         <f>COUNTIF($G$3:G90,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="91" spans="1:11" ht="20" customHeight="1">
@@ -5790,13 +5796,13 @@
       </c>
       <c r="H91" s="6"/>
       <c r="I91" s="3"/>
-      <c r="J91" t="str">
+      <c r="J91" s="21" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="K91" s="24">
         <f>COUNTIF($G$3:G91,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="92" spans="1:11" ht="20" customHeight="1">
@@ -5822,13 +5828,13 @@
       </c>
       <c r="H92" s="6"/>
       <c r="I92" s="8"/>
-      <c r="J92" t="str">
+      <c r="J92" s="21" t="str">
         <f t="shared" ref="J92:J155" si="7">IF(G92="Pending","",K92/195)</f>
         <v/>
       </c>
       <c r="K92" s="24">
         <f>COUNTIF($G$3:G92,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="93" spans="1:11" ht="20" customHeight="1">
@@ -5854,13 +5860,13 @@
       </c>
       <c r="H93" s="6"/>
       <c r="I93" s="3"/>
-      <c r="J93" t="str">
+      <c r="J93" s="21" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K93" s="24">
         <f>COUNTIF($G$3:G93,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="94" spans="1:11" ht="20" customHeight="1">
@@ -5877,7 +5883,7 @@
       <c r="I94" s="1"/>
       <c r="K94" s="24">
         <f>COUNTIF($G$3:G94,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="95" spans="1:11" ht="20" customHeight="1">
@@ -5903,13 +5909,13 @@
       </c>
       <c r="H95" s="6"/>
       <c r="I95" s="8"/>
-      <c r="J95" t="str">
+      <c r="J95" s="21" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K95" s="24">
         <f>COUNTIF($G$3:G95,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="96" spans="1:11" ht="20" customHeight="1">
@@ -5935,13 +5941,13 @@
       </c>
       <c r="H96" s="6"/>
       <c r="I96" s="3"/>
-      <c r="J96" t="str">
+      <c r="J96" s="21" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K96" s="24">
         <f>COUNTIF($G$3:G96,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="97" spans="1:11" ht="20" customHeight="1">
@@ -5967,13 +5973,13 @@
       </c>
       <c r="H97" s="6"/>
       <c r="I97" s="8"/>
-      <c r="J97" t="str">
+      <c r="J97" s="21" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K97" s="24">
         <f>COUNTIF($G$3:G97,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="98" spans="1:11" ht="20" customHeight="1">
@@ -5999,13 +6005,13 @@
       </c>
       <c r="H98" s="6"/>
       <c r="I98" s="3"/>
-      <c r="J98" t="str">
+      <c r="J98" s="21" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K98" s="24">
         <f>COUNTIF($G$3:G98,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="99" spans="1:11" ht="20" customHeight="1">
@@ -6031,13 +6037,13 @@
       </c>
       <c r="H99" s="6"/>
       <c r="I99" s="8"/>
-      <c r="J99" t="str">
+      <c r="J99" s="21" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K99" s="24">
         <f>COUNTIF($G$3:G99,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="100" spans="1:11" ht="20" customHeight="1">
@@ -6063,13 +6069,13 @@
       </c>
       <c r="H100" s="6"/>
       <c r="I100" s="3"/>
-      <c r="J100" t="str">
+      <c r="J100" s="21" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K100" s="24">
         <f>COUNTIF($G$3:G100,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="101" spans="1:11" ht="20" customHeight="1">
@@ -6095,13 +6101,13 @@
       </c>
       <c r="H101" s="6"/>
       <c r="I101" s="8"/>
-      <c r="J101" t="str">
+      <c r="J101" s="21" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K101" s="24">
         <f>COUNTIF($G$3:G101,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="102" spans="1:11" ht="20" customHeight="1">
@@ -6127,13 +6133,13 @@
       </c>
       <c r="H102" s="6"/>
       <c r="I102" s="3"/>
-      <c r="J102" t="str">
+      <c r="J102" s="21" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K102" s="24">
         <f>COUNTIF($G$3:G102,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="103" spans="1:11" ht="20" customHeight="1">
@@ -6159,13 +6165,13 @@
       </c>
       <c r="H103" s="6"/>
       <c r="I103" s="8"/>
-      <c r="J103" t="str">
+      <c r="J103" s="21" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K103" s="24">
         <f>COUNTIF($G$3:G103,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="104" spans="1:11" ht="20" customHeight="1">
@@ -6191,13 +6197,13 @@
       </c>
       <c r="H104" s="6"/>
       <c r="I104" s="3"/>
-      <c r="J104" t="str">
+      <c r="J104" s="21" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K104" s="24">
         <f>COUNTIF($G$3:G104,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="105" spans="1:11" ht="20" customHeight="1">
@@ -6223,13 +6229,13 @@
       </c>
       <c r="H105" s="6"/>
       <c r="I105" s="8"/>
-      <c r="J105" t="str">
+      <c r="J105" s="21" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K105" s="24">
         <f>COUNTIF($G$3:G105,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="106" spans="1:11" ht="20" customHeight="1">
@@ -6255,13 +6261,13 @@
       </c>
       <c r="H106" s="6"/>
       <c r="I106" s="3"/>
-      <c r="J106" t="str">
+      <c r="J106" s="21" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K106" s="24">
         <f>COUNTIF($G$3:G106,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="107" spans="1:11" ht="20" customHeight="1">
@@ -6287,13 +6293,13 @@
       </c>
       <c r="H107" s="6"/>
       <c r="I107" s="8"/>
-      <c r="J107" t="str">
+      <c r="J107" s="21" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K107" s="24">
         <f>COUNTIF($G$3:G107,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="108" spans="1:11" ht="20" customHeight="1">
@@ -6319,13 +6325,13 @@
       </c>
       <c r="H108" s="6"/>
       <c r="I108" s="3"/>
-      <c r="J108" t="str">
+      <c r="J108" s="21" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K108" s="24">
         <f>COUNTIF($G$3:G108,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="109" spans="1:11" ht="20" customHeight="1">
@@ -6351,13 +6357,13 @@
       </c>
       <c r="H109" s="6"/>
       <c r="I109" s="8"/>
-      <c r="J109" t="str">
+      <c r="J109" s="21" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K109" s="24">
         <f>COUNTIF($G$3:G109,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="110" spans="1:11" ht="20" customHeight="1">
@@ -6383,13 +6389,13 @@
       </c>
       <c r="H110" s="6"/>
       <c r="I110" s="3"/>
-      <c r="J110" t="str">
+      <c r="J110" s="21" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K110" s="24">
         <f>COUNTIF($G$3:G110,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="111" spans="1:11" ht="20" customHeight="1">
@@ -6415,13 +6421,13 @@
       </c>
       <c r="H111" s="6"/>
       <c r="I111" s="8"/>
-      <c r="J111" t="str">
+      <c r="J111" s="21" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K111" s="24">
         <f>COUNTIF($G$3:G111,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="112" spans="1:11" ht="20" customHeight="1">
@@ -6447,13 +6453,13 @@
       </c>
       <c r="H112" s="6"/>
       <c r="I112" s="3"/>
-      <c r="J112" t="str">
+      <c r="J112" s="21" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K112" s="24">
         <f>COUNTIF($G$3:G112,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="113" spans="1:11" ht="20" customHeight="1">
@@ -6479,13 +6485,13 @@
       </c>
       <c r="H113" s="6"/>
       <c r="I113" s="8"/>
-      <c r="J113" t="str">
+      <c r="J113" s="21" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K113" s="24">
         <f>COUNTIF($G$3:G113,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="114" spans="1:11" ht="20" customHeight="1">
@@ -6511,13 +6517,13 @@
       </c>
       <c r="H114" s="6"/>
       <c r="I114" s="3"/>
-      <c r="J114" t="str">
+      <c r="J114" s="21" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K114" s="24">
         <f>COUNTIF($G$3:G114,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="115" spans="1:11" ht="20" customHeight="1">
@@ -6543,13 +6549,13 @@
       </c>
       <c r="H115" s="6"/>
       <c r="I115" s="8"/>
-      <c r="J115" t="str">
+      <c r="J115" s="21" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K115" s="24">
         <f>COUNTIF($G$3:G115,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="116" spans="1:11" ht="20" customHeight="1">
@@ -6575,13 +6581,13 @@
       </c>
       <c r="H116" s="6"/>
       <c r="I116" s="3"/>
-      <c r="J116" t="str">
+      <c r="J116" s="21" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K116" s="24">
         <f>COUNTIF($G$3:G116,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="117" spans="1:11" ht="20" customHeight="1">
@@ -6607,13 +6613,13 @@
       </c>
       <c r="H117" s="6"/>
       <c r="I117" s="8"/>
-      <c r="J117" t="str">
+      <c r="J117" s="21" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K117" s="24">
         <f>COUNTIF($G$3:G117,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="118" spans="1:11" ht="20" customHeight="1">
@@ -6639,13 +6645,13 @@
       </c>
       <c r="H118" s="6"/>
       <c r="I118" s="3"/>
-      <c r="J118" t="str">
+      <c r="J118" s="21" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K118" s="24">
         <f>COUNTIF($G$3:G118,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="119" spans="1:11" ht="20" customHeight="1">
@@ -6671,13 +6677,13 @@
       </c>
       <c r="H119" s="6"/>
       <c r="I119" s="8"/>
-      <c r="J119" t="str">
+      <c r="J119" s="21" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K119" s="24">
         <f>COUNTIF($G$3:G119,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="120" spans="1:11" ht="20" customHeight="1">
@@ -6694,7 +6700,7 @@
       <c r="I120" s="1"/>
       <c r="K120" s="24">
         <f>COUNTIF($G$3:G120,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="121" spans="1:11" ht="20" customHeight="1">
@@ -6726,7 +6732,7 @@
       </c>
       <c r="K121" s="24">
         <f>COUNTIF($G$3:G121,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="122" spans="1:11" ht="20" customHeight="1">
@@ -6758,7 +6764,7 @@
       </c>
       <c r="K122" s="24">
         <f>COUNTIF($G$3:G122,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="123" spans="1:11" ht="20" customHeight="1">
@@ -6790,7 +6796,7 @@
       </c>
       <c r="K123" s="24">
         <f>COUNTIF($G$3:G123,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="124" spans="1:11" ht="20" customHeight="1">
@@ -6822,7 +6828,7 @@
       </c>
       <c r="K124" s="24">
         <f>COUNTIF($G$3:G124,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="125" spans="1:11" ht="20" customHeight="1">
@@ -6854,7 +6860,7 @@
       </c>
       <c r="K125" s="24">
         <f>COUNTIF($G$3:G125,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="126" spans="1:11" ht="20" customHeight="1">
@@ -6871,7 +6877,7 @@
       <c r="I126" s="1"/>
       <c r="K126" s="24">
         <f>COUNTIF($G$3:G126,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="127" spans="1:11" ht="20" customHeight="1">
@@ -6903,7 +6909,7 @@
       </c>
       <c r="K127" s="24">
         <f>COUNTIF($G$3:G127,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="128" spans="1:11" ht="20" customHeight="1">
@@ -6935,7 +6941,7 @@
       </c>
       <c r="K128" s="24">
         <f>COUNTIF($G$3:G128,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="129" spans="1:11" ht="20" customHeight="1">
@@ -6967,7 +6973,7 @@
       </c>
       <c r="K129" s="24">
         <f>COUNTIF($G$3:G129,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="130" spans="1:11" ht="20" customHeight="1">
@@ -6999,7 +7005,7 @@
       </c>
       <c r="K130" s="24">
         <f>COUNTIF($G$3:G130,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="131" spans="1:11" ht="20" customHeight="1">
@@ -7031,7 +7037,7 @@
       </c>
       <c r="K131" s="24">
         <f>COUNTIF($G$3:G131,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="132" spans="1:11" ht="20" customHeight="1">
@@ -7063,7 +7069,7 @@
       </c>
       <c r="K132" s="24">
         <f>COUNTIF($G$3:G132,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="133" spans="1:11" ht="20" customHeight="1">
@@ -7080,7 +7086,7 @@
       <c r="I133" s="1"/>
       <c r="K133" s="24">
         <f>COUNTIF($G$3:G133,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="134" spans="1:11" ht="20" customHeight="1">
@@ -7112,7 +7118,7 @@
       </c>
       <c r="K134" s="24">
         <f>COUNTIF($G$3:G134,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="135" spans="1:11" ht="20" customHeight="1">
@@ -7144,7 +7150,7 @@
       </c>
       <c r="K135" s="24">
         <f>COUNTIF($G$3:G135,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="136" spans="1:11" ht="20" customHeight="1">
@@ -7176,7 +7182,7 @@
       </c>
       <c r="K136" s="24">
         <f>COUNTIF($G$3:G136,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="137" spans="1:11" ht="20" customHeight="1">
@@ -7208,7 +7214,7 @@
       </c>
       <c r="K137" s="24">
         <f>COUNTIF($G$3:G137,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="138" spans="1:11" ht="20" customHeight="1">
@@ -7240,7 +7246,7 @@
       </c>
       <c r="K138" s="24">
         <f>COUNTIF($G$3:G138,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="139" spans="1:11" ht="20" customHeight="1">
@@ -7257,7 +7263,7 @@
       <c r="I139" s="1"/>
       <c r="K139" s="24">
         <f>COUNTIF($G$3:G139,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="140" spans="1:11" ht="20" customHeight="1">
@@ -7289,7 +7295,7 @@
       </c>
       <c r="K140" s="24">
         <f>COUNTIF($G$3:G140,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="141" spans="1:11" ht="20" customHeight="1">
@@ -7321,7 +7327,7 @@
       </c>
       <c r="K141" s="24">
         <f>COUNTIF($G$3:G141,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="142" spans="1:11" ht="20" customHeight="1">
@@ -7353,7 +7359,7 @@
       </c>
       <c r="K142" s="24">
         <f>COUNTIF($G$3:G142,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="143" spans="1:11" ht="20" customHeight="1">
@@ -7385,7 +7391,7 @@
       </c>
       <c r="K143" s="24">
         <f>COUNTIF($G$3:G143,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="144" spans="1:11" ht="20" customHeight="1">
@@ -7417,7 +7423,7 @@
       </c>
       <c r="K144" s="24">
         <f>COUNTIF($G$3:G144,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="145" spans="1:11" ht="20" customHeight="1">
@@ -7449,7 +7455,7 @@
       </c>
       <c r="K145" s="24">
         <f>COUNTIF($G$3:G145,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="146" spans="1:11" ht="20" customHeight="1">
@@ -7481,7 +7487,7 @@
       </c>
       <c r="K146" s="24">
         <f>COUNTIF($G$3:G146,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="147" spans="1:11" ht="20" customHeight="1">
@@ -7498,7 +7504,7 @@
       <c r="I147" s="1"/>
       <c r="K147" s="24">
         <f>COUNTIF($G$3:G147,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="148" spans="1:11" ht="20" customHeight="1">
@@ -7530,7 +7536,7 @@
       </c>
       <c r="K148" s="24">
         <f>COUNTIF($G$3:G148,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="149" spans="1:11" ht="20" customHeight="1">
@@ -7562,7 +7568,7 @@
       </c>
       <c r="K149" s="24">
         <f>COUNTIF($G$3:G149,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="150" spans="1:11" ht="20" customHeight="1">
@@ -7594,7 +7600,7 @@
       </c>
       <c r="K150" s="24">
         <f>COUNTIF($G$3:G150,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="151" spans="1:11" ht="20" customHeight="1">
@@ -7626,7 +7632,7 @@
       </c>
       <c r="K151" s="24">
         <f>COUNTIF($G$3:G151,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="152" spans="1:11" ht="20" customHeight="1">
@@ -7658,7 +7664,7 @@
       </c>
       <c r="K152" s="24">
         <f>COUNTIF($G$3:G152,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="153" spans="1:11" ht="20" customHeight="1">
@@ -7690,7 +7696,7 @@
       </c>
       <c r="K153" s="24">
         <f>COUNTIF($G$3:G153,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="154" spans="1:11" ht="20" customHeight="1">
@@ -7707,7 +7713,7 @@
       <c r="I154" s="1"/>
       <c r="K154" s="24">
         <f>COUNTIF($G$3:G154,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="155" spans="1:11" ht="20" customHeight="1">
@@ -7739,7 +7745,7 @@
       </c>
       <c r="K155" s="24">
         <f>COUNTIF($G$3:G155,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="156" spans="1:11" ht="20" customHeight="1">
@@ -7771,7 +7777,7 @@
       </c>
       <c r="K156" s="24">
         <f>COUNTIF($G$3:G156,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="157" spans="1:11" ht="20" customHeight="1">
@@ -7803,7 +7809,7 @@
       </c>
       <c r="K157" s="24">
         <f>COUNTIF($G$3:G157,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="158" spans="1:11" ht="20" customHeight="1">
@@ -7835,7 +7841,7 @@
       </c>
       <c r="K158" s="24">
         <f>COUNTIF($G$3:G158,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="159" spans="1:11" ht="20" customHeight="1">
@@ -7852,7 +7858,7 @@
       <c r="I159" s="1"/>
       <c r="K159" s="24">
         <f>COUNTIF($G$3:G159,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="160" spans="1:11" ht="20" customHeight="1">
@@ -7884,7 +7890,7 @@
       </c>
       <c r="K160" s="24">
         <f>COUNTIF($G$3:G160,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="161" spans="1:11" ht="20" customHeight="1">
@@ -7916,7 +7922,7 @@
       </c>
       <c r="K161" s="24">
         <f>COUNTIF($G$3:G161,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="162" spans="1:11" ht="20" customHeight="1">
@@ -7948,7 +7954,7 @@
       </c>
       <c r="K162" s="24">
         <f>COUNTIF($G$3:G162,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="163" spans="1:11" ht="20" customHeight="1">
@@ -7965,7 +7971,7 @@
       <c r="I163" s="1"/>
       <c r="K163" s="24">
         <f>COUNTIF($G$3:G163,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="164" spans="1:11" ht="20" customHeight="1">
@@ -7997,7 +8003,7 @@
       </c>
       <c r="K164" s="24">
         <f>COUNTIF($G$3:G164,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="165" spans="1:11" ht="20" customHeight="1">
@@ -8029,7 +8035,7 @@
       </c>
       <c r="K165" s="24">
         <f>COUNTIF($G$3:G165,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="166" spans="1:11" ht="20" customHeight="1">
@@ -8061,7 +8067,7 @@
       </c>
       <c r="K166" s="24">
         <f>COUNTIF($G$3:G166,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="167" spans="1:11" ht="20" customHeight="1">
@@ -8093,7 +8099,7 @@
       </c>
       <c r="K167" s="24">
         <f>COUNTIF($G$3:G167,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="168" spans="1:11" ht="20" customHeight="1">
@@ -8110,7 +8116,7 @@
       <c r="I168" s="1"/>
       <c r="K168" s="24">
         <f>COUNTIF($G$3:G168,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="169" spans="1:11" ht="20" customHeight="1">
@@ -8142,7 +8148,7 @@
       </c>
       <c r="K169" s="24">
         <f>COUNTIF($G$3:G169,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="170" spans="1:11" ht="20" customHeight="1">
@@ -8174,7 +8180,7 @@
       </c>
       <c r="K170" s="24">
         <f>COUNTIF($G$3:G170,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="171" spans="1:11" ht="20" customHeight="1">
@@ -8206,7 +8212,7 @@
       </c>
       <c r="K171" s="24">
         <f>COUNTIF($G$3:G171,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="172" spans="1:11" ht="20" customHeight="1">
@@ -8238,7 +8244,7 @@
       </c>
       <c r="K172" s="24">
         <f>COUNTIF($G$3:G172,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="173" spans="1:11" ht="20" customHeight="1">
@@ -8255,7 +8261,7 @@
       <c r="I173" s="1"/>
       <c r="K173" s="24">
         <f>COUNTIF($G$3:G173,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="174" spans="1:11" ht="20" customHeight="1">
@@ -8287,7 +8293,7 @@
       </c>
       <c r="K174" s="24">
         <f>COUNTIF($G$3:G174,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="175" spans="1:11" ht="20" customHeight="1">
@@ -8319,7 +8325,7 @@
       </c>
       <c r="K175" s="24">
         <f>COUNTIF($G$3:G175,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="176" spans="1:11" ht="20" customHeight="1">
@@ -8351,7 +8357,7 @@
       </c>
       <c r="K176" s="24">
         <f>COUNTIF($G$3:G176,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="177" spans="1:11" ht="20" customHeight="1">
@@ -8383,7 +8389,7 @@
       </c>
       <c r="K177" s="24">
         <f>COUNTIF($G$3:G177,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="178" spans="1:11" ht="20" customHeight="1">
@@ -8415,7 +8421,7 @@
       </c>
       <c r="K178" s="24">
         <f>COUNTIF($G$3:G178,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="179" spans="1:11" ht="20" customHeight="1">
@@ -8447,7 +8453,7 @@
       </c>
       <c r="K179" s="24">
         <f>COUNTIF($G$3:G179,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="180" spans="1:11" ht="20" customHeight="1">
@@ -8479,7 +8485,7 @@
       </c>
       <c r="K180" s="24">
         <f>COUNTIF($G$3:G180,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="181" spans="1:11" ht="20" customHeight="1">
@@ -8511,7 +8517,7 @@
       </c>
       <c r="K181" s="24">
         <f>COUNTIF($G$3:G181,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="182" spans="1:11" ht="20" customHeight="1">
@@ -8543,7 +8549,7 @@
       </c>
       <c r="K182" s="24">
         <f>COUNTIF($G$3:G182,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="183" spans="1:11" ht="20" customHeight="1">
@@ -8575,7 +8581,7 @@
       </c>
       <c r="K183" s="24">
         <f>COUNTIF($G$3:G183,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="184" spans="1:11" ht="20" customHeight="1">
@@ -8592,7 +8598,7 @@
       <c r="I184" s="1"/>
       <c r="K184" s="24">
         <f>COUNTIF($G$3:G184,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="185" spans="1:11" ht="20" customHeight="1">
@@ -8624,7 +8630,7 @@
       </c>
       <c r="K185" s="24">
         <f>COUNTIF($G$3:G185,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="186" spans="1:11" ht="20" customHeight="1">
@@ -8656,7 +8662,7 @@
       </c>
       <c r="K186" s="24">
         <f>COUNTIF($G$3:G186,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="187" spans="1:11" ht="20" customHeight="1">
@@ -8688,7 +8694,7 @@
       </c>
       <c r="K187" s="24">
         <f>COUNTIF($G$3:G187,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="188" spans="1:11" ht="20" customHeight="1">
@@ -8720,7 +8726,7 @@
       </c>
       <c r="K188" s="24">
         <f>COUNTIF($G$3:G188,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="189" spans="1:11" ht="20" customHeight="1">
@@ -8752,7 +8758,7 @@
       </c>
       <c r="K189" s="24">
         <f>COUNTIF($G$3:G189,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="190" spans="1:11" ht="20" customHeight="1">
@@ -8784,7 +8790,7 @@
       </c>
       <c r="K190" s="24">
         <f>COUNTIF($G$3:G190,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="191" spans="1:11" ht="20" customHeight="1">
@@ -8816,7 +8822,7 @@
       </c>
       <c r="K191" s="24">
         <f>COUNTIF($G$3:G191,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="192" spans="1:11" ht="20" customHeight="1">
@@ -8848,7 +8854,7 @@
       </c>
       <c r="K192" s="24">
         <f>COUNTIF($G$3:G192,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="193" spans="1:11" ht="20" customHeight="1">
@@ -8880,7 +8886,7 @@
       </c>
       <c r="K193" s="24">
         <f>COUNTIF($G$3:G193,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="194" spans="1:11" ht="20" customHeight="1">
@@ -8912,7 +8918,7 @@
       </c>
       <c r="K194" s="24">
         <f>COUNTIF($G$3:G194,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="195" spans="1:11" ht="20" customHeight="1">
@@ -8944,7 +8950,7 @@
       </c>
       <c r="K195" s="24">
         <f>COUNTIF($G$3:G195,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="196" spans="1:11" ht="20" customHeight="1">
@@ -8976,7 +8982,7 @@
       </c>
       <c r="K196" s="24">
         <f>COUNTIF($G$3:G196,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="197" spans="1:11" ht="20" customHeight="1">
@@ -8993,7 +8999,7 @@
       <c r="I197" s="1"/>
       <c r="K197" s="24">
         <f>COUNTIF($G$3:G197,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="198" spans="1:11" ht="20" customHeight="1">
@@ -9025,7 +9031,7 @@
       </c>
       <c r="K198" s="24">
         <f>COUNTIF($G$3:G198,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="199" spans="1:11" ht="20" customHeight="1">
@@ -9057,7 +9063,7 @@
       </c>
       <c r="K199" s="24">
         <f>COUNTIF($G$3:G199,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="200" spans="1:11" ht="20" customHeight="1">
@@ -9089,7 +9095,7 @@
       </c>
       <c r="K200" s="24">
         <f>COUNTIF($G$3:G200,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="201" spans="1:11" ht="20" customHeight="1">
@@ -9121,7 +9127,7 @@
       </c>
       <c r="K201" s="24">
         <f>COUNTIF($G$3:G201,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="202" spans="1:11" ht="20" customHeight="1">
@@ -9153,7 +9159,7 @@
       </c>
       <c r="K202" s="24">
         <f>COUNTIF($G$3:G202,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="203" spans="1:11" ht="20" customHeight="1">
@@ -9185,7 +9191,7 @@
       </c>
       <c r="K203" s="24">
         <f>COUNTIF($G$3:G203,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="204" spans="1:11" ht="20" customHeight="1">
@@ -9217,7 +9223,7 @@
       </c>
       <c r="K204" s="24">
         <f>COUNTIF($G$3:G204,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="205" spans="1:11" ht="20" customHeight="1">
@@ -9234,7 +9240,7 @@
       <c r="I205" s="1"/>
       <c r="K205" s="24">
         <f>COUNTIF($G$3:G205,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="206" spans="1:11" ht="20" customHeight="1">
@@ -9266,7 +9272,7 @@
       </c>
       <c r="K206" s="24">
         <f>COUNTIF($G$3:G206,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="207" spans="1:11" ht="20" customHeight="1">
@@ -9298,7 +9304,7 @@
       </c>
       <c r="K207" s="24">
         <f>COUNTIF($G$3:G207,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="208" spans="1:11" ht="20" customHeight="1">
@@ -9330,7 +9336,7 @@
       </c>
       <c r="K208" s="24">
         <f>COUNTIF($G$3:G208,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="209" spans="1:11" ht="20" customHeight="1">
@@ -9362,7 +9368,7 @@
       </c>
       <c r="K209" s="24">
         <f>COUNTIF($G$3:G209,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="210" spans="1:11" ht="20" customHeight="1">
@@ -9394,7 +9400,7 @@
       </c>
       <c r="K210" s="24">
         <f>COUNTIF($G$3:G210,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="211" spans="1:11" ht="20" customHeight="1">
@@ -9411,7 +9417,7 @@
       <c r="I211" s="1"/>
       <c r="K211" s="24">
         <f>COUNTIF($G$3:G211,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="212" spans="1:11" ht="20" customHeight="1">
@@ -9443,7 +9449,7 @@
       </c>
       <c r="K212" s="24">
         <f>COUNTIF($G$3:G212,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="213" spans="1:11" ht="20" customHeight="1">
@@ -9475,7 +9481,7 @@
       </c>
       <c r="K213" s="24">
         <f>COUNTIF($G$3:G213,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="214" spans="1:11" ht="20" customHeight="1">
@@ -9507,7 +9513,7 @@
       </c>
       <c r="K214" s="24">
         <f>COUNTIF($G$3:G214,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="215" spans="1:11" ht="20" customHeight="1">
@@ -9539,7 +9545,7 @@
       </c>
       <c r="K215" s="24">
         <f>COUNTIF($G$3:G215,"Done")</f>
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: JS fundamentals uploaded on 261009
</commit_message>
<xml_diff>
--- a/side-project/Scrimba全栈学习路径进度追踪表.xlsx
+++ b/side-project/Scrimba全栈学习路径进度追踪表.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ersheng/Desktop/web_project/public-note/side-project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F32077F-9EB0-7F47-B1C0-B2DF8B1A4B80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CB4AAD2-1301-7A4D-B4F4-DBA4F2814CDA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10240" yWindow="3820" windowWidth="40960" windowHeight="23360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="8160" yWindow="3980" windowWidth="40960" windowHeight="23360" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="学习进度追踪" sheetId="1" r:id="rId1"/>
@@ -64,7 +64,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="973" uniqueCount="461">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="978" uniqueCount="466">
   <si>
     <t>Introduction</t>
   </si>
@@ -1932,9 +1932,6 @@
     <t>命令行使用学习路径</t>
   </si>
   <si>
-    <t>每天进行15分钟左右的实操，走gitByBit路线</t>
-  </si>
-  <si>
     <t>Git命令实操每日练习</t>
   </si>
   <si>
@@ -1996,6 +1993,24 @@
   </si>
   <si>
     <t>Scrimba Docs</t>
+  </si>
+  <si>
+    <t>内容</t>
+  </si>
+  <si>
+    <t>日期</t>
+  </si>
+  <si>
+    <t>Git remote</t>
+  </si>
+  <si>
+    <t>2026年10月06日</t>
+  </si>
+  <si>
+    <t>下一步</t>
+  </si>
+  <si>
+    <t>测试题</t>
   </si>
 </sst>
 </file>
@@ -2267,7 +2282,7 @@
     <xf numFmtId="9" fontId="9" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -2331,9 +2346,6 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -2830,7 +2842,7 @@
         <v>419</v>
       </c>
       <c r="J1" s="20" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="K1" s="22"/>
       <c r="L1" s="23"/>
@@ -3607,7 +3619,7 @@
         <v>46289</v>
       </c>
       <c r="I28" s="3" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="J28" s="21">
         <f t="shared" si="3"/>
@@ -3681,7 +3693,7 @@
         <v>46289</v>
       </c>
       <c r="I30" s="3" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="J30" s="21">
         <f t="shared" si="3"/>
@@ -5350,23 +5362,23 @@
     </row>
     <row r="77" spans="1:11" ht="20" customHeight="1">
       <c r="A77" s="2" t="s">
+        <v>443</v>
+      </c>
+      <c r="B77" s="3" t="s">
         <v>444</v>
       </c>
-      <c r="B77" s="3" t="s">
+      <c r="C77" s="3" t="s">
         <v>445</v>
-      </c>
-      <c r="C77" s="3" t="s">
-        <v>446</v>
       </c>
       <c r="D77" s="3"/>
       <c r="E77" s="2"/>
       <c r="F77" s="4"/>
       <c r="G77" s="5"/>
       <c r="H77" s="6" t="s">
+        <v>446</v>
+      </c>
+      <c r="I77" s="3" t="s">
         <v>447</v>
-      </c>
-      <c r="I77" s="3" t="s">
-        <v>448</v>
       </c>
       <c r="J77" s="21"/>
       <c r="K77" s="24"/>
@@ -5398,7 +5410,7 @@
         <v>46296</v>
       </c>
       <c r="I78" s="8" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="J78" s="21">
         <f t="shared" si="3"/>
@@ -5583,17 +5595,19 @@
       </c>
       <c r="G84" s="5" t="str">
         <f t="shared" si="5"/>
-        <v>Pending</v>
-      </c>
-      <c r="H84" s="6"/>
+        <v>Done</v>
+      </c>
+      <c r="H84" s="6">
+        <v>46301</v>
+      </c>
       <c r="I84" s="3"/>
-      <c r="J84" s="21" t="str">
+      <c r="J84" s="21">
         <f t="shared" si="3"/>
-        <v/>
+        <v>0.40512820512820513</v>
       </c>
       <c r="K84" s="24">
         <f>COUNTIF($G$3:G84,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="85" spans="1:11" ht="20" customHeight="1">
@@ -5625,7 +5639,7 @@
       </c>
       <c r="K85" s="24">
         <f>COUNTIF($G$3:G85,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="86" spans="1:11" ht="20" customHeight="1">
@@ -5657,7 +5671,7 @@
       </c>
       <c r="K86" s="24">
         <f>COUNTIF($G$3:G86,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="87" spans="1:11" ht="20" customHeight="1">
@@ -5689,7 +5703,7 @@
       </c>
       <c r="K87" s="24">
         <f>COUNTIF($G$3:G87,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="88" spans="1:11" ht="20" customHeight="1">
@@ -5721,7 +5735,7 @@
       </c>
       <c r="K88" s="24">
         <f>COUNTIF($G$3:G88,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="89" spans="1:11" ht="20" customHeight="1">
@@ -5738,7 +5752,7 @@
       <c r="I89" s="1"/>
       <c r="K89" s="24">
         <f>COUNTIF($G$3:G89,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="90" spans="1:11" ht="20" customHeight="1">
@@ -5770,7 +5784,7 @@
       </c>
       <c r="K90" s="24">
         <f>COUNTIF($G$3:G90,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="91" spans="1:11" ht="20" customHeight="1">
@@ -5802,7 +5816,7 @@
       </c>
       <c r="K91" s="24">
         <f>COUNTIF($G$3:G91,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="92" spans="1:11" ht="20" customHeight="1">
@@ -5834,7 +5848,7 @@
       </c>
       <c r="K92" s="24">
         <f>COUNTIF($G$3:G92,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="93" spans="1:11" ht="20" customHeight="1">
@@ -5866,7 +5880,7 @@
       </c>
       <c r="K93" s="24">
         <f>COUNTIF($G$3:G93,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="94" spans="1:11" ht="20" customHeight="1">
@@ -5883,7 +5897,7 @@
       <c r="I94" s="1"/>
       <c r="K94" s="24">
         <f>COUNTIF($G$3:G94,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="95" spans="1:11" ht="20" customHeight="1">
@@ -5915,7 +5929,7 @@
       </c>
       <c r="K95" s="24">
         <f>COUNTIF($G$3:G95,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="96" spans="1:11" ht="20" customHeight="1">
@@ -5947,7 +5961,7 @@
       </c>
       <c r="K96" s="24">
         <f>COUNTIF($G$3:G96,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="97" spans="1:11" ht="20" customHeight="1">
@@ -5979,7 +5993,7 @@
       </c>
       <c r="K97" s="24">
         <f>COUNTIF($G$3:G97,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="98" spans="1:11" ht="20" customHeight="1">
@@ -6011,7 +6025,7 @@
       </c>
       <c r="K98" s="24">
         <f>COUNTIF($G$3:G98,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="99" spans="1:11" ht="20" customHeight="1">
@@ -6043,7 +6057,7 @@
       </c>
       <c r="K99" s="24">
         <f>COUNTIF($G$3:G99,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="100" spans="1:11" ht="20" customHeight="1">
@@ -6075,7 +6089,7 @@
       </c>
       <c r="K100" s="24">
         <f>COUNTIF($G$3:G100,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="101" spans="1:11" ht="20" customHeight="1">
@@ -6107,7 +6121,7 @@
       </c>
       <c r="K101" s="24">
         <f>COUNTIF($G$3:G101,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="102" spans="1:11" ht="20" customHeight="1">
@@ -6139,7 +6153,7 @@
       </c>
       <c r="K102" s="24">
         <f>COUNTIF($G$3:G102,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="103" spans="1:11" ht="20" customHeight="1">
@@ -6171,7 +6185,7 @@
       </c>
       <c r="K103" s="24">
         <f>COUNTIF($G$3:G103,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="104" spans="1:11" ht="20" customHeight="1">
@@ -6203,7 +6217,7 @@
       </c>
       <c r="K104" s="24">
         <f>COUNTIF($G$3:G104,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="105" spans="1:11" ht="20" customHeight="1">
@@ -6235,7 +6249,7 @@
       </c>
       <c r="K105" s="24">
         <f>COUNTIF($G$3:G105,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="106" spans="1:11" ht="20" customHeight="1">
@@ -6267,7 +6281,7 @@
       </c>
       <c r="K106" s="24">
         <f>COUNTIF($G$3:G106,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="107" spans="1:11" ht="20" customHeight="1">
@@ -6299,7 +6313,7 @@
       </c>
       <c r="K107" s="24">
         <f>COUNTIF($G$3:G107,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="108" spans="1:11" ht="20" customHeight="1">
@@ -6331,7 +6345,7 @@
       </c>
       <c r="K108" s="24">
         <f>COUNTIF($G$3:G108,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="109" spans="1:11" ht="20" customHeight="1">
@@ -6363,7 +6377,7 @@
       </c>
       <c r="K109" s="24">
         <f>COUNTIF($G$3:G109,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="110" spans="1:11" ht="20" customHeight="1">
@@ -6395,7 +6409,7 @@
       </c>
       <c r="K110" s="24">
         <f>COUNTIF($G$3:G110,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="111" spans="1:11" ht="20" customHeight="1">
@@ -6427,7 +6441,7 @@
       </c>
       <c r="K111" s="24">
         <f>COUNTIF($G$3:G111,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="112" spans="1:11" ht="20" customHeight="1">
@@ -6459,7 +6473,7 @@
       </c>
       <c r="K112" s="24">
         <f>COUNTIF($G$3:G112,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="113" spans="1:11" ht="20" customHeight="1">
@@ -6491,7 +6505,7 @@
       </c>
       <c r="K113" s="24">
         <f>COUNTIF($G$3:G113,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="114" spans="1:11" ht="20" customHeight="1">
@@ -6523,7 +6537,7 @@
       </c>
       <c r="K114" s="24">
         <f>COUNTIF($G$3:G114,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="115" spans="1:11" ht="20" customHeight="1">
@@ -6555,7 +6569,7 @@
       </c>
       <c r="K115" s="24">
         <f>COUNTIF($G$3:G115,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="116" spans="1:11" ht="20" customHeight="1">
@@ -6587,7 +6601,7 @@
       </c>
       <c r="K116" s="24">
         <f>COUNTIF($G$3:G116,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="117" spans="1:11" ht="20" customHeight="1">
@@ -6619,7 +6633,7 @@
       </c>
       <c r="K117" s="24">
         <f>COUNTIF($G$3:G117,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="118" spans="1:11" ht="20" customHeight="1">
@@ -6651,7 +6665,7 @@
       </c>
       <c r="K118" s="24">
         <f>COUNTIF($G$3:G118,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="119" spans="1:11" ht="20" customHeight="1">
@@ -6683,7 +6697,7 @@
       </c>
       <c r="K119" s="24">
         <f>COUNTIF($G$3:G119,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="120" spans="1:11" ht="20" customHeight="1">
@@ -6700,7 +6714,7 @@
       <c r="I120" s="1"/>
       <c r="K120" s="24">
         <f>COUNTIF($G$3:G120,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="121" spans="1:11" ht="20" customHeight="1">
@@ -6732,7 +6746,7 @@
       </c>
       <c r="K121" s="24">
         <f>COUNTIF($G$3:G121,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="122" spans="1:11" ht="20" customHeight="1">
@@ -6764,7 +6778,7 @@
       </c>
       <c r="K122" s="24">
         <f>COUNTIF($G$3:G122,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="123" spans="1:11" ht="20" customHeight="1">
@@ -6796,7 +6810,7 @@
       </c>
       <c r="K123" s="24">
         <f>COUNTIF($G$3:G123,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="124" spans="1:11" ht="20" customHeight="1">
@@ -6828,7 +6842,7 @@
       </c>
       <c r="K124" s="24">
         <f>COUNTIF($G$3:G124,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="125" spans="1:11" ht="20" customHeight="1">
@@ -6860,7 +6874,7 @@
       </c>
       <c r="K125" s="24">
         <f>COUNTIF($G$3:G125,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="126" spans="1:11" ht="20" customHeight="1">
@@ -6877,7 +6891,7 @@
       <c r="I126" s="1"/>
       <c r="K126" s="24">
         <f>COUNTIF($G$3:G126,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="127" spans="1:11" ht="20" customHeight="1">
@@ -6909,7 +6923,7 @@
       </c>
       <c r="K127" s="24">
         <f>COUNTIF($G$3:G127,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="128" spans="1:11" ht="20" customHeight="1">
@@ -6941,7 +6955,7 @@
       </c>
       <c r="K128" s="24">
         <f>COUNTIF($G$3:G128,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="129" spans="1:11" ht="20" customHeight="1">
@@ -6973,7 +6987,7 @@
       </c>
       <c r="K129" s="24">
         <f>COUNTIF($G$3:G129,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="130" spans="1:11" ht="20" customHeight="1">
@@ -7005,7 +7019,7 @@
       </c>
       <c r="K130" s="24">
         <f>COUNTIF($G$3:G130,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="131" spans="1:11" ht="20" customHeight="1">
@@ -7037,7 +7051,7 @@
       </c>
       <c r="K131" s="24">
         <f>COUNTIF($G$3:G131,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="132" spans="1:11" ht="20" customHeight="1">
@@ -7069,7 +7083,7 @@
       </c>
       <c r="K132" s="24">
         <f>COUNTIF($G$3:G132,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="133" spans="1:11" ht="20" customHeight="1">
@@ -7086,7 +7100,7 @@
       <c r="I133" s="1"/>
       <c r="K133" s="24">
         <f>COUNTIF($G$3:G133,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="134" spans="1:11" ht="20" customHeight="1">
@@ -7118,7 +7132,7 @@
       </c>
       <c r="K134" s="24">
         <f>COUNTIF($G$3:G134,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="135" spans="1:11" ht="20" customHeight="1">
@@ -7150,7 +7164,7 @@
       </c>
       <c r="K135" s="24">
         <f>COUNTIF($G$3:G135,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="136" spans="1:11" ht="20" customHeight="1">
@@ -7182,7 +7196,7 @@
       </c>
       <c r="K136" s="24">
         <f>COUNTIF($G$3:G136,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="137" spans="1:11" ht="20" customHeight="1">
@@ -7214,7 +7228,7 @@
       </c>
       <c r="K137" s="24">
         <f>COUNTIF($G$3:G137,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="138" spans="1:11" ht="20" customHeight="1">
@@ -7246,7 +7260,7 @@
       </c>
       <c r="K138" s="24">
         <f>COUNTIF($G$3:G138,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="139" spans="1:11" ht="20" customHeight="1">
@@ -7263,7 +7277,7 @@
       <c r="I139" s="1"/>
       <c r="K139" s="24">
         <f>COUNTIF($G$3:G139,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="140" spans="1:11" ht="20" customHeight="1">
@@ -7295,7 +7309,7 @@
       </c>
       <c r="K140" s="24">
         <f>COUNTIF($G$3:G140,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="141" spans="1:11" ht="20" customHeight="1">
@@ -7327,7 +7341,7 @@
       </c>
       <c r="K141" s="24">
         <f>COUNTIF($G$3:G141,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="142" spans="1:11" ht="20" customHeight="1">
@@ -7359,7 +7373,7 @@
       </c>
       <c r="K142" s="24">
         <f>COUNTIF($G$3:G142,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="143" spans="1:11" ht="20" customHeight="1">
@@ -7391,7 +7405,7 @@
       </c>
       <c r="K143" s="24">
         <f>COUNTIF($G$3:G143,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="144" spans="1:11" ht="20" customHeight="1">
@@ -7423,7 +7437,7 @@
       </c>
       <c r="K144" s="24">
         <f>COUNTIF($G$3:G144,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="145" spans="1:11" ht="20" customHeight="1">
@@ -7455,7 +7469,7 @@
       </c>
       <c r="K145" s="24">
         <f>COUNTIF($G$3:G145,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="146" spans="1:11" ht="20" customHeight="1">
@@ -7487,7 +7501,7 @@
       </c>
       <c r="K146" s="24">
         <f>COUNTIF($G$3:G146,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="147" spans="1:11" ht="20" customHeight="1">
@@ -7504,7 +7518,7 @@
       <c r="I147" s="1"/>
       <c r="K147" s="24">
         <f>COUNTIF($G$3:G147,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="148" spans="1:11" ht="20" customHeight="1">
@@ -7536,7 +7550,7 @@
       </c>
       <c r="K148" s="24">
         <f>COUNTIF($G$3:G148,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="149" spans="1:11" ht="20" customHeight="1">
@@ -7568,7 +7582,7 @@
       </c>
       <c r="K149" s="24">
         <f>COUNTIF($G$3:G149,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="150" spans="1:11" ht="20" customHeight="1">
@@ -7600,7 +7614,7 @@
       </c>
       <c r="K150" s="24">
         <f>COUNTIF($G$3:G150,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="151" spans="1:11" ht="20" customHeight="1">
@@ -7632,7 +7646,7 @@
       </c>
       <c r="K151" s="24">
         <f>COUNTIF($G$3:G151,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="152" spans="1:11" ht="20" customHeight="1">
@@ -7664,7 +7678,7 @@
       </c>
       <c r="K152" s="24">
         <f>COUNTIF($G$3:G152,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="153" spans="1:11" ht="20" customHeight="1">
@@ -7696,7 +7710,7 @@
       </c>
       <c r="K153" s="24">
         <f>COUNTIF($G$3:G153,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="154" spans="1:11" ht="20" customHeight="1">
@@ -7713,7 +7727,7 @@
       <c r="I154" s="1"/>
       <c r="K154" s="24">
         <f>COUNTIF($G$3:G154,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="155" spans="1:11" ht="20" customHeight="1">
@@ -7745,7 +7759,7 @@
       </c>
       <c r="K155" s="24">
         <f>COUNTIF($G$3:G155,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="156" spans="1:11" ht="20" customHeight="1">
@@ -7777,7 +7791,7 @@
       </c>
       <c r="K156" s="24">
         <f>COUNTIF($G$3:G156,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="157" spans="1:11" ht="20" customHeight="1">
@@ -7809,7 +7823,7 @@
       </c>
       <c r="K157" s="24">
         <f>COUNTIF($G$3:G157,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="158" spans="1:11" ht="20" customHeight="1">
@@ -7841,7 +7855,7 @@
       </c>
       <c r="K158" s="24">
         <f>COUNTIF($G$3:G158,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="159" spans="1:11" ht="20" customHeight="1">
@@ -7858,7 +7872,7 @@
       <c r="I159" s="1"/>
       <c r="K159" s="24">
         <f>COUNTIF($G$3:G159,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="160" spans="1:11" ht="20" customHeight="1">
@@ -7890,7 +7904,7 @@
       </c>
       <c r="K160" s="24">
         <f>COUNTIF($G$3:G160,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="161" spans="1:11" ht="20" customHeight="1">
@@ -7922,7 +7936,7 @@
       </c>
       <c r="K161" s="24">
         <f>COUNTIF($G$3:G161,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="162" spans="1:11" ht="20" customHeight="1">
@@ -7954,7 +7968,7 @@
       </c>
       <c r="K162" s="24">
         <f>COUNTIF($G$3:G162,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="163" spans="1:11" ht="20" customHeight="1">
@@ -7971,7 +7985,7 @@
       <c r="I163" s="1"/>
       <c r="K163" s="24">
         <f>COUNTIF($G$3:G163,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="164" spans="1:11" ht="20" customHeight="1">
@@ -8003,7 +8017,7 @@
       </c>
       <c r="K164" s="24">
         <f>COUNTIF($G$3:G164,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="165" spans="1:11" ht="20" customHeight="1">
@@ -8035,7 +8049,7 @@
       </c>
       <c r="K165" s="24">
         <f>COUNTIF($G$3:G165,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="166" spans="1:11" ht="20" customHeight="1">
@@ -8067,7 +8081,7 @@
       </c>
       <c r="K166" s="24">
         <f>COUNTIF($G$3:G166,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="167" spans="1:11" ht="20" customHeight="1">
@@ -8099,7 +8113,7 @@
       </c>
       <c r="K167" s="24">
         <f>COUNTIF($G$3:G167,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="168" spans="1:11" ht="20" customHeight="1">
@@ -8116,7 +8130,7 @@
       <c r="I168" s="1"/>
       <c r="K168" s="24">
         <f>COUNTIF($G$3:G168,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="169" spans="1:11" ht="20" customHeight="1">
@@ -8148,7 +8162,7 @@
       </c>
       <c r="K169" s="24">
         <f>COUNTIF($G$3:G169,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="170" spans="1:11" ht="20" customHeight="1">
@@ -8180,7 +8194,7 @@
       </c>
       <c r="K170" s="24">
         <f>COUNTIF($G$3:G170,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="171" spans="1:11" ht="20" customHeight="1">
@@ -8212,7 +8226,7 @@
       </c>
       <c r="K171" s="24">
         <f>COUNTIF($G$3:G171,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="172" spans="1:11" ht="20" customHeight="1">
@@ -8244,7 +8258,7 @@
       </c>
       <c r="K172" s="24">
         <f>COUNTIF($G$3:G172,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="173" spans="1:11" ht="20" customHeight="1">
@@ -8261,7 +8275,7 @@
       <c r="I173" s="1"/>
       <c r="K173" s="24">
         <f>COUNTIF($G$3:G173,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="174" spans="1:11" ht="20" customHeight="1">
@@ -8293,7 +8307,7 @@
       </c>
       <c r="K174" s="24">
         <f>COUNTIF($G$3:G174,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="175" spans="1:11" ht="20" customHeight="1">
@@ -8325,7 +8339,7 @@
       </c>
       <c r="K175" s="24">
         <f>COUNTIF($G$3:G175,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="176" spans="1:11" ht="20" customHeight="1">
@@ -8357,7 +8371,7 @@
       </c>
       <c r="K176" s="24">
         <f>COUNTIF($G$3:G176,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="177" spans="1:11" ht="20" customHeight="1">
@@ -8389,7 +8403,7 @@
       </c>
       <c r="K177" s="24">
         <f>COUNTIF($G$3:G177,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="178" spans="1:11" ht="20" customHeight="1">
@@ -8421,7 +8435,7 @@
       </c>
       <c r="K178" s="24">
         <f>COUNTIF($G$3:G178,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="179" spans="1:11" ht="20" customHeight="1">
@@ -8453,7 +8467,7 @@
       </c>
       <c r="K179" s="24">
         <f>COUNTIF($G$3:G179,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="180" spans="1:11" ht="20" customHeight="1">
@@ -8485,7 +8499,7 @@
       </c>
       <c r="K180" s="24">
         <f>COUNTIF($G$3:G180,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="181" spans="1:11" ht="20" customHeight="1">
@@ -8517,7 +8531,7 @@
       </c>
       <c r="K181" s="24">
         <f>COUNTIF($G$3:G181,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="182" spans="1:11" ht="20" customHeight="1">
@@ -8549,7 +8563,7 @@
       </c>
       <c r="K182" s="24">
         <f>COUNTIF($G$3:G182,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="183" spans="1:11" ht="20" customHeight="1">
@@ -8581,7 +8595,7 @@
       </c>
       <c r="K183" s="24">
         <f>COUNTIF($G$3:G183,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="184" spans="1:11" ht="20" customHeight="1">
@@ -8598,7 +8612,7 @@
       <c r="I184" s="1"/>
       <c r="K184" s="24">
         <f>COUNTIF($G$3:G184,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="185" spans="1:11" ht="20" customHeight="1">
@@ -8630,7 +8644,7 @@
       </c>
       <c r="K185" s="24">
         <f>COUNTIF($G$3:G185,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="186" spans="1:11" ht="20" customHeight="1">
@@ -8662,7 +8676,7 @@
       </c>
       <c r="K186" s="24">
         <f>COUNTIF($G$3:G186,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="187" spans="1:11" ht="20" customHeight="1">
@@ -8694,7 +8708,7 @@
       </c>
       <c r="K187" s="24">
         <f>COUNTIF($G$3:G187,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="188" spans="1:11" ht="20" customHeight="1">
@@ -8726,7 +8740,7 @@
       </c>
       <c r="K188" s="24">
         <f>COUNTIF($G$3:G188,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="189" spans="1:11" ht="20" customHeight="1">
@@ -8758,7 +8772,7 @@
       </c>
       <c r="K189" s="24">
         <f>COUNTIF($G$3:G189,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="190" spans="1:11" ht="20" customHeight="1">
@@ -8790,7 +8804,7 @@
       </c>
       <c r="K190" s="24">
         <f>COUNTIF($G$3:G190,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="191" spans="1:11" ht="20" customHeight="1">
@@ -8822,7 +8836,7 @@
       </c>
       <c r="K191" s="24">
         <f>COUNTIF($G$3:G191,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="192" spans="1:11" ht="20" customHeight="1">
@@ -8854,7 +8868,7 @@
       </c>
       <c r="K192" s="24">
         <f>COUNTIF($G$3:G192,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="193" spans="1:11" ht="20" customHeight="1">
@@ -8886,7 +8900,7 @@
       </c>
       <c r="K193" s="24">
         <f>COUNTIF($G$3:G193,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="194" spans="1:11" ht="20" customHeight="1">
@@ -8918,7 +8932,7 @@
       </c>
       <c r="K194" s="24">
         <f>COUNTIF($G$3:G194,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="195" spans="1:11" ht="20" customHeight="1">
@@ -8950,7 +8964,7 @@
       </c>
       <c r="K195" s="24">
         <f>COUNTIF($G$3:G195,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="196" spans="1:11" ht="20" customHeight="1">
@@ -8982,7 +8996,7 @@
       </c>
       <c r="K196" s="24">
         <f>COUNTIF($G$3:G196,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="197" spans="1:11" ht="20" customHeight="1">
@@ -8999,7 +9013,7 @@
       <c r="I197" s="1"/>
       <c r="K197" s="24">
         <f>COUNTIF($G$3:G197,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="198" spans="1:11" ht="20" customHeight="1">
@@ -9031,7 +9045,7 @@
       </c>
       <c r="K198" s="24">
         <f>COUNTIF($G$3:G198,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="199" spans="1:11" ht="20" customHeight="1">
@@ -9063,7 +9077,7 @@
       </c>
       <c r="K199" s="24">
         <f>COUNTIF($G$3:G199,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="200" spans="1:11" ht="20" customHeight="1">
@@ -9095,7 +9109,7 @@
       </c>
       <c r="K200" s="24">
         <f>COUNTIF($G$3:G200,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="201" spans="1:11" ht="20" customHeight="1">
@@ -9127,7 +9141,7 @@
       </c>
       <c r="K201" s="24">
         <f>COUNTIF($G$3:G201,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="202" spans="1:11" ht="20" customHeight="1">
@@ -9159,7 +9173,7 @@
       </c>
       <c r="K202" s="24">
         <f>COUNTIF($G$3:G202,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="203" spans="1:11" ht="20" customHeight="1">
@@ -9191,7 +9205,7 @@
       </c>
       <c r="K203" s="24">
         <f>COUNTIF($G$3:G203,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="204" spans="1:11" ht="20" customHeight="1">
@@ -9223,7 +9237,7 @@
       </c>
       <c r="K204" s="24">
         <f>COUNTIF($G$3:G204,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="205" spans="1:11" ht="20" customHeight="1">
@@ -9240,7 +9254,7 @@
       <c r="I205" s="1"/>
       <c r="K205" s="24">
         <f>COUNTIF($G$3:G205,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="206" spans="1:11" ht="20" customHeight="1">
@@ -9272,7 +9286,7 @@
       </c>
       <c r="K206" s="24">
         <f>COUNTIF($G$3:G206,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="207" spans="1:11" ht="20" customHeight="1">
@@ -9304,7 +9318,7 @@
       </c>
       <c r="K207" s="24">
         <f>COUNTIF($G$3:G207,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="208" spans="1:11" ht="20" customHeight="1">
@@ -9336,7 +9350,7 @@
       </c>
       <c r="K208" s="24">
         <f>COUNTIF($G$3:G208,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="209" spans="1:11" ht="20" customHeight="1">
@@ -9368,7 +9382,7 @@
       </c>
       <c r="K209" s="24">
         <f>COUNTIF($G$3:G209,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="210" spans="1:11" ht="20" customHeight="1">
@@ -9400,7 +9414,7 @@
       </c>
       <c r="K210" s="24">
         <f>COUNTIF($G$3:G210,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="211" spans="1:11" ht="20" customHeight="1">
@@ -9417,7 +9431,7 @@
       <c r="I211" s="1"/>
       <c r="K211" s="24">
         <f>COUNTIF($G$3:G211,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="212" spans="1:11" ht="20" customHeight="1">
@@ -9449,7 +9463,7 @@
       </c>
       <c r="K212" s="24">
         <f>COUNTIF($G$3:G212,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="213" spans="1:11" ht="20" customHeight="1">
@@ -9481,7 +9495,7 @@
       </c>
       <c r="K213" s="24">
         <f>COUNTIF($G$3:G213,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="214" spans="1:11" ht="20" customHeight="1">
@@ -9513,7 +9527,7 @@
       </c>
       <c r="K214" s="24">
         <f>COUNTIF($G$3:G214,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="215" spans="1:11" ht="20" customHeight="1">
@@ -9545,7 +9559,7 @@
       </c>
       <c r="K215" s="24">
         <f>COUNTIF($G$3:G215,"Done")</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
   </sheetData>
@@ -9601,12 +9615,13 @@
     <col min="6" max="6" width="20.83203125" customWidth="1"/>
     <col min="7" max="7" width="27.5" customWidth="1"/>
     <col min="8" max="8" width="87.5" style="15" customWidth="1"/>
-    <col min="11" max="11" width="41.6640625" customWidth="1"/>
+    <col min="11" max="11" width="15.5" customWidth="1"/>
     <col min="12" max="12" width="23.1640625" customWidth="1"/>
-    <col min="14" max="14" width="27.5" style="35" customWidth="1"/>
+    <col min="13" max="13" width="15.5" customWidth="1"/>
+    <col min="14" max="14" width="27.5" style="34" customWidth="1"/>
     <col min="15" max="15" width="21.83203125" style="27" customWidth="1"/>
     <col min="16" max="16" width="13.5" style="27" customWidth="1"/>
-    <col min="17" max="17" width="11.83203125" style="37" customWidth="1"/>
+    <col min="17" max="17" width="11.83203125" style="36" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="28" customHeight="1">
@@ -9620,11 +9635,11 @@
       <c r="G1" s="26"/>
       <c r="H1" s="26"/>
       <c r="K1" s="26" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="L1" s="26"/>
       <c r="N1" s="26" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="O1" s="26"/>
       <c r="Q1" s="27"/>
@@ -9643,24 +9658,29 @@
       <c r="H2" s="16" t="s">
         <v>425</v>
       </c>
-      <c r="K2" s="28" t="s">
-        <v>439</v>
-      </c>
-      <c r="L2" s="28"/>
-      <c r="N2" s="29" t="s">
+      <c r="K2" s="12" t="s">
+        <v>460</v>
+      </c>
+      <c r="L2" s="12" t="s">
+        <v>461</v>
+      </c>
+      <c r="M2" t="s">
+        <v>464</v>
+      </c>
+      <c r="N2" s="28" t="s">
+        <v>456</v>
+      </c>
+      <c r="O2" s="29" t="s">
+        <v>455</v>
+      </c>
+      <c r="P2" s="29" t="s">
+        <v>417</v>
+      </c>
+      <c r="Q2" s="29" t="s">
         <v>457</v>
       </c>
-      <c r="O2" s="30" t="s">
-        <v>456</v>
-      </c>
-      <c r="P2" s="30" t="s">
-        <v>417</v>
-      </c>
-      <c r="Q2" s="30" t="s">
-        <v>458</v>
-      </c>
-    </row>
-    <row r="3" spans="1:17" ht="37" customHeight="1">
+    </row>
+    <row r="3" spans="1:17" ht="25" customHeight="1">
       <c r="A3" s="11" t="s">
         <v>380</v>
       </c>
@@ -9676,17 +9696,26 @@
       <c r="H3" s="19" t="s">
         <v>434</v>
       </c>
-      <c r="N3" s="31" t="s">
-        <v>450</v>
-      </c>
-      <c r="O3" s="32" t="s">
-        <v>455</v>
-      </c>
-      <c r="P3" s="38" t="str">
+      <c r="K3" t="s">
+        <v>462</v>
+      </c>
+      <c r="L3" t="s">
+        <v>463</v>
+      </c>
+      <c r="M3" t="s">
+        <v>465</v>
+      </c>
+      <c r="N3" s="30" t="s">
+        <v>449</v>
+      </c>
+      <c r="O3" s="31" t="s">
+        <v>454</v>
+      </c>
+      <c r="P3" s="37" t="str">
         <f>IF(Q3&lt;&gt;"","Done","Pending")</f>
         <v>Done</v>
       </c>
-      <c r="Q3" s="36">
+      <c r="Q3" s="35">
         <v>46297</v>
       </c>
     </row>
@@ -9706,11 +9735,11 @@
       <c r="H4" s="19" t="s">
         <v>435</v>
       </c>
-      <c r="N4" s="33"/>
-      <c r="O4" s="32" t="s">
-        <v>459</v>
-      </c>
-      <c r="P4" s="38" t="str">
+      <c r="N4" s="32"/>
+      <c r="O4" s="31" t="s">
+        <v>458</v>
+      </c>
+      <c r="P4" s="37" t="str">
         <f t="shared" ref="P4:P32" si="0">IF(Q4&lt;&gt;"","Done","Pending")</f>
         <v>Pending</v>
       </c>
@@ -9727,9 +9756,9 @@
       <c r="H5" s="19" t="s">
         <v>436</v>
       </c>
-      <c r="N5" s="33"/>
-      <c r="O5" s="32"/>
-      <c r="P5" s="38" t="str">
+      <c r="N5" s="32"/>
+      <c r="O5" s="31"/>
+      <c r="P5" s="37" t="str">
         <f t="shared" si="0"/>
         <v>Pending</v>
       </c>
@@ -9748,9 +9777,9 @@
       <c r="H6" s="19" t="s">
         <v>437</v>
       </c>
-      <c r="N6" s="33"/>
-      <c r="O6" s="32"/>
-      <c r="P6" s="38" t="str">
+      <c r="N6" s="32"/>
+      <c r="O6" s="31"/>
+      <c r="P6" s="37" t="str">
         <f t="shared" si="0"/>
         <v>Pending</v>
       </c>
@@ -9762,11 +9791,11 @@
       <c r="B7" s="11" t="s">
         <v>386</v>
       </c>
-      <c r="N7" s="34" t="s">
-        <v>452</v>
-      </c>
-      <c r="O7" s="32"/>
-      <c r="P7" s="38" t="str">
+      <c r="N7" s="33" t="s">
+        <v>451</v>
+      </c>
+      <c r="O7" s="31"/>
+      <c r="P7" s="37" t="str">
         <f t="shared" si="0"/>
         <v>Pending</v>
       </c>
@@ -9778,11 +9807,11 @@
       <c r="B8" s="11" t="s">
         <v>388</v>
       </c>
-      <c r="N8" s="34" t="s">
-        <v>453</v>
-      </c>
-      <c r="O8" s="32"/>
-      <c r="P8" s="38" t="str">
+      <c r="N8" s="33" t="s">
+        <v>452</v>
+      </c>
+      <c r="O8" s="31"/>
+      <c r="P8" s="37" t="str">
         <f t="shared" si="0"/>
         <v>Pending</v>
       </c>
@@ -9794,11 +9823,11 @@
       <c r="B9" s="11" t="s">
         <v>390</v>
       </c>
-      <c r="N9" s="31" t="s">
-        <v>451</v>
-      </c>
-      <c r="O9" s="32"/>
-      <c r="P9" s="38" t="str">
+      <c r="N9" s="30" t="s">
+        <v>450</v>
+      </c>
+      <c r="O9" s="31"/>
+      <c r="P9" s="37" t="str">
         <f t="shared" si="0"/>
         <v>Pending</v>
       </c>
@@ -9810,7 +9839,7 @@
       <c r="B10" s="11" t="s">
         <v>392</v>
       </c>
-      <c r="P10" s="38" t="str">
+      <c r="P10" s="37" t="str">
         <f t="shared" si="0"/>
         <v>Pending</v>
       </c>
@@ -9822,7 +9851,7 @@
       <c r="B11" s="11" t="s">
         <v>394</v>
       </c>
-      <c r="P11" s="38" t="str">
+      <c r="P11" s="37" t="str">
         <f t="shared" si="0"/>
         <v>Pending</v>
       </c>
@@ -9830,10 +9859,10 @@
     <row r="12" spans="1:17" ht="21" customHeight="1">
       <c r="A12" s="11"/>
       <c r="B12" s="11"/>
-      <c r="N12" s="39" t="s">
-        <v>460</v>
-      </c>
-      <c r="P12" s="38" t="str">
+      <c r="N12" s="38" t="s">
+        <v>459</v>
+      </c>
+      <c r="P12" s="37" t="str">
         <f t="shared" si="0"/>
         <v>Pending</v>
       </c>
@@ -9843,7 +9872,7 @@
         <v>395</v>
       </c>
       <c r="B13" s="11"/>
-      <c r="P13" s="38" t="str">
+      <c r="P13" s="37" t="str">
         <f t="shared" si="0"/>
         <v>Pending</v>
       </c>
@@ -9855,7 +9884,7 @@
       <c r="B14" s="11" t="s">
         <v>396</v>
       </c>
-      <c r="P14" s="38" t="str">
+      <c r="P14" s="37" t="str">
         <f t="shared" si="0"/>
         <v>Pending</v>
       </c>
@@ -9867,7 +9896,7 @@
       <c r="B15" s="11" t="s">
         <v>397</v>
       </c>
-      <c r="P15" s="38" t="str">
+      <c r="P15" s="37" t="str">
         <f t="shared" si="0"/>
         <v>Pending</v>
       </c>
@@ -9879,7 +9908,7 @@
       <c r="B16" s="11" t="s">
         <v>398</v>
       </c>
-      <c r="P16" s="38" t="str">
+      <c r="P16" s="37" t="str">
         <f t="shared" si="0"/>
         <v>Pending</v>
       </c>
@@ -9887,7 +9916,7 @@
     <row r="17" spans="1:16" ht="21" customHeight="1">
       <c r="A17" s="11"/>
       <c r="B17" s="11"/>
-      <c r="P17" s="38" t="str">
+      <c r="P17" s="37" t="str">
         <f t="shared" si="0"/>
         <v>Pending</v>
       </c>
@@ -9897,7 +9926,7 @@
         <v>399</v>
       </c>
       <c r="B18" s="11"/>
-      <c r="P18" s="38" t="str">
+      <c r="P18" s="37" t="str">
         <f t="shared" si="0"/>
         <v>Pending</v>
       </c>
@@ -9909,7 +9938,7 @@
       <c r="B19" s="11" t="s">
         <v>401</v>
       </c>
-      <c r="P19" s="38" t="str">
+      <c r="P19" s="37" t="str">
         <f t="shared" si="0"/>
         <v>Pending</v>
       </c>
@@ -9921,7 +9950,7 @@
       <c r="B20" s="11" t="s">
         <v>403</v>
       </c>
-      <c r="P20" s="38" t="str">
+      <c r="P20" s="37" t="str">
         <f t="shared" si="0"/>
         <v>Pending</v>
       </c>
@@ -9933,7 +9962,7 @@
       <c r="B21" s="11" t="s">
         <v>405</v>
       </c>
-      <c r="P21" s="38" t="str">
+      <c r="P21" s="37" t="str">
         <f t="shared" si="0"/>
         <v>Pending</v>
       </c>
@@ -9945,7 +9974,7 @@
       <c r="B22" s="11" t="s">
         <v>407</v>
       </c>
-      <c r="P22" s="38" t="str">
+      <c r="P22" s="37" t="str">
         <f t="shared" si="0"/>
         <v>Pending</v>
       </c>
@@ -9957,71 +9986,70 @@
       <c r="B23" s="11" t="s">
         <v>409</v>
       </c>
-      <c r="P23" s="38" t="str">
+      <c r="P23" s="37" t="str">
         <f t="shared" si="0"/>
         <v>Pending</v>
       </c>
     </row>
     <row r="24" spans="1:16" ht="21" customHeight="1">
-      <c r="P24" s="38" t="str">
+      <c r="P24" s="37" t="str">
         <f t="shared" si="0"/>
         <v>Pending</v>
       </c>
     </row>
     <row r="25" spans="1:16" ht="37" customHeight="1">
-      <c r="P25" s="38" t="str">
+      <c r="P25" s="37" t="str">
         <f t="shared" si="0"/>
         <v>Pending</v>
       </c>
     </row>
     <row r="26" spans="1:16" ht="37" customHeight="1">
-      <c r="P26" s="38" t="str">
+      <c r="P26" s="37" t="str">
         <f t="shared" si="0"/>
         <v>Pending</v>
       </c>
     </row>
     <row r="27" spans="1:16" ht="37" customHeight="1">
-      <c r="P27" s="38" t="str">
+      <c r="P27" s="37" t="str">
         <f t="shared" si="0"/>
         <v>Pending</v>
       </c>
     </row>
     <row r="28" spans="1:16" ht="37" customHeight="1">
-      <c r="P28" s="38" t="str">
+      <c r="P28" s="37" t="str">
         <f t="shared" si="0"/>
         <v>Pending</v>
       </c>
     </row>
     <row r="29" spans="1:16" ht="37" customHeight="1">
-      <c r="P29" s="38" t="str">
+      <c r="P29" s="37" t="str">
         <f t="shared" si="0"/>
         <v>Pending</v>
       </c>
     </row>
     <row r="30" spans="1:16" ht="37" customHeight="1">
-      <c r="P30" s="38" t="str">
+      <c r="P30" s="37" t="str">
         <f t="shared" si="0"/>
         <v>Pending</v>
       </c>
     </row>
     <row r="31" spans="1:16" ht="37" customHeight="1">
-      <c r="P31" s="38" t="str">
+      <c r="P31" s="37" t="str">
         <f t="shared" si="0"/>
         <v>Pending</v>
       </c>
     </row>
     <row r="32" spans="1:16" ht="37" customHeight="1">
-      <c r="P32" s="38" t="str">
+      <c r="P32" s="37" t="str">
         <f t="shared" si="0"/>
         <v>Pending</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="4">
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="K1:L1"/>
     <mergeCell ref="F1:H1"/>
-    <mergeCell ref="K2:L2"/>
     <mergeCell ref="N1:O1"/>
   </mergeCells>
   <conditionalFormatting sqref="P3:P32">

</xml_diff>

<commit_message>
feat: routinely update all the files.
</commit_message>
<xml_diff>
--- a/side-project/Scrimba全栈学习路径进度追踪表.xlsx
+++ b/side-project/Scrimba全栈学习路径进度追踪表.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11004"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11011"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ersheng/Desktop/web_project/public-note/side-project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0E8B4A2-BF58-C840-AC96-4A96F0787D5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{718C1319-041D-F54D-AF74-AA1025FF8626}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="620" windowWidth="40960" windowHeight="20800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="0" yWindow="2240" windowWidth="40960" windowHeight="20800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="学习进度追踪" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,6 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">学习进度追踪!$A$1:$I$215</definedName>
   </definedNames>
   <calcPr calcId="191029" iterateDelta="1E-4"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -39,6 +38,24 @@
 </file>
 
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>tc={916FE1D1-8C3B-3344-A5BF-C1D423B7A1B9}</author>
+  </authors>
+  <commentList>
+    <comment ref="I88" authorId="0" shapeId="0" xr:uid="{916FE1D1-8C3B-3344-A5BF-C1D423B7A1B9}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    https://www.figma.com/design/cqtGul0V8RFXY4vTcIv1Kc/Unit-Conversion?node-id=0-1&amp;p=f&amp;t=kC8zGEMjOdvpEov1-0</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>tc={1F17599A-7801-DD42-9181-9FD3B35CA247}</author>
@@ -65,7 +82,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="978" uniqueCount="466">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="980" uniqueCount="468">
   <si>
     <t>Introduction</t>
   </si>
@@ -2013,6 +2030,12 @@
   <si>
     <t>测试题</t>
   </si>
+  <si>
+    <t>待周末，用逆向方式重做项目</t>
+  </si>
+  <si>
+    <t>暂停，后续再回补</t>
+  </si>
 </sst>
 </file>
 
@@ -2022,7 +2045,7 @@
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="20">
+  <fonts count="21">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2158,6 +2181,12 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="12">
@@ -2373,11 +2402,11 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="2" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -2771,6 +2800,20 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="I88" dT="2026-10-16T00:54:02.37" personId="{46818ABC-E3D4-9746-B9F4-E2842DECFE29}" id="{916FE1D1-8C3B-3344-A5BF-C1D423B7A1B9}">
+    <text>https://www.figma.com/design/cqtGul0V8RFXY4vTcIv1Kc/Unit-Conversion?node-id=0-1&amp;p=f&amp;t=kC8zGEMjOdvpEov1-0</text>
+    <extLst>
+      <x:ext xmlns:xltc2="http://schemas.microsoft.com/office/spreadsheetml/2020/threadedcomments2" uri="{F7C98A9C-CBB3-438F-8F68-D28B6AF4A901}">
+        <xltc2:checksum>1839205944</xltc2:checksum>
+        <xltc2:hyperlink startIndex="0" length="104" url="https://www.figma.com/design/cqtGul0V8RFXY4vTcIv1Kc/Unit-Conversion?node-id=0-1&amp;p=f&amp;t=kC8zGEMjOdvpEov1-0"/>
+      </x:ext>
+    </extLst>
+  </threadedComment>
+</ThreadedComments>
+</file>
+
+<file path=xl/threadedComments/threadedComment2.xml><?xml version="1.0" encoding="utf-8"?>
+<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <threadedComment ref="O3" dT="2026-10-02T14:53:42.82" personId="{46818ABC-E3D4-9746-B9F4-E2842DECFE29}" id="{1F17599A-7801-DD42-9181-9FD3B35CA247}">
     <text xml:space="preserve">ERSHENG:
 2026-10-02，下载了firefox浏览器，以满足网页测试中的相关要求（多rendiner engine测试
@@ -2791,7 +2834,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:L215"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="20" customHeight="1"/>
   <cols>
@@ -2803,7 +2846,7 @@
     <col min="6" max="6" width="8" customWidth="1"/>
     <col min="7" max="7" width="10" customWidth="1"/>
     <col min="8" max="8" width="14" customWidth="1"/>
-    <col min="9" max="9" width="20" customWidth="1"/>
+    <col min="9" max="9" width="27.33203125" customWidth="1"/>
     <col min="11" max="11" width="12.5" customWidth="1"/>
     <col min="12" max="12" width="11" customWidth="1"/>
   </cols>
@@ -2844,10 +2887,10 @@
     </row>
     <row r="2" spans="1:12" ht="20" customHeight="1">
       <c r="A2" s="1"/>
-      <c r="B2" s="38" t="s">
+      <c r="B2" s="37" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="38"/>
+      <c r="C2" s="37"/>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
       <c r="F2" s="1"/>
@@ -3109,10 +3152,10 @@
     </row>
     <row r="12" spans="1:12" ht="20" customHeight="1">
       <c r="A12" s="1"/>
-      <c r="B12" s="38" t="s">
+      <c r="B12" s="37" t="s">
         <v>410</v>
       </c>
-      <c r="C12" s="38"/>
+      <c r="C12" s="37"/>
       <c r="D12" s="1"/>
       <c r="E12" s="1"/>
       <c r="F12" s="1"/>
@@ -5454,10 +5497,10 @@
     </row>
     <row r="80" spans="1:11" ht="20" customHeight="1">
       <c r="A80" s="1"/>
-      <c r="B80" s="38" t="s">
+      <c r="B80" s="37" t="s">
         <v>153</v>
       </c>
-      <c r="C80" s="38"/>
+      <c r="C80" s="37"/>
       <c r="D80" s="1"/>
       <c r="E80" s="1"/>
       <c r="F80" s="1"/>
@@ -5692,17 +5735,21 @@
       </c>
       <c r="G87" s="5" t="str">
         <f t="shared" si="5"/>
-        <v>Pending</v>
-      </c>
-      <c r="H87" s="6"/>
-      <c r="I87" s="8"/>
-      <c r="J87" s="21" t="str">
+        <v>Done</v>
+      </c>
+      <c r="H87" s="6">
+        <v>46310</v>
+      </c>
+      <c r="I87" s="8" t="s">
+        <v>466</v>
+      </c>
+      <c r="J87" s="21">
         <f t="shared" si="3"/>
-        <v/>
+        <v>0.42051282051282052</v>
       </c>
       <c r="K87" s="24">
         <f>COUNTIF($G$3:G87,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="88" spans="1:11" ht="20" customHeight="1">
@@ -5727,22 +5774,24 @@
         <v>Pending</v>
       </c>
       <c r="H88" s="6"/>
-      <c r="I88" s="3"/>
+      <c r="I88" s="3" t="s">
+        <v>467</v>
+      </c>
       <c r="J88" s="21" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="K88" s="24">
         <f>COUNTIF($G$3:G88,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="89" spans="1:11" ht="20" customHeight="1">
       <c r="A89" s="1"/>
-      <c r="B89" s="38" t="s">
+      <c r="B89" s="37" t="s">
         <v>170</v>
       </c>
-      <c r="C89" s="38"/>
+      <c r="C89" s="37"/>
       <c r="D89" s="1"/>
       <c r="E89" s="1"/>
       <c r="F89" s="1"/>
@@ -5751,7 +5800,7 @@
       <c r="I89" s="1"/>
       <c r="K89" s="24">
         <f>COUNTIF($G$3:G89,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="90" spans="1:11" ht="20" customHeight="1">
@@ -5783,7 +5832,7 @@
       </c>
       <c r="K90" s="24">
         <f>COUNTIF($G$3:G90,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="91" spans="1:11" ht="20" customHeight="1">
@@ -5815,7 +5864,7 @@
       </c>
       <c r="K91" s="24">
         <f>COUNTIF($G$3:G91,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="92" spans="1:11" ht="20" customHeight="1">
@@ -5847,7 +5896,7 @@
       </c>
       <c r="K92" s="24">
         <f>COUNTIF($G$3:G92,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="93" spans="1:11" ht="20" customHeight="1">
@@ -5879,15 +5928,15 @@
       </c>
       <c r="K93" s="24">
         <f>COUNTIF($G$3:G93,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="94" spans="1:11" ht="20" customHeight="1">
       <c r="A94" s="1"/>
-      <c r="B94" s="38" t="s">
+      <c r="B94" s="37" t="s">
         <v>179</v>
       </c>
-      <c r="C94" s="38"/>
+      <c r="C94" s="37"/>
       <c r="D94" s="1"/>
       <c r="E94" s="1"/>
       <c r="F94" s="1"/>
@@ -5896,7 +5945,7 @@
       <c r="I94" s="1"/>
       <c r="K94" s="24">
         <f>COUNTIF($G$3:G94,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="95" spans="1:11" ht="20" customHeight="1">
@@ -5928,7 +5977,7 @@
       </c>
       <c r="K95" s="24">
         <f>COUNTIF($G$3:G95,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="96" spans="1:11" ht="20" customHeight="1">
@@ -5960,7 +6009,7 @@
       </c>
       <c r="K96" s="24">
         <f>COUNTIF($G$3:G96,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="97" spans="1:11" ht="20" customHeight="1">
@@ -5992,7 +6041,7 @@
       </c>
       <c r="K97" s="24">
         <f>COUNTIF($G$3:G97,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="98" spans="1:11" ht="20" customHeight="1">
@@ -6024,7 +6073,7 @@
       </c>
       <c r="K98" s="24">
         <f>COUNTIF($G$3:G98,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="99" spans="1:11" ht="20" customHeight="1">
@@ -6056,7 +6105,7 @@
       </c>
       <c r="K99" s="24">
         <f>COUNTIF($G$3:G99,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="100" spans="1:11" ht="20" customHeight="1">
@@ -6088,7 +6137,7 @@
       </c>
       <c r="K100" s="24">
         <f>COUNTIF($G$3:G100,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="101" spans="1:11" ht="20" customHeight="1">
@@ -6120,7 +6169,7 @@
       </c>
       <c r="K101" s="24">
         <f>COUNTIF($G$3:G101,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="102" spans="1:11" ht="20" customHeight="1">
@@ -6152,7 +6201,7 @@
       </c>
       <c r="K102" s="24">
         <f>COUNTIF($G$3:G102,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="103" spans="1:11" ht="20" customHeight="1">
@@ -6184,7 +6233,7 @@
       </c>
       <c r="K103" s="24">
         <f>COUNTIF($G$3:G103,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="104" spans="1:11" ht="20" customHeight="1">
@@ -6216,7 +6265,7 @@
       </c>
       <c r="K104" s="24">
         <f>COUNTIF($G$3:G104,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="105" spans="1:11" ht="20" customHeight="1">
@@ -6248,7 +6297,7 @@
       </c>
       <c r="K105" s="24">
         <f>COUNTIF($G$3:G105,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="106" spans="1:11" ht="20" customHeight="1">
@@ -6280,7 +6329,7 @@
       </c>
       <c r="K106" s="24">
         <f>COUNTIF($G$3:G106,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="107" spans="1:11" ht="20" customHeight="1">
@@ -6312,7 +6361,7 @@
       </c>
       <c r="K107" s="24">
         <f>COUNTIF($G$3:G107,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="108" spans="1:11" ht="20" customHeight="1">
@@ -6344,7 +6393,7 @@
       </c>
       <c r="K108" s="24">
         <f>COUNTIF($G$3:G108,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="109" spans="1:11" ht="20" customHeight="1">
@@ -6376,7 +6425,7 @@
       </c>
       <c r="K109" s="24">
         <f>COUNTIF($G$3:G109,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="110" spans="1:11" ht="20" customHeight="1">
@@ -6408,7 +6457,7 @@
       </c>
       <c r="K110" s="24">
         <f>COUNTIF($G$3:G110,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="111" spans="1:11" ht="20" customHeight="1">
@@ -6440,7 +6489,7 @@
       </c>
       <c r="K111" s="24">
         <f>COUNTIF($G$3:G111,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="112" spans="1:11" ht="20" customHeight="1">
@@ -6472,7 +6521,7 @@
       </c>
       <c r="K112" s="24">
         <f>COUNTIF($G$3:G112,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="113" spans="1:11" ht="20" customHeight="1">
@@ -6504,7 +6553,7 @@
       </c>
       <c r="K113" s="24">
         <f>COUNTIF($G$3:G113,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="114" spans="1:11" ht="20" customHeight="1">
@@ -6536,7 +6585,7 @@
       </c>
       <c r="K114" s="24">
         <f>COUNTIF($G$3:G114,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="115" spans="1:11" ht="20" customHeight="1">
@@ -6568,7 +6617,7 @@
       </c>
       <c r="K115" s="24">
         <f>COUNTIF($G$3:G115,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="116" spans="1:11" ht="20" customHeight="1">
@@ -6600,7 +6649,7 @@
       </c>
       <c r="K116" s="24">
         <f>COUNTIF($G$3:G116,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="117" spans="1:11" ht="20" customHeight="1">
@@ -6632,7 +6681,7 @@
       </c>
       <c r="K117" s="24">
         <f>COUNTIF($G$3:G117,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="118" spans="1:11" ht="20" customHeight="1">
@@ -6664,7 +6713,7 @@
       </c>
       <c r="K118" s="24">
         <f>COUNTIF($G$3:G118,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="119" spans="1:11" ht="20" customHeight="1">
@@ -6696,15 +6745,15 @@
       </c>
       <c r="K119" s="24">
         <f>COUNTIF($G$3:G119,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="120" spans="1:11" ht="20" customHeight="1">
       <c r="A120" s="1"/>
-      <c r="B120" s="38" t="s">
+      <c r="B120" s="37" t="s">
         <v>223</v>
       </c>
-      <c r="C120" s="38"/>
+      <c r="C120" s="37"/>
       <c r="D120" s="1"/>
       <c r="E120" s="1"/>
       <c r="F120" s="1"/>
@@ -6713,7 +6762,7 @@
       <c r="I120" s="1"/>
       <c r="K120" s="24">
         <f>COUNTIF($G$3:G120,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="121" spans="1:11" ht="20" customHeight="1">
@@ -6745,7 +6794,7 @@
       </c>
       <c r="K121" s="24">
         <f>COUNTIF($G$3:G121,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="122" spans="1:11" ht="20" customHeight="1">
@@ -6777,7 +6826,7 @@
       </c>
       <c r="K122" s="24">
         <f>COUNTIF($G$3:G122,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="123" spans="1:11" ht="20" customHeight="1">
@@ -6809,7 +6858,7 @@
       </c>
       <c r="K123" s="24">
         <f>COUNTIF($G$3:G123,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="124" spans="1:11" ht="20" customHeight="1">
@@ -6841,7 +6890,7 @@
       </c>
       <c r="K124" s="24">
         <f>COUNTIF($G$3:G124,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="125" spans="1:11" ht="20" customHeight="1">
@@ -6873,15 +6922,15 @@
       </c>
       <c r="K125" s="24">
         <f>COUNTIF($G$3:G125,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="126" spans="1:11" ht="20" customHeight="1">
       <c r="A126" s="1"/>
-      <c r="B126" s="38" t="s">
+      <c r="B126" s="37" t="s">
         <v>234</v>
       </c>
-      <c r="C126" s="38"/>
+      <c r="C126" s="37"/>
       <c r="D126" s="1"/>
       <c r="E126" s="1"/>
       <c r="F126" s="1"/>
@@ -6890,7 +6939,7 @@
       <c r="I126" s="1"/>
       <c r="K126" s="24">
         <f>COUNTIF($G$3:G126,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="127" spans="1:11" ht="20" customHeight="1">
@@ -6922,7 +6971,7 @@
       </c>
       <c r="K127" s="24">
         <f>COUNTIF($G$3:G127,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="128" spans="1:11" ht="20" customHeight="1">
@@ -6954,7 +7003,7 @@
       </c>
       <c r="K128" s="24">
         <f>COUNTIF($G$3:G128,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="129" spans="1:11" ht="20" customHeight="1">
@@ -6986,7 +7035,7 @@
       </c>
       <c r="K129" s="24">
         <f>COUNTIF($G$3:G129,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="130" spans="1:11" ht="20" customHeight="1">
@@ -7018,7 +7067,7 @@
       </c>
       <c r="K130" s="24">
         <f>COUNTIF($G$3:G130,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="131" spans="1:11" ht="20" customHeight="1">
@@ -7050,7 +7099,7 @@
       </c>
       <c r="K131" s="24">
         <f>COUNTIF($G$3:G131,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="132" spans="1:11" ht="20" customHeight="1">
@@ -7082,15 +7131,15 @@
       </c>
       <c r="K132" s="24">
         <f>COUNTIF($G$3:G132,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="133" spans="1:11" ht="20" customHeight="1">
       <c r="A133" s="1"/>
-      <c r="B133" s="38" t="s">
+      <c r="B133" s="37" t="s">
         <v>245</v>
       </c>
-      <c r="C133" s="38"/>
+      <c r="C133" s="37"/>
       <c r="D133" s="1"/>
       <c r="E133" s="1"/>
       <c r="F133" s="1"/>
@@ -7099,7 +7148,7 @@
       <c r="I133" s="1"/>
       <c r="K133" s="24">
         <f>COUNTIF($G$3:G133,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="134" spans="1:11" ht="20" customHeight="1">
@@ -7131,7 +7180,7 @@
       </c>
       <c r="K134" s="24">
         <f>COUNTIF($G$3:G134,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="135" spans="1:11" ht="20" customHeight="1">
@@ -7163,7 +7212,7 @@
       </c>
       <c r="K135" s="24">
         <f>COUNTIF($G$3:G135,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="136" spans="1:11" ht="20" customHeight="1">
@@ -7195,7 +7244,7 @@
       </c>
       <c r="K136" s="24">
         <f>COUNTIF($G$3:G136,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="137" spans="1:11" ht="20" customHeight="1">
@@ -7227,7 +7276,7 @@
       </c>
       <c r="K137" s="24">
         <f>COUNTIF($G$3:G137,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="138" spans="1:11" ht="20" customHeight="1">
@@ -7259,15 +7308,15 @@
       </c>
       <c r="K138" s="24">
         <f>COUNTIF($G$3:G138,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="139" spans="1:11" ht="20" customHeight="1">
       <c r="A139" s="1"/>
-      <c r="B139" s="38" t="s">
+      <c r="B139" s="37" t="s">
         <v>256</v>
       </c>
-      <c r="C139" s="38"/>
+      <c r="C139" s="37"/>
       <c r="D139" s="1"/>
       <c r="E139" s="1"/>
       <c r="F139" s="1"/>
@@ -7276,7 +7325,7 @@
       <c r="I139" s="1"/>
       <c r="K139" s="24">
         <f>COUNTIF($G$3:G139,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="140" spans="1:11" ht="20" customHeight="1">
@@ -7308,7 +7357,7 @@
       </c>
       <c r="K140" s="24">
         <f>COUNTIF($G$3:G140,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="141" spans="1:11" ht="20" customHeight="1">
@@ -7340,7 +7389,7 @@
       </c>
       <c r="K141" s="24">
         <f>COUNTIF($G$3:G141,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="142" spans="1:11" ht="20" customHeight="1">
@@ -7372,7 +7421,7 @@
       </c>
       <c r="K142" s="24">
         <f>COUNTIF($G$3:G142,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="143" spans="1:11" ht="20" customHeight="1">
@@ -7404,7 +7453,7 @@
       </c>
       <c r="K143" s="24">
         <f>COUNTIF($G$3:G143,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="144" spans="1:11" ht="20" customHeight="1">
@@ -7436,7 +7485,7 @@
       </c>
       <c r="K144" s="24">
         <f>COUNTIF($G$3:G144,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="145" spans="1:11" ht="20" customHeight="1">
@@ -7468,7 +7517,7 @@
       </c>
       <c r="K145" s="24">
         <f>COUNTIF($G$3:G145,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="146" spans="1:11" ht="20" customHeight="1">
@@ -7500,15 +7549,15 @@
       </c>
       <c r="K146" s="24">
         <f>COUNTIF($G$3:G146,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="147" spans="1:11" ht="20" customHeight="1">
       <c r="A147" s="1"/>
-      <c r="B147" s="38" t="s">
+      <c r="B147" s="37" t="s">
         <v>268</v>
       </c>
-      <c r="C147" s="38"/>
+      <c r="C147" s="37"/>
       <c r="D147" s="1"/>
       <c r="E147" s="1"/>
       <c r="F147" s="1"/>
@@ -7517,7 +7566,7 @@
       <c r="I147" s="1"/>
       <c r="K147" s="24">
         <f>COUNTIF($G$3:G147,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="148" spans="1:11" ht="20" customHeight="1">
@@ -7549,7 +7598,7 @@
       </c>
       <c r="K148" s="24">
         <f>COUNTIF($G$3:G148,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="149" spans="1:11" ht="20" customHeight="1">
@@ -7581,7 +7630,7 @@
       </c>
       <c r="K149" s="24">
         <f>COUNTIF($G$3:G149,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="150" spans="1:11" ht="20" customHeight="1">
@@ -7613,7 +7662,7 @@
       </c>
       <c r="K150" s="24">
         <f>COUNTIF($G$3:G150,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="151" spans="1:11" ht="20" customHeight="1">
@@ -7645,7 +7694,7 @@
       </c>
       <c r="K151" s="24">
         <f>COUNTIF($G$3:G151,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="152" spans="1:11" ht="20" customHeight="1">
@@ -7677,7 +7726,7 @@
       </c>
       <c r="K152" s="24">
         <f>COUNTIF($G$3:G152,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="153" spans="1:11" ht="20" customHeight="1">
@@ -7709,15 +7758,15 @@
       </c>
       <c r="K153" s="24">
         <f>COUNTIF($G$3:G153,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="154" spans="1:11" ht="20" customHeight="1">
       <c r="A154" s="1"/>
-      <c r="B154" s="38" t="s">
+      <c r="B154" s="37" t="s">
         <v>279</v>
       </c>
-      <c r="C154" s="38"/>
+      <c r="C154" s="37"/>
       <c r="D154" s="1"/>
       <c r="E154" s="1"/>
       <c r="F154" s="1"/>
@@ -7726,7 +7775,7 @@
       <c r="I154" s="1"/>
       <c r="K154" s="24">
         <f>COUNTIF($G$3:G154,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="155" spans="1:11" ht="20" customHeight="1">
@@ -7758,7 +7807,7 @@
       </c>
       <c r="K155" s="24">
         <f>COUNTIF($G$3:G155,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="156" spans="1:11" ht="20" customHeight="1">
@@ -7790,7 +7839,7 @@
       </c>
       <c r="K156" s="24">
         <f>COUNTIF($G$3:G156,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="157" spans="1:11" ht="20" customHeight="1">
@@ -7822,7 +7871,7 @@
       </c>
       <c r="K157" s="24">
         <f>COUNTIF($G$3:G157,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="158" spans="1:11" ht="20" customHeight="1">
@@ -7854,15 +7903,15 @@
       </c>
       <c r="K158" s="24">
         <f>COUNTIF($G$3:G158,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="159" spans="1:11" ht="20" customHeight="1">
       <c r="A159" s="1"/>
-      <c r="B159" s="38" t="s">
+      <c r="B159" s="37" t="s">
         <v>288</v>
       </c>
-      <c r="C159" s="38"/>
+      <c r="C159" s="37"/>
       <c r="D159" s="1"/>
       <c r="E159" s="1"/>
       <c r="F159" s="1"/>
@@ -7871,7 +7920,7 @@
       <c r="I159" s="1"/>
       <c r="K159" s="24">
         <f>COUNTIF($G$3:G159,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="160" spans="1:11" ht="20" customHeight="1">
@@ -7903,7 +7952,7 @@
       </c>
       <c r="K160" s="24">
         <f>COUNTIF($G$3:G160,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="161" spans="1:11" ht="20" customHeight="1">
@@ -7935,7 +7984,7 @@
       </c>
       <c r="K161" s="24">
         <f>COUNTIF($G$3:G161,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="162" spans="1:11" ht="20" customHeight="1">
@@ -7967,15 +8016,15 @@
       </c>
       <c r="K162" s="24">
         <f>COUNTIF($G$3:G162,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="163" spans="1:11" ht="20" customHeight="1">
       <c r="A163" s="1"/>
-      <c r="B163" s="38" t="s">
+      <c r="B163" s="37" t="s">
         <v>295</v>
       </c>
-      <c r="C163" s="38"/>
+      <c r="C163" s="37"/>
       <c r="D163" s="1"/>
       <c r="E163" s="1"/>
       <c r="F163" s="1"/>
@@ -7984,7 +8033,7 @@
       <c r="I163" s="1"/>
       <c r="K163" s="24">
         <f>COUNTIF($G$3:G163,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="164" spans="1:11" ht="20" customHeight="1">
@@ -8016,7 +8065,7 @@
       </c>
       <c r="K164" s="24">
         <f>COUNTIF($G$3:G164,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="165" spans="1:11" ht="20" customHeight="1">
@@ -8048,7 +8097,7 @@
       </c>
       <c r="K165" s="24">
         <f>COUNTIF($G$3:G165,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="166" spans="1:11" ht="20" customHeight="1">
@@ -8080,7 +8129,7 @@
       </c>
       <c r="K166" s="24">
         <f>COUNTIF($G$3:G166,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="167" spans="1:11" ht="20" customHeight="1">
@@ -8112,15 +8161,15 @@
       </c>
       <c r="K167" s="24">
         <f>COUNTIF($G$3:G167,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="168" spans="1:11" ht="20" customHeight="1">
       <c r="A168" s="1"/>
-      <c r="B168" s="38" t="s">
+      <c r="B168" s="37" t="s">
         <v>302</v>
       </c>
-      <c r="C168" s="38"/>
+      <c r="C168" s="37"/>
       <c r="D168" s="1"/>
       <c r="E168" s="1"/>
       <c r="F168" s="1"/>
@@ -8129,7 +8178,7 @@
       <c r="I168" s="1"/>
       <c r="K168" s="24">
         <f>COUNTIF($G$3:G168,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="169" spans="1:11" ht="20" customHeight="1">
@@ -8161,7 +8210,7 @@
       </c>
       <c r="K169" s="24">
         <f>COUNTIF($G$3:G169,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="170" spans="1:11" ht="20" customHeight="1">
@@ -8193,7 +8242,7 @@
       </c>
       <c r="K170" s="24">
         <f>COUNTIF($G$3:G170,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="171" spans="1:11" ht="20" customHeight="1">
@@ -8225,7 +8274,7 @@
       </c>
       <c r="K171" s="24">
         <f>COUNTIF($G$3:G171,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="172" spans="1:11" ht="20" customHeight="1">
@@ -8257,15 +8306,15 @@
       </c>
       <c r="K172" s="24">
         <f>COUNTIF($G$3:G172,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="173" spans="1:11" ht="20" customHeight="1">
       <c r="A173" s="1"/>
-      <c r="B173" s="38" t="s">
+      <c r="B173" s="37" t="s">
         <v>309</v>
       </c>
-      <c r="C173" s="38"/>
+      <c r="C173" s="37"/>
       <c r="D173" s="1"/>
       <c r="E173" s="1"/>
       <c r="F173" s="1"/>
@@ -8274,7 +8323,7 @@
       <c r="I173" s="1"/>
       <c r="K173" s="24">
         <f>COUNTIF($G$3:G173,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="174" spans="1:11" ht="20" customHeight="1">
@@ -8306,7 +8355,7 @@
       </c>
       <c r="K174" s="24">
         <f>COUNTIF($G$3:G174,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="175" spans="1:11" ht="20" customHeight="1">
@@ -8338,7 +8387,7 @@
       </c>
       <c r="K175" s="24">
         <f>COUNTIF($G$3:G175,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="176" spans="1:11" ht="20" customHeight="1">
@@ -8370,7 +8419,7 @@
       </c>
       <c r="K176" s="24">
         <f>COUNTIF($G$3:G176,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="177" spans="1:11" ht="20" customHeight="1">
@@ -8402,7 +8451,7 @@
       </c>
       <c r="K177" s="24">
         <f>COUNTIF($G$3:G177,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="178" spans="1:11" ht="20" customHeight="1">
@@ -8434,7 +8483,7 @@
       </c>
       <c r="K178" s="24">
         <f>COUNTIF($G$3:G178,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="179" spans="1:11" ht="20" customHeight="1">
@@ -8466,7 +8515,7 @@
       </c>
       <c r="K179" s="24">
         <f>COUNTIF($G$3:G179,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="180" spans="1:11" ht="20" customHeight="1">
@@ -8498,7 +8547,7 @@
       </c>
       <c r="K180" s="24">
         <f>COUNTIF($G$3:G180,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="181" spans="1:11" ht="20" customHeight="1">
@@ -8530,7 +8579,7 @@
       </c>
       <c r="K181" s="24">
         <f>COUNTIF($G$3:G181,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="182" spans="1:11" ht="20" customHeight="1">
@@ -8562,7 +8611,7 @@
       </c>
       <c r="K182" s="24">
         <f>COUNTIF($G$3:G182,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="183" spans="1:11" ht="20" customHeight="1">
@@ -8594,15 +8643,15 @@
       </c>
       <c r="K183" s="24">
         <f>COUNTIF($G$3:G183,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="184" spans="1:11" ht="20" customHeight="1">
       <c r="A184" s="1"/>
-      <c r="B184" s="38" t="s">
+      <c r="B184" s="37" t="s">
         <v>329</v>
       </c>
-      <c r="C184" s="38"/>
+      <c r="C184" s="37"/>
       <c r="D184" s="1"/>
       <c r="E184" s="1"/>
       <c r="F184" s="1"/>
@@ -8611,7 +8660,7 @@
       <c r="I184" s="1"/>
       <c r="K184" s="24">
         <f>COUNTIF($G$3:G184,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="185" spans="1:11" ht="20" customHeight="1">
@@ -8643,7 +8692,7 @@
       </c>
       <c r="K185" s="24">
         <f>COUNTIF($G$3:G185,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="186" spans="1:11" ht="20" customHeight="1">
@@ -8675,7 +8724,7 @@
       </c>
       <c r="K186" s="24">
         <f>COUNTIF($G$3:G186,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="187" spans="1:11" ht="20" customHeight="1">
@@ -8707,7 +8756,7 @@
       </c>
       <c r="K187" s="24">
         <f>COUNTIF($G$3:G187,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="188" spans="1:11" ht="20" customHeight="1">
@@ -8739,7 +8788,7 @@
       </c>
       <c r="K188" s="24">
         <f>COUNTIF($G$3:G188,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="189" spans="1:11" ht="20" customHeight="1">
@@ -8771,7 +8820,7 @@
       </c>
       <c r="K189" s="24">
         <f>COUNTIF($G$3:G189,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="190" spans="1:11" ht="20" customHeight="1">
@@ -8803,7 +8852,7 @@
       </c>
       <c r="K190" s="24">
         <f>COUNTIF($G$3:G190,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="191" spans="1:11" ht="20" customHeight="1">
@@ -8835,7 +8884,7 @@
       </c>
       <c r="K191" s="24">
         <f>COUNTIF($G$3:G191,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="192" spans="1:11" ht="20" customHeight="1">
@@ -8867,7 +8916,7 @@
       </c>
       <c r="K192" s="24">
         <f>COUNTIF($G$3:G192,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="193" spans="1:11" ht="20" customHeight="1">
@@ -8899,7 +8948,7 @@
       </c>
       <c r="K193" s="24">
         <f>COUNTIF($G$3:G193,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="194" spans="1:11" ht="20" customHeight="1">
@@ -8931,7 +8980,7 @@
       </c>
       <c r="K194" s="24">
         <f>COUNTIF($G$3:G194,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="195" spans="1:11" ht="20" customHeight="1">
@@ -8963,7 +9012,7 @@
       </c>
       <c r="K195" s="24">
         <f>COUNTIF($G$3:G195,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="196" spans="1:11" ht="20" customHeight="1">
@@ -8995,15 +9044,15 @@
       </c>
       <c r="K196" s="24">
         <f>COUNTIF($G$3:G196,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="197" spans="1:11" ht="20" customHeight="1">
       <c r="A197" s="1"/>
-      <c r="B197" s="38" t="s">
+      <c r="B197" s="37" t="s">
         <v>348</v>
       </c>
-      <c r="C197" s="38"/>
+      <c r="C197" s="37"/>
       <c r="D197" s="1"/>
       <c r="E197" s="1"/>
       <c r="F197" s="1"/>
@@ -9012,7 +9061,7 @@
       <c r="I197" s="1"/>
       <c r="K197" s="24">
         <f>COUNTIF($G$3:G197,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="198" spans="1:11" ht="20" customHeight="1">
@@ -9044,7 +9093,7 @@
       </c>
       <c r="K198" s="24">
         <f>COUNTIF($G$3:G198,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="199" spans="1:11" ht="20" customHeight="1">
@@ -9076,7 +9125,7 @@
       </c>
       <c r="K199" s="24">
         <f>COUNTIF($G$3:G199,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="200" spans="1:11" ht="20" customHeight="1">
@@ -9108,7 +9157,7 @@
       </c>
       <c r="K200" s="24">
         <f>COUNTIF($G$3:G200,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="201" spans="1:11" ht="20" customHeight="1">
@@ -9140,7 +9189,7 @@
       </c>
       <c r="K201" s="24">
         <f>COUNTIF($G$3:G201,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="202" spans="1:11" ht="20" customHeight="1">
@@ -9172,7 +9221,7 @@
       </c>
       <c r="K202" s="24">
         <f>COUNTIF($G$3:G202,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="203" spans="1:11" ht="20" customHeight="1">
@@ -9204,7 +9253,7 @@
       </c>
       <c r="K203" s="24">
         <f>COUNTIF($G$3:G203,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="204" spans="1:11" ht="20" customHeight="1">
@@ -9236,15 +9285,15 @@
       </c>
       <c r="K204" s="24">
         <f>COUNTIF($G$3:G204,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="205" spans="1:11" ht="20" customHeight="1">
       <c r="A205" s="1"/>
-      <c r="B205" s="38" t="s">
+      <c r="B205" s="37" t="s">
         <v>361</v>
       </c>
-      <c r="C205" s="38"/>
+      <c r="C205" s="37"/>
       <c r="D205" s="1"/>
       <c r="E205" s="1"/>
       <c r="F205" s="1"/>
@@ -9253,7 +9302,7 @@
       <c r="I205" s="1"/>
       <c r="K205" s="24">
         <f>COUNTIF($G$3:G205,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="206" spans="1:11" ht="20" customHeight="1">
@@ -9285,7 +9334,7 @@
       </c>
       <c r="K206" s="24">
         <f>COUNTIF($G$3:G206,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="207" spans="1:11" ht="20" customHeight="1">
@@ -9317,7 +9366,7 @@
       </c>
       <c r="K207" s="24">
         <f>COUNTIF($G$3:G207,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="208" spans="1:11" ht="20" customHeight="1">
@@ -9349,7 +9398,7 @@
       </c>
       <c r="K208" s="24">
         <f>COUNTIF($G$3:G208,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="209" spans="1:11" ht="20" customHeight="1">
@@ -9381,7 +9430,7 @@
       </c>
       <c r="K209" s="24">
         <f>COUNTIF($G$3:G209,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="210" spans="1:11" ht="20" customHeight="1">
@@ -9413,15 +9462,15 @@
       </c>
       <c r="K210" s="24">
         <f>COUNTIF($G$3:G210,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="211" spans="1:11" ht="20" customHeight="1">
       <c r="A211" s="1"/>
-      <c r="B211" s="38" t="s">
+      <c r="B211" s="37" t="s">
         <v>372</v>
       </c>
-      <c r="C211" s="38"/>
+      <c r="C211" s="37"/>
       <c r="D211" s="1"/>
       <c r="E211" s="1"/>
       <c r="F211" s="1"/>
@@ -9430,7 +9479,7 @@
       <c r="I211" s="1"/>
       <c r="K211" s="24">
         <f>COUNTIF($G$3:G211,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="212" spans="1:11" ht="20" customHeight="1">
@@ -9462,7 +9511,7 @@
       </c>
       <c r="K212" s="24">
         <f>COUNTIF($G$3:G212,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="213" spans="1:11" ht="20" customHeight="1">
@@ -9494,7 +9543,7 @@
       </c>
       <c r="K213" s="24">
         <f>COUNTIF($G$3:G213,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="214" spans="1:11" ht="20" customHeight="1">
@@ -9526,7 +9575,7 @@
       </c>
       <c r="K214" s="24">
         <f>COUNTIF($G$3:G214,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="215" spans="1:11" ht="20" customHeight="1">
@@ -9558,12 +9607,18 @@
       </c>
       <c r="K215" s="24">
         <f>COUNTIF($G$3:G215,"Done")</f>
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:I215" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <mergeCells count="19">
+    <mergeCell ref="B168:C168"/>
+    <mergeCell ref="B211:C211"/>
+    <mergeCell ref="B197:C197"/>
+    <mergeCell ref="B173:C173"/>
+    <mergeCell ref="B184:C184"/>
+    <mergeCell ref="B205:C205"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="B133:C133"/>
     <mergeCell ref="B89:C89"/>
@@ -9577,12 +9632,6 @@
     <mergeCell ref="B126:C126"/>
     <mergeCell ref="B94:C94"/>
     <mergeCell ref="B12:C12"/>
-    <mergeCell ref="B168:C168"/>
-    <mergeCell ref="B211:C211"/>
-    <mergeCell ref="B197:C197"/>
-    <mergeCell ref="B173:C173"/>
-    <mergeCell ref="B184:C184"/>
-    <mergeCell ref="B205:C205"/>
   </mergeCells>
   <conditionalFormatting sqref="G1:G1048576">
     <cfRule type="cellIs" dxfId="8" priority="1" operator="equal">
@@ -9601,6 +9650,7 @@
   <ignoredErrors>
     <ignoredError sqref="J26" formula="1"/>
   </ignoredErrors>
+  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -9624,23 +9674,23 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="28" customHeight="1">
-      <c r="A1" s="37" t="s">
+      <c r="A1" s="38" t="s">
         <v>378</v>
       </c>
-      <c r="B1" s="37"/>
-      <c r="F1" s="37" t="s">
+      <c r="B1" s="38"/>
+      <c r="F1" s="38" t="s">
         <v>438</v>
       </c>
-      <c r="G1" s="37"/>
-      <c r="H1" s="37"/>
-      <c r="K1" s="37" t="s">
+      <c r="G1" s="38"/>
+      <c r="H1" s="38"/>
+      <c r="K1" s="38" t="s">
         <v>439</v>
       </c>
-      <c r="L1" s="37"/>
-      <c r="N1" s="37" t="s">
+      <c r="L1" s="38"/>
+      <c r="N1" s="38" t="s">
         <v>448</v>
       </c>
-      <c r="O1" s="37"/>
+      <c r="O1" s="38"/>
       <c r="Q1" s="25"/>
     </row>
     <row r="2" spans="1:17" ht="19" customHeight="1">
@@ -10110,10 +10160,10 @@
     </row>
     <row r="2" spans="2:10" ht="17">
       <c r="B2" s="1"/>
-      <c r="C2" s="38" t="s">
+      <c r="C2" s="37" t="s">
         <v>0</v>
       </c>
-      <c r="D2" s="38"/>
+      <c r="D2" s="37"/>
       <c r="E2" s="1"/>
       <c r="F2" s="1"/>
       <c r="G2" s="1"/>

</xml_diff>